<commit_message>
File dei poteri aggiornato alla versione 0.19.0
Il file compilato dall'autore con lo stato attuale: righe verdi per le
carte a posto (30 poteri programmati, 5 tolti), stato e "cosa fa oggi"
aggiornati per le carte cambiate, dubbi da confermare nella colonna J,
ordine dei poteri aggiornato nel foglio Riferimento. Le colonne gialle
dell'autore non sono state toccate.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/NEXUM_poteri.xlsx
+++ b/docs/NEXUM_poteri.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni" sheetId="1" state="visible" r:id="rId1"/>
@@ -15,7 +14,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Poteri'!$A$4:$P$108</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -24,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,13 +39,13 @@
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="004B5563"/>
+      <color rgb="FF4B5563"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -65,7 +64,7 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="000000FF"/>
+      <color rgb="FF0000FF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -73,8 +72,14 @@
       <b val="1"/>
       <sz val="18"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF065F46"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -83,37 +88,42 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F2937"/>
+        <fgColor rgb="FF1F2937"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B8860B"/>
+        <fgColor rgb="FFB8860B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F3F4F6"/>
+        <fgColor rgb="FFF3F4F6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E5E7EB"/>
+        <fgColor rgb="FFE5E7EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEDD5"/>
+        <fgColor rgb="FFFFEDD5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D1FAE5"/>
+        <fgColor rgb="FFD1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA7F3D0"/>
       </patternFill>
     </fill>
   </fills>
@@ -127,23 +137,24 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D1D5DB"/>
+        <color rgb="FFD1D5DB"/>
       </left>
       <right style="thin">
-        <color rgb="00D1D5DB"/>
+        <color rgb="FFD1D5DB"/>
       </right>
       <top style="thin">
-        <color rgb="00D1D5DB"/>
+        <color rgb="FFD1D5DB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D1D5DB"/>
+        <color rgb="FFD1D5DB"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -199,9 +210,18 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -564,14 +584,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B36"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:B37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="22.8" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>NEXUM · Poteri delle carte</t>
@@ -581,18 +601,19 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Catalogo pubblicato versione 1 · preparato da Claude il 27/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+          <t>Preparato da Claude il 27/10/2026 · aggiornato il 28/10/2026 con le tue decisioni (gioco alla versione 0.19.0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="16.8" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Cosa c'è nel file</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
+    <row r="5" ht="31.95" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Poteri</t>
@@ -604,7 +625,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1">
+    <row r="6" ht="31.95" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Decisioni generali</t>
@@ -616,7 +637,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1">
+    <row r="7" ht="31.95" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Riferimento</t>
@@ -628,14 +649,15 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="8"/>
+    <row r="9" ht="16.8" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Come compilarlo</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="19" customHeight="1">
+    <row r="10" ht="19.05" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>1</t>
@@ -647,7 +669,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1">
+    <row r="11" ht="31.95" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>2</t>
@@ -659,7 +681,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="32" customHeight="1">
+    <row r="12" ht="31.95" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>3</t>
@@ -671,7 +693,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="19" customHeight="1">
+    <row r="13" ht="19.05" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>4</t>
@@ -695,7 +717,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="19" customHeight="1">
+    <row r="15" ht="19.05" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>6</t>
@@ -707,7 +729,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="19" customHeight="1">
+    <row r="16" ht="19.05" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>7</t>
@@ -719,7 +741,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="32" customHeight="1">
+    <row r="17" ht="31.95" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>8</t>
@@ -731,14 +753,15 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="18"/>
+    <row r="19" ht="16.8" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Colori</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="19" customHeight="1">
+    <row r="20" ht="19.05" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Giallo</t>
@@ -750,7 +773,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="19" customHeight="1">
+    <row r="21" ht="19.05" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
           <t>Verde</t>
@@ -758,11 +781,11 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Potere programmato: il gioco lo applica.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="19" customHeight="1">
+          <t>Riga verde: carta a posto. Il potere è programmato (il gioco lo applica) oppure è stato tolto su tua decisione. Puoi sempre cambiarla: compila le colonne gialle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="19.05" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Arancione</t>
@@ -774,7 +797,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="19" customHeight="1">
+    <row r="23" ht="19.05" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
           <t>Grigio</t>
@@ -786,14 +809,15 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="24"/>
+    <row r="25" ht="16.8" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Esempio di compilazione (riga di Morrowshade)</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="19" customHeight="1">
+    <row r="26" ht="19.05" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>La tua decisione</t>
@@ -805,7 +829,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="19" customHeight="1">
+    <row r="27" ht="19.05" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
           <t>Nuovo testo sulla carta</t>
@@ -829,7 +853,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="19" customHeight="1">
+    <row r="29" ht="19.05" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
           <t>Note e domande</t>
@@ -841,7 +865,8 @@
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="30"/>
+    <row r="31" ht="16.8" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Riepilogo (si aggiorna da solo)</t>
@@ -884,21 +909,32 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
+          <t>Poteri tolti</t>
+        </is>
+      </c>
+      <c r="B35" s="10">
+        <f>COUNTIF(Poteri!$F$5:$F$108,"Potere tolto")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
           <t>Decisioni compilate (Poteri)</t>
         </is>
       </c>
-      <c r="B35" s="10">
+      <c r="B36" s="10">
         <f>COUNTA(Poteri!$M$5:$M$108)</f>
         <v/>
       </c>
     </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>Decisioni generali compilate</t>
         </is>
       </c>
-      <c r="B36" s="10">
+      <c r="B37" s="10">
         <f>COUNTA('Decisioni generali'!$F$5:$F$13)&amp;" su 9"</f>
         <v/>
       </c>
@@ -915,7 +951,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P108"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -925,8 +961,7 @@
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="44" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
-    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="9" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="40" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
@@ -935,7 +970,7 @@
     <col width="30" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
           <t>NEXUM · Poteri delle carte</t>
@@ -945,11 +980,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Catalogo pubblicato versione 1 · 104 carte · colonne grigie = informazioni, colonne gialle (M–P) = da compilare. Filtri e menu nella riga delle intestazioni.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="32" customHeight="1">
+          <t>Aggiornato il 28/10/2026 con il gioco alla versione 0.19.0 · 104 carte · righe verdi = carte a posto (potere programmato o tolto) · colonne gialle (M–P) = da compilare. Filtri e menu nella riga delle intestazioni.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="31.95" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Codice</t>
@@ -1070,16 +1105,16 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I5" s="14" t="inlineStr"/>
-      <c r="J5" s="14" t="inlineStr"/>
-      <c r="K5" s="14" t="inlineStr"/>
-      <c r="L5" s="14" t="inlineStr"/>
+      <c r="I5" s="14" t="n"/>
+      <c r="J5" s="14" t="n"/>
+      <c r="K5" s="14" t="n"/>
+      <c r="L5" s="14" t="n"/>
       <c r="M5" s="17" t="n"/>
       <c r="N5" s="17" t="n"/>
       <c r="O5" s="17" t="n"/>
       <c r="P5" s="17" t="n"/>
     </row>
-    <row r="6" ht="71" customHeight="1">
+    <row r="6" ht="70.95" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Custodes-1</t>
@@ -1118,7 +1153,7 @@
           <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="n"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>Non è definito cosa vuol dire 'protetta'.</t>
@@ -1140,63 +1175,71 @@
       <c r="P6" s="17" t="n"/>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Custodes-2</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Custodes</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="C7" s="24" t="inlineStr">
         <is>
           <t>Vigil</t>
         </is>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="19" t="n">
         <v>76</v>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>Controllo.</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>Non programmato</t>
-        </is>
-      </c>
-      <c r="G7" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H7" s="14" t="inlineStr">
-        <is>
-          <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
-        </is>
-      </c>
-      <c r="I7" s="14" t="inlineStr"/>
-      <c r="J7" s="14" t="inlineStr">
+      <c r="F7" s="25" t="inlineStr">
+        <is>
+          <t>Programmato</t>
+        </is>
+      </c>
+      <c r="G7" s="19" t="inlineStr">
+        <is>
+          <t>Quando apre la presa</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>Se Vigil apre la presa, chi segue e ha quella fazione deve giocare la sua carta più alta di quella fazione: il gioco solleva solo quella carta.</t>
+        </is>
+      </c>
+      <c r="I7" s="19" t="n"/>
+      <c r="J7" s="19" t="inlineStr">
         <is>
           <t>'Controllo.' non descrive una regola.</t>
         </is>
       </c>
-      <c r="K7" s="14" t="inlineStr">
-        <is>
-          <t>A · Serve solo la regola esatta. Nessuna meccanica nuova: basta approvare la regola.</t>
-        </is>
-      </c>
-      <c r="L7" s="14" t="inlineStr">
+      <c r="K7" s="19" t="inlineStr">
+        <is>
+          <t>Programmato nella versione 0.18.0.</t>
+        </is>
+      </c>
+      <c r="L7" s="19" t="inlineStr">
         <is>
           <t>Se Vigil apre la presa, chi segue deve giocare la sua carta più alta di quella fazione.</t>
         </is>
       </c>
-      <c r="M7" s="17" t="n"/>
+      <c r="M7" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
       <c r="N7" s="17" t="n"/>
-      <c r="O7" s="17" t="n"/>
+      <c r="O7" s="14" t="inlineStr">
+        <is>
+          <t>Se Vigil apre la presa, chi segue deve giocare la sua carta più alta di quella fazione.</t>
+        </is>
+      </c>
       <c r="P7" s="17" t="n"/>
     </row>
     <row r="8" ht="42" customHeight="1">
@@ -1238,131 +1281,131 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I8" s="14" t="inlineStr"/>
-      <c r="J8" s="14" t="inlineStr"/>
-      <c r="K8" s="14" t="inlineStr"/>
-      <c r="L8" s="14" t="inlineStr"/>
+      <c r="I8" s="14" t="n"/>
+      <c r="J8" s="14" t="n"/>
+      <c r="K8" s="14" t="n"/>
+      <c r="L8" s="14" t="n"/>
       <c r="M8" s="17" t="n"/>
       <c r="N8" s="17" t="n"/>
       <c r="O8" s="17" t="n"/>
       <c r="P8" s="17" t="n"/>
     </row>
     <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Custodes-4</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>Custodes</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="24" t="inlineStr">
         <is>
           <t>Foreseer</t>
         </is>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="19" t="n">
         <v>63</v>
       </c>
-      <c r="E9" s="14" t="inlineStr">
-        <is>
-          <t>Predizione.</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>Non programmato</t>
-        </is>
-      </c>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H9" s="14" t="inlineStr">
-        <is>
-          <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
-        </is>
-      </c>
-      <c r="I9" s="14" t="inlineStr"/>
-      <c r="J9" s="14" t="inlineStr">
+      <c r="E9" s="19" t="inlineStr"/>
+      <c r="F9" s="25" t="inlineStr">
+        <is>
+          <t>Potere tolto</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>Nessun potere: tolto su tua decisione (versione 0.18.0). La carta resta, senza testo.</t>
+        </is>
+      </c>
+      <c r="I9" s="19" t="n"/>
+      <c r="J9" s="19" t="inlineStr">
         <is>
           <t>'Predizione.' non descrive una regola.</t>
         </is>
       </c>
-      <c r="K9" s="14" t="inlineStr">
-        <is>
-          <t>E · Informazione e pronostici. Una finestra che mostra un'informazione nascosta o chiede un pronostico.</t>
-        </is>
-      </c>
-      <c r="L9" s="14" t="inlineStr">
+      <c r="K9" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L9" s="19" t="inlineStr">
         <is>
           <t>Quando la giochi, vedi la mano del giocatore che gioca subito dopo di te, solo per questa presa.</t>
         </is>
       </c>
-      <c r="M9" s="17" t="n"/>
+      <c r="M9" s="17" t="inlineStr">
+        <is>
+          <t>Togli il potere</t>
+        </is>
+      </c>
       <c r="N9" s="17" t="n"/>
       <c r="O9" s="17" t="n"/>
       <c r="P9" s="17" t="n"/>
     </row>
     <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Custodes-5</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>Custodes</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr">
+      <c r="C10" s="24" t="inlineStr">
         <is>
           <t>Locke</t>
         </is>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="19" t="n">
         <v>57</v>
       </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>Se prende la presa, limita modifiche nella presa successiva.</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>Non programmato</t>
-        </is>
-      </c>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H10" s="14" t="inlineStr">
-        <is>
-          <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
-        </is>
-      </c>
-      <c r="I10" s="14" t="inlineStr"/>
-      <c r="J10" s="14" t="inlineStr">
+      <c r="E10" s="19" t="inlineStr"/>
+      <c r="F10" s="25" t="inlineStr">
+        <is>
+          <t>Potere tolto</t>
+        </is>
+      </c>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>Nessun potere: tolto su tua decisione (versione 0.18.0). La carta resta, senza testo.</t>
+        </is>
+      </c>
+      <c r="I10" s="19" t="n"/>
+      <c r="J10" s="19" t="inlineStr">
         <is>
           <t>'Limita modifiche' non dice quali né quanto.</t>
         </is>
       </c>
-      <c r="K10" s="14" t="inlineStr">
-        <is>
-          <t>D · Protezione. Definire cosa vuol dire 'protetta' (foglio 'Decisioni generali', punto 3).</t>
-        </is>
-      </c>
-      <c r="L10" s="14" t="inlineStr">
+      <c r="K10" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L10" s="19" t="inlineStr">
         <is>
           <t>Se vince la presa, nella presa successiva nessun potere può cambiare i valori (come un Axiom ritardato).</t>
         </is>
       </c>
-      <c r="M10" s="17" t="n"/>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>Togli il potere</t>
+        </is>
+      </c>
       <c r="N10" s="17" t="n"/>
       <c r="O10" s="17" t="n"/>
       <c r="P10" s="17" t="n"/>
@@ -1406,73 +1449,85 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I11" s="14" t="inlineStr"/>
-      <c r="J11" s="14" t="inlineStr"/>
-      <c r="K11" s="14" t="inlineStr"/>
-      <c r="L11" s="14" t="inlineStr"/>
+      <c r="I11" s="14" t="n"/>
+      <c r="J11" s="14" t="n"/>
+      <c r="K11" s="14" t="n"/>
+      <c r="L11" s="14" t="n"/>
       <c r="M11" s="17" t="n"/>
       <c r="N11" s="17" t="n"/>
       <c r="O11" s="17" t="n"/>
       <c r="P11" s="17" t="n"/>
     </row>
     <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>Custodes-7</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B12" s="19" t="inlineStr">
         <is>
           <t>Custodes</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="C12" s="24" t="inlineStr">
         <is>
           <t>Reversal</t>
         </is>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="19" t="n">
         <v>44</v>
       </c>
-      <c r="E12" s="14" t="inlineStr">
-        <is>
-          <t>Può annullare effetti di vittoria.</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
-        <is>
-          <t>Non programmato</t>
-        </is>
-      </c>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H12" s="14" t="inlineStr">
-        <is>
-          <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
-        </is>
-      </c>
-      <c r="I12" s="14" t="inlineStr"/>
-      <c r="J12" s="14" t="inlineStr">
-        <is>
-          <t>Non dice quali effetti annulla, né se si sceglie.</t>
-        </is>
-      </c>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>A · Serve solo la regola esatta. Nessuna meccanica nuova: basta approvare la regola.</t>
-        </is>
-      </c>
-      <c r="L12" s="14" t="inlineStr">
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>Può annullare effetti di presa.</t>
+        </is>
+      </c>
+      <c r="F12" s="25" t="inlineStr">
+        <is>
+          <t>Programmato</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="inlineStr">
+        <is>
+          <t>Dopo la presa (scelta)</t>
+        </is>
+      </c>
+      <c r="H12" s="19" t="inlineStr">
+        <is>
+          <t>Se Reversal è nella presa e la presa ha dato o tolto punti, chi l'ha catturata sceglie 'Annulla i punti' o 'Tienili'. Annullando, tornano indietro per tutti i giocatori i punti del Contratto e dei poteri nati da quella presa (non i punti pagati per Fury o Ashen, né i bonus sulla prossima carta). La CPU li annulla quando le costano.</t>
+        </is>
+      </c>
+      <c r="I12" s="19" t="n"/>
+      <c r="J12" s="19" t="inlineStr">
+        <is>
+          <t>Da confermare: ho fatto annullare i punti di tutti i giocatori. Se deve annullare solo quelli di chi la cattura, scrivilo nelle note.</t>
+        </is>
+      </c>
+      <c r="K12" s="19" t="inlineStr">
+        <is>
+          <t>Programmato nella versione 0.19.0.</t>
+        </is>
+      </c>
+      <c r="L12" s="19" t="inlineStr">
         <is>
           <t>Se Reversal è nella presa, i poteri 'se vince la presa' (Origin, Zero, Praetor, Vesper Null, Ravager) non si attivano.</t>
         </is>
       </c>
-      <c r="M12" s="17" t="n"/>
-      <c r="N12" s="17" t="n"/>
-      <c r="O12" s="17" t="n"/>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>Nuova regola (scrivi in O)</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Può annullare effetti di presa.</t>
+        </is>
+      </c>
+      <c r="O12" s="17" t="inlineStr">
+        <is>
+          <t>chi prende questa carta può scegliere se annullare i punteggi derivati dalla presa in cui si trova questa carta, ma solo alla fine della presa in cui è presente, non a fine a partita</t>
+        </is>
+      </c>
       <c r="P12" s="17" t="n"/>
     </row>
     <row r="13" ht="42" customHeight="1">
@@ -1514,10 +1569,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
-      <c r="J13" s="14" t="inlineStr"/>
-      <c r="K13" s="14" t="inlineStr"/>
-      <c r="L13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="n"/>
+      <c r="J13" s="14" t="n"/>
+      <c r="K13" s="14" t="n"/>
+      <c r="L13" s="14" t="n"/>
       <c r="M13" s="17" t="n"/>
       <c r="N13" s="17" t="n"/>
       <c r="O13" s="17" t="n"/>
@@ -1562,7 +1617,7 @@
           <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
         </is>
       </c>
-      <c r="I14" s="14" t="inlineStr"/>
+      <c r="I14" s="14" t="n"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
           <t>'Informazione futura.' non descrive una regola.</t>
@@ -1570,7 +1625,7 @@
       </c>
       <c r="K14" s="14" t="inlineStr">
         <is>
-          <t>E · Informazione e pronostici. Una finestra che mostra un'informazione nascosta o chiede un pronostico.</t>
+          <t>Deciso il 28/10/2026: si programma insieme agli altri poteri di informazioni nascoste.</t>
         </is>
       </c>
       <c r="L14" s="14" t="inlineStr">
@@ -1578,12 +1633,16 @@
           <t>Quando la giochi, vedi una carta a caso della mano di ogni avversario.</t>
         </is>
       </c>
-      <c r="M14" s="17" t="n"/>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
       <c r="N14" s="17" t="n"/>
       <c r="O14" s="17" t="n"/>
       <c r="P14" s="17" t="n"/>
     </row>
-    <row r="15" ht="58" customHeight="1">
+    <row r="15" ht="58.05" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Custodes-10</t>
@@ -1622,7 +1681,7 @@
           <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
         </is>
       </c>
-      <c r="I15" s="14" t="inlineStr"/>
+      <c r="I15" s="14" t="n"/>
       <c r="J15" s="14" t="inlineStr">
         <is>
           <t>Dipende dai recuperi, che oggi non esistono.</t>
@@ -1630,7 +1689,7 @@
       </c>
       <c r="K15" s="14" t="inlineStr">
         <is>
-          <t>C · Scarti e recuperi. Una regola generale sulle carte che escono o rientrano in mano (foglio 'Decisioni generali', punto 2).</t>
+          <t>Deciso il 28/10/2026: si programma insieme agli altri poteri di scarti e recuperi.</t>
         </is>
       </c>
       <c r="L15" s="14" t="inlineStr">
@@ -1638,7 +1697,11 @@
           <t>Se Anchor è nella presa, in questa presa nessuno può recuperare carte (Black Echo, Echo Prime, Mnemos).</t>
         </is>
       </c>
-      <c r="M15" s="17" t="n"/>
+      <c r="M15" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
       <c r="N15" s="17" t="n"/>
       <c r="O15" s="17" t="n"/>
       <c r="P15" s="17" t="n"/>
@@ -1682,7 +1745,7 @@
           <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
         </is>
       </c>
-      <c r="I16" s="14" t="inlineStr"/>
+      <c r="I16" s="14" t="n"/>
       <c r="J16" s="14" t="inlineStr">
         <is>
           <t>'Molto bassa' e 'informazione' non sono definiti.</t>
@@ -1690,7 +1753,7 @@
       </c>
       <c r="K16" s="14" t="inlineStr">
         <is>
-          <t>E · Informazione e pronostici. Una finestra che mostra un'informazione nascosta o chiede un pronostico.</t>
+          <t>Deciso il 28/10/2026: si programma insieme agli altri poteri di informazioni nascoste.</t>
         </is>
       </c>
       <c r="L16" s="14" t="inlineStr">
@@ -1698,66 +1761,70 @@
           <t>Se è la carta di valore più basso della presa, vedi la mano di chi vince la presa.</t>
         </is>
       </c>
-      <c r="M16" s="17" t="n"/>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
       <c r="N16" s="17" t="n"/>
       <c r="O16" s="17" t="n"/>
       <c r="P16" s="17" t="n"/>
     </row>
     <row r="17" ht="84" customHeight="1">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>Custodes-12</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>Custodes</t>
         </is>
       </c>
-      <c r="C17" s="15" t="inlineStr">
+      <c r="C17" s="24" t="inlineStr">
         <is>
           <t>Origin</t>
         </is>
       </c>
-      <c r="D17" s="14" t="n">
+      <c r="D17" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="E17" s="19" t="inlineStr">
         <is>
           <t>Se prende la presa: +3 punti bonus Contratto.</t>
         </is>
       </c>
-      <c r="F17" s="19" t="inlineStr">
+      <c r="F17" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G17" s="14" t="inlineStr">
+      <c r="G17" s="19" t="inlineStr">
         <is>
           <t>Dopo la presa</t>
         </is>
       </c>
-      <c r="H17" s="14" t="inlineStr">
+      <c r="H17" s="19" t="inlineStr">
         <is>
           <t>Se Origin vince la presa, chi l'ha giocata guadagna 3 punti Contratto in più, oltre a quelli del Contratto.</t>
         </is>
       </c>
-      <c r="I17" s="14" t="inlineStr">
+      <c r="I17" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 2% delle giocate (2 giocatori: 11% · 4 giocatori: 3% · 8 giocatori: 1%). Vince il 3% delle prese in cui segue la fazione; le carte senza potere da 0–9 ne vincono il 3%. Effetto medio sui punti: +0,06 per giocata.</t>
         </is>
       </c>
-      <c r="J17" s="14" t="inlineStr">
+      <c r="J17" s="19" t="inlineStr">
         <is>
           <t>Con valore 3 non vince quasi mai: si attiva nel 2% delle giocate. In pratica è una carta senza potere.</t>
         </is>
       </c>
-      <c r="K17" s="14" t="inlineStr">
+      <c r="K17" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L17" s="14" t="inlineStr">
+      <c r="L17" s="19" t="inlineStr">
         <is>
           <t>Origin sostiene la sua fazione: se la presa la vince un'altra carta Custodes, chi ha giocato Origin guadagna 2 punti.</t>
         </is>
@@ -1806,80 +1873,84 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I18" s="14" t="inlineStr"/>
-      <c r="J18" s="14" t="inlineStr"/>
-      <c r="K18" s="14" t="inlineStr"/>
-      <c r="L18" s="14" t="inlineStr"/>
+      <c r="I18" s="14" t="n"/>
+      <c r="J18" s="14" t="n"/>
+      <c r="K18" s="14" t="n"/>
+      <c r="L18" s="14" t="n"/>
       <c r="M18" s="17" t="n"/>
       <c r="N18" s="17" t="n"/>
       <c r="O18" s="17" t="n"/>
       <c r="P18" s="17" t="n"/>
     </row>
-    <row r="19" ht="71" customHeight="1">
-      <c r="A19" s="14" t="inlineStr">
+    <row r="19" ht="70.95" customHeight="1">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>Nullarii-1</t>
         </is>
       </c>
-      <c r="B19" s="14" t="inlineStr">
+      <c r="B19" s="19" t="inlineStr">
         <is>
           <t>Nullarii</t>
         </is>
       </c>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="C19" s="24" t="inlineStr">
         <is>
           <t>Vesper Null</t>
         </is>
       </c>
-      <c r="D19" s="14" t="n">
+      <c r="D19" s="19" t="n">
         <v>88</v>
       </c>
-      <c r="E19" s="14" t="inlineStr">
+      <c r="E19" s="19" t="inlineStr">
         <is>
           <t>Se prende la presa: -15 alla prossima carta di un avversario.</t>
         </is>
       </c>
-      <c r="F19" s="19" t="inlineStr">
+      <c r="F19" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G19" s="14" t="inlineStr">
+      <c r="G19" s="19" t="inlineStr">
         <is>
           <t>Dopo la presa</t>
         </is>
       </c>
-      <c r="H19" s="14" t="inlineStr">
+      <c r="H19" s="19" t="inlineStr">
         <is>
           <t>Se vince la presa, l'avversario con più punti nella mano (a parità, il primo in ordine di posto) avrà −15 sulla prossima carta che gioca.</t>
         </is>
       </c>
-      <c r="I19" s="14" t="inlineStr">
+      <c r="I19" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 44% delle giocate (2 giocatori: 72% · 4 giocatori: 50% · 8 giocatori: 33%). Vince il 64% delle prese in cui segue la fazione; le carte senza potere da 80–89 ne vincono il 63%.</t>
         </is>
       </c>
-      <c r="J19" s="14" t="inlineStr">
+      <c r="J19" s="19" t="inlineStr">
         <is>
           <t>'Un avversario' lo sceglie il gioco (quello in testa), non chi gioca la carta.</t>
         </is>
       </c>
-      <c r="K19" s="14" t="inlineStr">
+      <c r="K19" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L19" s="14" t="inlineStr">
+      <c r="L19" s="19" t="inlineStr">
         <is>
           <t>Va bene così; oppure lo sceglie chi gioca la carta (serve la finestra di scelta).</t>
         </is>
       </c>
-      <c r="M19" s="17" t="n"/>
+      <c r="M19" s="17" t="inlineStr">
+        <is>
+          <t>Va bene così</t>
+        </is>
+      </c>
       <c r="N19" s="17" t="n"/>
       <c r="O19" s="17" t="n"/>
       <c r="P19" s="17" t="n"/>
     </row>
-    <row r="20" ht="58" customHeight="1">
+    <row r="20" ht="58.05" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
           <t>Nullarii-2</t>
@@ -1918,7 +1989,7 @@
           <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
         </is>
       </c>
-      <c r="I20" s="14" t="inlineStr"/>
+      <c r="I20" s="14" t="n"/>
       <c r="J20" s="14" t="inlineStr">
         <is>
           <t>Scartare dalla mano lascia a ognuno meno carte delle prese che restano.</t>
@@ -1926,7 +1997,7 @@
       </c>
       <c r="K20" s="14" t="inlineStr">
         <is>
-          <t>C · Scarti e recuperi. Una regola generale sulle carte che escono o rientrano in mano (foglio 'Decisioni generali', punto 2).</t>
+          <t>Deciso il 28/10/2026: si programma insieme agli altri poteri di scarti e prese variabili.</t>
         </is>
       </c>
       <c r="L20" s="14" t="inlineStr">
@@ -1934,66 +2005,74 @@
           <t>Con le 'prese variabili': se vince la presa, ogni avversario scarta una carta a scelta dalla mano (esce dal gioco) e salterà l'ultima presa.</t>
         </is>
       </c>
-      <c r="M20" s="17" t="n"/>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>Nuova regola (scrivi in O)</t>
+        </is>
+      </c>
       <c r="N20" s="17" t="n"/>
-      <c r="O20" s="17" t="n"/>
+      <c r="O20" s="14" t="inlineStr">
+        <is>
+          <t>Con le 'prese variabili': se vince la presa, ogni giocatore scarta una carta a scelta dalla mano (esce dal gioco) e si salterà l'ultima presa.</t>
+        </is>
+      </c>
       <c r="P20" s="17" t="n"/>
     </row>
     <row r="21" ht="84" customHeight="1">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>Nullarii-3</t>
         </is>
       </c>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B21" s="19" t="inlineStr">
         <is>
           <t>Nullarii</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="C21" s="24" t="inlineStr">
         <is>
           <t>Maledict</t>
         </is>
       </c>
-      <c r="D21" s="14" t="n">
+      <c r="D21" s="19" t="n">
         <v>73</v>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E21" s="19" t="inlineStr">
         <is>
           <t>Se non prende la presa, il vincitore perde 1 punto Contratto.</t>
         </is>
       </c>
-      <c r="F21" s="19" t="inlineStr">
+      <c r="F21" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G21" s="14" t="inlineStr">
+      <c r="G21" s="19" t="inlineStr">
         <is>
           <t>Dopo la presa</t>
         </is>
       </c>
-      <c r="H21" s="14" t="inlineStr">
+      <c r="H21" s="19" t="inlineStr">
         <is>
           <t>Se non vince la presa, chi l'ha vinta perde 1 punto Contratto. Vale anche se Maledict è stata giocata fuori fazione e non poteva vincere.</t>
         </is>
       </c>
-      <c r="I21" s="14" t="inlineStr">
+      <c r="I21" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 74% delle giocate (2 giocatori: 38% · 4 giocatori: 66% · 8 giocatori: 85%). Vince il 37% delle prese in cui segue la fazione; le carte senza potere da 70–79 ne vincono il 43%. Effetto medio sui punti: -0,74 per giocata.</t>
         </is>
       </c>
-      <c r="J21" s="14" t="inlineStr">
+      <c r="J21" s="19" t="inlineStr">
         <is>
           <t>Il potere più pesante sui punti: in media toglie 0,74 punti a ogni giocata; in 8 giocatori si attiva nell'85% dei casi.</t>
         </is>
       </c>
-      <c r="K21" s="14" t="inlineStr">
+      <c r="K21" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L21" s="14" t="inlineStr">
+      <c r="L21" s="19" t="inlineStr">
         <is>
           <t>Si attiva solo se Maledict ha seguito la fazione d'apertura.</t>
         </is>
@@ -2003,7 +2082,7 @@
       <c r="O21" s="17" t="n"/>
       <c r="P21" s="17" t="n"/>
     </row>
-    <row r="22" ht="58" customHeight="1">
+    <row r="22" ht="58.05" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
           <t>Nullarii-4</t>
@@ -2024,7 +2103,7 @@
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>La prima volta che perde può tornare in mano.</t>
+          <t>La prima volta che perde può tornare in mano, scartando un'altra carta non giocata a tua scelta.</t>
         </is>
       </c>
       <c r="F22" s="18" t="inlineStr">
@@ -2042,7 +2121,7 @@
           <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
         </is>
       </c>
-      <c r="I22" s="14" t="inlineStr"/>
+      <c r="I22" s="14" t="n"/>
       <c r="J22" s="14" t="inlineStr">
         <is>
           <t>Tornare in mano lascia una carta in più a fine mano.</t>
@@ -2050,7 +2129,7 @@
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t>C · Scarti e recuperi. Una regola generale sulle carte che escono o rientrano in mano (foglio 'Decisioni generali', punto 2).</t>
+          <t>Deciso il 28/10/2026: si programma insieme agli altri poteri di scarti e recuperi.</t>
         </is>
       </c>
       <c r="L22" s="14" t="inlineStr">
@@ -2058,8 +2137,16 @@
           <t>La prima volta che perde una presa, puoi riprenderla in mano scartando un'altra carta (regola dello 'scambio').</t>
         </is>
       </c>
-      <c r="M22" s="17" t="n"/>
-      <c r="N22" s="17" t="n"/>
+      <c r="M22" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
+      <c r="N22" s="14" t="inlineStr">
+        <is>
+          <t>La prima volta che perde può tornare in mano, scartando un'altra carta non giocata a tua scelta.</t>
+        </is>
+      </c>
       <c r="O22" s="17" t="n"/>
       <c r="P22" s="17" t="n"/>
     </row>
@@ -2102,137 +2189,153 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I23" s="14" t="inlineStr"/>
-      <c r="J23" s="14" t="inlineStr"/>
-      <c r="K23" s="14" t="inlineStr"/>
-      <c r="L23" s="14" t="inlineStr"/>
+      <c r="I23" s="14" t="n"/>
+      <c r="J23" s="14" t="n"/>
+      <c r="K23" s="14" t="n"/>
+      <c r="L23" s="14" t="n"/>
       <c r="M23" s="17" t="n"/>
       <c r="N23" s="17" t="n"/>
       <c r="O23" s="17" t="n"/>
       <c r="P23" s="17" t="n"/>
     </row>
-    <row r="24" ht="58" customHeight="1">
-      <c r="A24" s="14" t="inlineStr">
+    <row r="24" ht="58.05" customHeight="1">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>Nullarii-6</t>
         </is>
       </c>
-      <c r="B24" s="14" t="inlineStr">
+      <c r="B24" s="19" t="inlineStr">
         <is>
           <t>Nullarii</t>
         </is>
       </c>
-      <c r="C24" s="15" t="inlineStr">
+      <c r="C24" s="24" t="inlineStr">
         <is>
           <t>Nullchild</t>
         </is>
       </c>
-      <c r="D24" s="14" t="n">
+      <c r="D24" s="19" t="n">
         <v>49</v>
       </c>
-      <c r="E24" s="14" t="inlineStr">
+      <c r="E24" s="19" t="inlineStr">
         <is>
           <t>Se prende la presa, un avversario salta la prossima.</t>
         </is>
       </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>Non programmato</t>
-        </is>
-      </c>
-      <c r="G24" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H24" s="14" t="inlineStr">
-        <is>
-          <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
-        </is>
-      </c>
-      <c r="I24" s="14" t="inlineStr"/>
-      <c r="J24" s="14" t="inlineStr">
+      <c r="F24" s="25" t="inlineStr">
+        <is>
+          <t>Programmato</t>
+        </is>
+      </c>
+      <c r="G24" s="19" t="inlineStr">
+        <is>
+          <t>Dopo la presa</t>
+        </is>
+      </c>
+      <c r="H24" s="19" t="inlineStr">
+        <is>
+          <t>Se vince la presa, l'avversario con più punti nella mano salta la presa successiva (nell'ultima presa non succede niente). La carta che gli avanza viene scartata a fine mano.</t>
+        </is>
+      </c>
+      <c r="I24" s="19" t="n"/>
+      <c r="J24" s="19" t="inlineStr">
         <is>
           <t>Saltare una presa lascia una carta in più a fine mano. Il motore sa già far saltare una presa.</t>
         </is>
       </c>
-      <c r="K24" s="14" t="inlineStr">
-        <is>
-          <t>C · Scarti e recuperi. Una regola generale sulle carte che escono o rientrano in mano (foglio 'Decisioni generali', punto 2).</t>
-        </is>
-      </c>
-      <c r="L24" s="14" t="inlineStr">
+      <c r="K24" s="19" t="inlineStr">
+        <is>
+          <t>Programmato nella versione 0.18.0.</t>
+        </is>
+      </c>
+      <c r="L24" s="19" t="inlineStr">
         <is>
           <t>Se vince la presa, l'avversario in testa salta la presa successiva; a fine mano la carta che gli avanza viene scartata.</t>
         </is>
       </c>
-      <c r="M24" s="17" t="n"/>
+      <c r="M24" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
       <c r="N24" s="17" t="n"/>
       <c r="O24" s="17" t="n"/>
       <c r="P24" s="17" t="n"/>
     </row>
-    <row r="25" ht="71" customHeight="1">
-      <c r="A25" s="14" t="inlineStr">
+    <row r="25" ht="70.95" customHeight="1">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>Nullarii-7</t>
         </is>
       </c>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B25" s="19" t="inlineStr">
         <is>
           <t>Nullarii</t>
         </is>
       </c>
-      <c r="C25" s="15" t="inlineStr">
+      <c r="C25" s="24" t="inlineStr">
         <is>
           <t>Gravemind</t>
         </is>
       </c>
-      <c r="D25" s="14" t="n">
+      <c r="D25" s="19" t="n">
         <v>41</v>
       </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>Cresce con le carte già giocate.</t>
-        </is>
-      </c>
-      <c r="F25" s="19" t="inlineStr">
+      <c r="E25" s="19" t="inlineStr">
+        <is>
+          <t>Cresce di +3 con le tue carte già giocate.</t>
+        </is>
+      </c>
+      <c r="F25" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G25" s="14" t="inlineStr">
+      <c r="G25" s="19" t="inlineStr">
         <is>
           <t>Alla giocata</t>
         </is>
       </c>
-      <c r="H25" s="14" t="inlineStr">
-        <is>
-          <t>+3 per ogni carta che hai già giocato in questa mano, al massimo +15: da 41 arriva a 56 dalla 6ª presa in poi.</t>
-        </is>
-      </c>
-      <c r="I25" s="14" t="inlineStr">
+      <c r="H25" s="19" t="inlineStr">
+        <is>
+          <t>+3 per ogni carta che hai già giocato in questa mano, al massimo +36: da 41 arriva a 77 nell'ultima presa.</t>
+        </is>
+      </c>
+      <c r="I25" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 91% delle giocate (2 giocatori: 95% · 4 giocatori: 92% · 8 giocatori: 90%). Vince il 17% delle prese in cui segue la fazione; le carte senza potere da 40–49 ne vincono il 14%.</t>
         </is>
       </c>
-      <c r="J25" s="14" t="inlineStr">
+      <c r="J25" s="19" t="inlineStr">
         <is>
           <t>Si attiva quasi sempre (91%) ma l'effetto è piccolo.</t>
         </is>
       </c>
-      <c r="K25" s="14" t="inlineStr">
-        <is>
-          <t>Già programmato.</t>
-        </is>
-      </c>
-      <c r="L25" s="14" t="inlineStr">
+      <c r="K25" s="19" t="inlineStr">
+        <is>
+          <t>Programmato nella versione 0.18.0.</t>
+        </is>
+      </c>
+      <c r="L25" s="19" t="inlineStr">
         <is>
           <t>Va bene così.</t>
         </is>
       </c>
-      <c r="M25" s="17" t="n"/>
-      <c r="N25" s="17" t="n"/>
-      <c r="O25" s="17" t="n"/>
+      <c r="M25" s="17" t="inlineStr">
+        <is>
+          <t>Nuova regola (scrivi in O)</t>
+        </is>
+      </c>
+      <c r="N25" s="14" t="inlineStr">
+        <is>
+          <t>Cresce di +3 con le tue carte già giocate.</t>
+        </is>
+      </c>
+      <c r="O25" s="23" t="inlineStr">
+        <is>
+          <t>+3 per ogni carta che hai già giocato in questa mano, al massimo +36</t>
+        </is>
+      </c>
       <c r="P25" s="17" t="n"/>
     </row>
     <row r="26" ht="42" customHeight="1">
@@ -2274,255 +2377,275 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I26" s="14" t="inlineStr"/>
-      <c r="J26" s="14" t="inlineStr"/>
-      <c r="K26" s="14" t="inlineStr"/>
-      <c r="L26" s="14" t="inlineStr"/>
+      <c r="I26" s="14" t="n"/>
+      <c r="J26" s="14" t="n"/>
+      <c r="K26" s="14" t="n"/>
+      <c r="L26" s="14" t="n"/>
       <c r="M26" s="17" t="n"/>
       <c r="N26" s="17" t="n"/>
       <c r="O26" s="17" t="n"/>
       <c r="P26" s="17" t="n"/>
     </row>
     <row r="27" ht="45" customHeight="1">
-      <c r="A27" s="14" t="inlineStr">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>Nullarii-9</t>
         </is>
       </c>
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B27" s="19" t="inlineStr">
         <is>
           <t>Nullarii</t>
         </is>
       </c>
-      <c r="C27" s="15" t="inlineStr">
+      <c r="C27" s="24" t="inlineStr">
         <is>
           <t>Morrowshade</t>
         </is>
       </c>
-      <c r="D27" s="14" t="n">
+      <c r="D27" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="E27" s="14" t="inlineStr">
+      <c r="E27" s="19" t="inlineStr">
         <is>
           <t>Bonus se è la più bassa.</t>
         </is>
       </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>Non programmato</t>
-        </is>
-      </c>
-      <c r="G27" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H27" s="14" t="inlineStr">
-        <is>
-          <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
-        </is>
-      </c>
-      <c r="I27" s="14" t="inlineStr"/>
-      <c r="J27" s="14" t="inlineStr">
-        <is>
-          <t>'Bonus' non dice quanto né di che tipo.</t>
-        </is>
-      </c>
-      <c r="K27" s="14" t="inlineStr">
-        <is>
-          <t>A · Serve solo la regola esatta. Nessuna meccanica nuova: basta approvare la regola.</t>
-        </is>
-      </c>
-      <c r="L27" s="14" t="inlineStr">
+      <c r="F27" s="25" t="inlineStr">
+        <is>
+          <t>Programmato</t>
+        </is>
+      </c>
+      <c r="G27" s="19" t="inlineStr">
+        <is>
+          <t>Dopo la presa</t>
+        </is>
+      </c>
+      <c r="H27" s="19" t="inlineStr">
+        <is>
+          <t>Se nessun'altra carta della presa ha un valore finale più basso, chi l'ha giocata guadagna 1 punto Contratto.</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="n"/>
+      <c r="J27" s="19" t="inlineStr">
+        <is>
+          <t>Scelta di Claude: a pari merito per la più bassa il punto lo prende comunque. Se non deve, scrivilo nelle note.</t>
+        </is>
+      </c>
+      <c r="K27" s="19" t="inlineStr">
+        <is>
+          <t>Programmato nella versione 0.18.0.</t>
+        </is>
+      </c>
+      <c r="L27" s="19" t="inlineStr">
         <is>
           <t>Se è la carta di valore finale più basso della presa, chi l'ha giocata guadagna 1 punto Contratto.</t>
         </is>
       </c>
-      <c r="M27" s="17" t="n"/>
+      <c r="M27" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
       <c r="N27" s="17" t="n"/>
       <c r="O27" s="17" t="n"/>
       <c r="P27" s="17" t="n"/>
     </row>
-    <row r="28" ht="58" customHeight="1">
-      <c r="A28" s="14" t="inlineStr">
+    <row r="28" ht="58.05" customHeight="1">
+      <c r="A28" s="19" t="inlineStr">
         <is>
           <t>Nullarii-10</t>
         </is>
       </c>
-      <c r="B28" s="14" t="inlineStr">
+      <c r="B28" s="19" t="inlineStr">
         <is>
           <t>Nullarii</t>
         </is>
       </c>
-      <c r="C28" s="15" t="inlineStr">
+      <c r="C28" s="24" t="inlineStr">
         <is>
           <t>Ashen</t>
         </is>
       </c>
-      <c r="D28" s="14" t="n">
+      <c r="D28" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="E28" s="14" t="inlineStr">
+      <c r="E28" s="19" t="inlineStr">
         <is>
           <t>Può aumentare pagando punti.</t>
         </is>
       </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>Non programmato</t>
-        </is>
-      </c>
-      <c r="G28" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H28" s="14" t="inlineStr">
-        <is>
-          <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
-        </is>
-      </c>
-      <c r="I28" s="14" t="inlineStr"/>
-      <c r="J28" s="14" t="inlineStr">
+      <c r="F28" s="25" t="inlineStr">
+        <is>
+          <t>Programmato</t>
+        </is>
+      </c>
+      <c r="G28" s="19" t="inlineStr">
+        <is>
+          <t>Alla giocata (scelta)</t>
+        </is>
+      </c>
+      <c r="H28" s="19" t="inlineStr">
+        <is>
+          <t>Quando la giochi scegli quante volte pagare 1 punto Contratto per +20, da 0 a 4 (fino a 97): un pulsante per ogni scelta. La CPU paga solo se vincere la presa le rende più di quanto spende.</t>
+        </is>
+      </c>
+      <c r="I28" s="19" t="n"/>
+      <c r="J28" s="19" t="inlineStr">
         <is>
           <t>Non dice quanti punti si pagano né quanto aumenta. Oggi ha lo stesso testo di Fury.</t>
         </is>
       </c>
-      <c r="K28" s="14" t="inlineStr">
-        <is>
-          <t>B · Scelta del giocatore. Una finestra in cui il giocatore sceglie quando gioca la carta, più la logica per la CPU.</t>
-        </is>
-      </c>
-      <c r="L28" s="14" t="inlineStr">
+      <c r="K28" s="19" t="inlineStr">
+        <is>
+          <t>Programmato nella versione 0.19.0.</t>
+        </is>
+      </c>
+      <c r="L28" s="19" t="inlineStr">
         <is>
           <t>Quando la giochi puoi pagare 1 punto Contratto per +20, al massimo 2 volte (fino a 57).</t>
         </is>
       </c>
-      <c r="M28" s="17" t="n"/>
+      <c r="M28" s="17" t="inlineStr">
+        <is>
+          <t>Nuova regola (scrivi in O)</t>
+        </is>
+      </c>
       <c r="N28" s="17" t="n"/>
-      <c r="O28" s="17" t="n"/>
+      <c r="O28" s="14" t="inlineStr">
+        <is>
+          <t>Quando la giochi puoi pagare 1 punto Contratto per +20, al massimo 4 volte (fino a 97).</t>
+        </is>
+      </c>
       <c r="P28" s="17" t="n"/>
     </row>
     <row r="29" ht="45" customHeight="1">
-      <c r="A29" s="14" t="inlineStr">
+      <c r="A29" s="19" t="inlineStr">
         <is>
           <t>Nullarii-11</t>
         </is>
       </c>
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B29" s="19" t="inlineStr">
         <is>
           <t>Nullarii</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr">
+      <c r="C29" s="24" t="inlineStr">
         <is>
           <t>Paradox</t>
         </is>
       </c>
-      <c r="D29" s="14" t="n">
+      <c r="D29" s="19" t="n">
         <v>9</v>
       </c>
-      <c r="E29" s="14" t="inlineStr">
+      <c r="E29" s="19" t="inlineStr">
         <is>
           <t>Interagisce con valori identici.</t>
         </is>
       </c>
-      <c r="F29" s="18" t="inlineStr">
-        <is>
-          <t>Non programmato</t>
-        </is>
-      </c>
-      <c r="G29" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H29" s="14" t="inlineStr">
-        <is>
-          <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
-        </is>
-      </c>
-      <c r="I29" s="14" t="inlineStr"/>
-      <c r="J29" s="14" t="inlineStr">
-        <is>
-          <t>'Interagisce' non dice cosa succede.</t>
-        </is>
-      </c>
-      <c r="K29" s="14" t="inlineStr">
-        <is>
-          <t>A · Serve solo la regola esatta. Nessuna meccanica nuova: basta approvare la regola.</t>
-        </is>
-      </c>
-      <c r="L29" s="14" t="inlineStr">
+      <c r="F29" s="25" t="inlineStr">
+        <is>
+          <t>Programmato</t>
+        </is>
+      </c>
+      <c r="G29" s="19" t="inlineStr">
+        <is>
+          <t>Alla rivelazione</t>
+        </is>
+      </c>
+      <c r="H29" s="19" t="inlineStr">
+        <is>
+          <t>Se due o più carte della presa hanno lo stesso valore finale, Paradox vale 99. Si controlla dopo gli altri poteri di valore e prima di Measure.</t>
+        </is>
+      </c>
+      <c r="I29" s="19" t="n"/>
+      <c r="J29" s="19" t="inlineStr">
+        <is>
+          <t>Scelta di Claude: conta anche il valore di Paradox (con Faded One, che vale 9 come lei, diventa 99).</t>
+        </is>
+      </c>
+      <c r="K29" s="19" t="inlineStr">
+        <is>
+          <t>Programmato nella versione 0.18.0.</t>
+        </is>
+      </c>
+      <c r="L29" s="19" t="inlineStr">
         <is>
           <t>Se due o più carte della presa hanno lo stesso valore finale, Paradox vale 99.</t>
         </is>
       </c>
-      <c r="M29" s="17" t="n"/>
+      <c r="M29" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
       <c r="N29" s="17" t="n"/>
       <c r="O29" s="17" t="n"/>
       <c r="P29" s="17" t="n"/>
     </row>
     <row r="30" ht="84" customHeight="1">
-      <c r="A30" s="14" t="inlineStr">
+      <c r="A30" s="19" t="inlineStr">
         <is>
           <t>Nullarii-12</t>
         </is>
       </c>
-      <c r="B30" s="14" t="inlineStr">
+      <c r="B30" s="19" t="inlineStr">
         <is>
           <t>Nullarii</t>
         </is>
       </c>
-      <c r="C30" s="15" t="inlineStr">
+      <c r="C30" s="24" t="inlineStr">
         <is>
           <t>Zero</t>
         </is>
       </c>
-      <c r="D30" s="14" t="n">
+      <c r="D30" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="E30" s="14" t="inlineStr">
+      <c r="E30" s="19" t="inlineStr">
         <is>
           <t>Se prende la presa: +4 punti bonus Contratto.</t>
         </is>
       </c>
-      <c r="F30" s="19" t="inlineStr">
+      <c r="F30" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G30" s="14" t="inlineStr">
+      <c r="G30" s="19" t="inlineStr">
         <is>
           <t>Dopo la presa</t>
         </is>
       </c>
-      <c r="H30" s="14" t="inlineStr">
+      <c r="H30" s="19" t="inlineStr">
         <is>
           <t>Se Zero vince la presa, chi l'ha giocata guadagna 4 punti Contratto in più.</t>
         </is>
       </c>
-      <c r="I30" s="14" t="inlineStr">
+      <c r="I30" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 2% delle giocate (2 giocatori: 7% · 4 giocatori: 3% · 8 giocatori: 1%). Vince il 3% delle prese in cui segue la fazione; le carte senza potere da 0–9 ne vincono il 3%. Effetto medio sui punti: +0,08 per giocata.</t>
         </is>
       </c>
-      <c r="J30" s="14" t="inlineStr">
+      <c r="J30" s="19" t="inlineStr">
         <is>
           <t>Con valore 1 non vince quasi mai: si attiva nel 2% delle giocate.</t>
         </is>
       </c>
-      <c r="K30" s="14" t="inlineStr">
+      <c r="K30" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L30" s="14" t="inlineStr">
+      <c r="L30" s="19" t="inlineStr">
         <is>
           <t>Chi cattura Zero (cioè vince la presa in cui c'è Zero) perde 2 punti. Diventa una carta da evitare, in tema con i Nullarii.</t>
         </is>
       </c>
-      <c r="M30" s="17" t="n"/>
+      <c r="M30" s="17" t="inlineStr">
+        <is>
+          <t>Va bene così</t>
+        </is>
+      </c>
       <c r="N30" s="17" t="n"/>
       <c r="O30" s="17" t="n"/>
       <c r="P30" s="17" t="n"/>
@@ -2566,9 +2689,9 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I31" s="14" t="inlineStr"/>
-      <c r="J31" s="14" t="inlineStr"/>
-      <c r="K31" s="14" t="inlineStr"/>
+      <c r="I31" s="14" t="n"/>
+      <c r="J31" s="14" t="n"/>
+      <c r="K31" s="14" t="n"/>
       <c r="L31" s="14" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
@@ -2618,9 +2741,9 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I32" s="14" t="inlineStr"/>
-      <c r="J32" s="14" t="inlineStr"/>
-      <c r="K32" s="14" t="inlineStr"/>
+      <c r="I32" s="14" t="n"/>
+      <c r="J32" s="14" t="n"/>
+      <c r="K32" s="14" t="n"/>
       <c r="L32" s="14" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
@@ -2632,121 +2755,121 @@
       <c r="P32" s="17" t="n"/>
     </row>
     <row r="33" ht="45" customHeight="1">
-      <c r="A33" s="14" t="inlineStr">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t>Auguria-2</t>
         </is>
       </c>
-      <c r="B33" s="14" t="inlineStr">
+      <c r="B33" s="19" t="inlineStr">
         <is>
           <t>Auguria</t>
         </is>
       </c>
-      <c r="C33" s="15" t="inlineStr">
+      <c r="C33" s="24" t="inlineStr">
         <is>
           <t>Sibyl</t>
         </is>
       </c>
-      <c r="D33" s="14" t="n">
+      <c r="D33" s="19" t="n">
         <v>78</v>
       </c>
-      <c r="E33" s="14" t="inlineStr">
-        <is>
-          <t>Predizione.</t>
-        </is>
-      </c>
-      <c r="F33" s="18" t="inlineStr">
-        <is>
-          <t>Non programmato</t>
-        </is>
-      </c>
-      <c r="G33" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H33" s="14" t="inlineStr">
-        <is>
-          <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
-        </is>
-      </c>
-      <c r="I33" s="14" t="inlineStr"/>
-      <c r="J33" s="14" t="inlineStr">
+      <c r="E33" s="19" t="inlineStr"/>
+      <c r="F33" s="25" t="inlineStr">
+        <is>
+          <t>Potere tolto</t>
+        </is>
+      </c>
+      <c r="G33" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H33" s="19" t="inlineStr">
+        <is>
+          <t>Nessun potere: tolto su tua decisione (versione 0.18.0). La carta resta, senza testo.</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="n"/>
+      <c r="J33" s="19" t="inlineStr">
         <is>
           <t>'Predizione.' non descrive una regola.</t>
         </is>
       </c>
-      <c r="K33" s="14" t="inlineStr">
-        <is>
-          <t>E · Informazione e pronostici. Una finestra che mostra un'informazione nascosta o chiede un pronostico.</t>
-        </is>
-      </c>
-      <c r="L33" s="14" t="inlineStr">
+      <c r="K33" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L33" s="19" t="inlineStr">
         <is>
           <t>Quando la giochi, pronostica chi vincerà la presa: se indovini, +2 punti.</t>
         </is>
       </c>
-      <c r="M33" s="17" t="n"/>
+      <c r="M33" s="17" t="inlineStr">
+        <is>
+          <t>Togli il potere</t>
+        </is>
+      </c>
       <c r="N33" s="17" t="n"/>
       <c r="O33" s="17" t="n"/>
       <c r="P33" s="17" t="n"/>
     </row>
     <row r="34" ht="45" customHeight="1">
-      <c r="A34" s="14" t="inlineStr">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>Auguria-3</t>
         </is>
       </c>
-      <c r="B34" s="14" t="inlineStr">
+      <c r="B34" s="19" t="inlineStr">
         <is>
           <t>Auguria</t>
         </is>
       </c>
-      <c r="C34" s="15" t="inlineStr">
+      <c r="C34" s="24" t="inlineStr">
         <is>
           <t>Decima</t>
         </is>
       </c>
-      <c r="D34" s="14" t="n">
+      <c r="D34" s="19" t="n">
         <v>70</v>
       </c>
-      <c r="E34" s="14" t="inlineStr">
-        <is>
-          <t>Predizione sopra/sotto 50.</t>
-        </is>
-      </c>
-      <c r="F34" s="18" t="inlineStr">
-        <is>
-          <t>Non programmato</t>
-        </is>
-      </c>
-      <c r="G34" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H34" s="14" t="inlineStr">
-        <is>
-          <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
-        </is>
-      </c>
-      <c r="I34" s="14" t="inlineStr"/>
-      <c r="J34" s="14" t="inlineStr">
+      <c r="E34" s="19" t="inlineStr"/>
+      <c r="F34" s="25" t="inlineStr">
+        <is>
+          <t>Potere tolto</t>
+        </is>
+      </c>
+      <c r="G34" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H34" s="19" t="inlineStr">
+        <is>
+          <t>Nessun potere: tolto su tua decisione (versione 0.18.0). La carta resta, senza testo.</t>
+        </is>
+      </c>
+      <c r="I34" s="19" t="n"/>
+      <c r="J34" s="19" t="inlineStr">
         <is>
           <t>Non dice cosa si vince se il pronostico è giusto.</t>
         </is>
       </c>
-      <c r="K34" s="14" t="inlineStr">
-        <is>
-          <t>E · Informazione e pronostici. Una finestra che mostra un'informazione nascosta o chiede un pronostico.</t>
-        </is>
-      </c>
-      <c r="L34" s="14" t="inlineStr">
+      <c r="K34" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L34" s="19" t="inlineStr">
         <is>
           <t>Quando la giochi, pronostica se la carta vincente avrà valore sopra o sotto 50: se indovini, +1 punto.</t>
         </is>
       </c>
-      <c r="M34" s="17" t="n"/>
+      <c r="M34" s="17" t="inlineStr">
+        <is>
+          <t>Togli il potere</t>
+        </is>
+      </c>
       <c r="N34" s="17" t="n"/>
       <c r="O34" s="17" t="n"/>
       <c r="P34" s="17" t="n"/>
@@ -2790,9 +2913,9 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I35" s="14" t="inlineStr"/>
-      <c r="J35" s="14" t="inlineStr"/>
-      <c r="K35" s="14" t="inlineStr"/>
+      <c r="I35" s="14" t="n"/>
+      <c r="J35" s="14" t="n"/>
+      <c r="K35" s="14" t="n"/>
       <c r="L35" s="14" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
@@ -2842,9 +2965,9 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I36" s="14" t="inlineStr"/>
-      <c r="J36" s="14" t="inlineStr"/>
-      <c r="K36" s="14" t="inlineStr"/>
+      <c r="I36" s="14" t="n"/>
+      <c r="J36" s="14" t="n"/>
+      <c r="K36" s="14" t="n"/>
       <c r="L36" s="14" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
@@ -2894,9 +3017,9 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I37" s="14" t="inlineStr"/>
-      <c r="J37" s="14" t="inlineStr"/>
-      <c r="K37" s="14" t="inlineStr"/>
+      <c r="I37" s="14" t="n"/>
+      <c r="J37" s="14" t="n"/>
+      <c r="K37" s="14" t="n"/>
       <c r="L37" s="14" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
@@ -2946,9 +3069,9 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I38" s="14" t="inlineStr"/>
-      <c r="J38" s="14" t="inlineStr"/>
-      <c r="K38" s="14" t="inlineStr"/>
+      <c r="I38" s="14" t="n"/>
+      <c r="J38" s="14" t="n"/>
+      <c r="K38" s="14" t="n"/>
       <c r="L38" s="14" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
@@ -2998,9 +3121,9 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I39" s="14" t="inlineStr"/>
-      <c r="J39" s="14" t="inlineStr"/>
-      <c r="K39" s="14" t="inlineStr"/>
+      <c r="I39" s="14" t="n"/>
+      <c r="J39" s="14" t="n"/>
+      <c r="K39" s="14" t="n"/>
       <c r="L39" s="14" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
@@ -3050,9 +3173,9 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I40" s="14" t="inlineStr"/>
-      <c r="J40" s="14" t="inlineStr"/>
-      <c r="K40" s="14" t="inlineStr"/>
+      <c r="I40" s="14" t="n"/>
+      <c r="J40" s="14" t="n"/>
+      <c r="K40" s="14" t="n"/>
       <c r="L40" s="14" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
@@ -3102,9 +3225,9 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I41" s="14" t="inlineStr"/>
-      <c r="J41" s="14" t="inlineStr"/>
-      <c r="K41" s="14" t="inlineStr"/>
+      <c r="I41" s="14" t="n"/>
+      <c r="J41" s="14" t="n"/>
+      <c r="K41" s="14" t="n"/>
       <c r="L41" s="14" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
@@ -3154,9 +3277,9 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I42" s="14" t="inlineStr"/>
-      <c r="J42" s="14" t="inlineStr"/>
-      <c r="K42" s="14" t="inlineStr"/>
+      <c r="I42" s="14" t="n"/>
+      <c r="J42" s="14" t="n"/>
+      <c r="K42" s="14" t="n"/>
       <c r="L42" s="14" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
@@ -3206,9 +3329,9 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I43" s="14" t="inlineStr"/>
-      <c r="J43" s="14" t="inlineStr"/>
-      <c r="K43" s="14" t="inlineStr"/>
+      <c r="I43" s="14" t="n"/>
+      <c r="J43" s="14" t="n"/>
+      <c r="K43" s="14" t="n"/>
       <c r="L43" s="14" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
@@ -3258,76 +3381,80 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I44" s="14" t="inlineStr"/>
-      <c r="J44" s="14" t="inlineStr"/>
-      <c r="K44" s="14" t="inlineStr"/>
-      <c r="L44" s="14" t="inlineStr"/>
+      <c r="I44" s="14" t="n"/>
+      <c r="J44" s="14" t="n"/>
+      <c r="K44" s="14" t="n"/>
+      <c r="L44" s="14" t="n"/>
       <c r="M44" s="17" t="n"/>
       <c r="N44" s="17" t="n"/>
       <c r="O44" s="17" t="n"/>
       <c r="P44" s="17" t="n"/>
     </row>
     <row r="45" ht="45" customHeight="1">
-      <c r="A45" s="14" t="inlineStr">
+      <c r="A45" s="19" t="inlineStr">
         <is>
           <t>Reliquiae-1</t>
         </is>
       </c>
-      <c r="B45" s="14" t="inlineStr">
+      <c r="B45" s="19" t="inlineStr">
         <is>
           <t>Reliquiae</t>
         </is>
       </c>
-      <c r="C45" s="15" t="inlineStr">
+      <c r="C45" s="24" t="inlineStr">
         <is>
           <t>Palimpsest</t>
         </is>
       </c>
-      <c r="D45" s="14" t="n">
+      <c r="D45" s="19" t="n">
         <v>84</v>
       </c>
-      <c r="E45" s="14" t="inlineStr">
+      <c r="E45" s="19" t="inlineStr">
         <is>
           <t>Copia un effetto precedente.</t>
         </is>
       </c>
-      <c r="F45" s="18" t="inlineStr">
-        <is>
-          <t>Non programmato</t>
-        </is>
-      </c>
-      <c r="G45" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H45" s="14" t="inlineStr">
-        <is>
-          <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
-        </is>
-      </c>
-      <c r="I45" s="14" t="inlineStr"/>
-      <c r="J45" s="14" t="inlineStr">
+      <c r="F45" s="25" t="inlineStr">
+        <is>
+          <t>Programmato</t>
+        </is>
+      </c>
+      <c r="G45" s="19" t="inlineStr">
+        <is>
+          <t>Alla giocata</t>
+        </is>
+      </c>
+      <c r="H45" s="19" t="inlineStr">
+        <is>
+          <t>Copia il potere programmato dell'ultima carta con potere giocata prima di lei nella stessa presa e lo usa come suo (sul valore, alla rivelazione o dopo la presa). Se prima non c'è nessun potere, non fa niente. Se copia Fury o Ashen, si può pagare.</t>
+        </is>
+      </c>
+      <c r="I45" s="19" t="n"/>
+      <c r="J45" s="19" t="inlineStr">
         <is>
           <t>Non dice quale effetto copia, né 'precedente' rispetto a cosa.</t>
         </is>
       </c>
-      <c r="K45" s="14" t="inlineStr">
-        <is>
-          <t>A · Serve solo la regola esatta. Nessuna meccanica nuova: basta approvare la regola.</t>
-        </is>
-      </c>
-      <c r="L45" s="14" t="inlineStr">
+      <c r="K45" s="19" t="inlineStr">
+        <is>
+          <t>Programmato nella versione 0.18.0.</t>
+        </is>
+      </c>
+      <c r="L45" s="19" t="inlineStr">
         <is>
           <t>Copia il potere programmato dell'ultima carta con potere giocata prima di lei nella presa.</t>
         </is>
       </c>
-      <c r="M45" s="17" t="n"/>
+      <c r="M45" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
       <c r="N45" s="17" t="n"/>
       <c r="O45" s="17" t="n"/>
       <c r="P45" s="17" t="n"/>
     </row>
-    <row r="46" ht="58" customHeight="1">
+    <row r="46" ht="58.05" customHeight="1">
       <c r="A46" s="14" t="inlineStr">
         <is>
           <t>Reliquiae-2</t>
@@ -3366,7 +3493,7 @@
           <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
         </is>
       </c>
-      <c r="I46" s="14" t="inlineStr"/>
+      <c r="I46" s="14" t="n"/>
       <c r="J46" s="14" t="inlineStr">
         <is>
           <t>Tornare in mano lascia una carta in più a fine mano.</t>
@@ -3374,7 +3501,7 @@
       </c>
       <c r="K46" s="14" t="inlineStr">
         <is>
-          <t>C · Scarti e recuperi. Una regola generale sulle carte che escono o rientrano in mano (foglio 'Decisioni generali', punto 2).</t>
+          <t>Deciso il 28/10/2026: si programma insieme agli altri poteri di scarti e recuperi.</t>
         </is>
       </c>
       <c r="L46" s="14" t="inlineStr">
@@ -3382,12 +3509,16 @@
           <t>Una volta per mano, dopo averla giocata puoi riprenderla in mano scartando un'altra carta.</t>
         </is>
       </c>
-      <c r="M46" s="17" t="n"/>
+      <c r="M46" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
       <c r="N46" s="17" t="n"/>
       <c r="O46" s="17" t="n"/>
       <c r="P46" s="17" t="n"/>
     </row>
-    <row r="47" ht="58" customHeight="1">
+    <row r="47" ht="58.05" customHeight="1">
       <c r="A47" s="14" t="inlineStr">
         <is>
           <t>Reliquiae-3</t>
@@ -3426,7 +3557,7 @@
           <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
         </is>
       </c>
-      <c r="I47" s="14" t="inlineStr"/>
+      <c r="I47" s="14" t="n"/>
       <c r="J47" s="14" t="inlineStr">
         <is>
           <t>'Carta bassa' non è definita e recuperare aggiunge una carta alla mano.</t>
@@ -3434,7 +3565,7 @@
       </c>
       <c r="K47" s="14" t="inlineStr">
         <is>
-          <t>C · Scarti e recuperi. Una regola generale sulle carte che escono o rientrano in mano (foglio 'Decisioni generali', punto 2).</t>
+          <t>Deciso il 28/10/2026: si programma insieme agli altri poteri di scarti e recuperi.</t>
         </is>
       </c>
       <c r="L47" s="14" t="inlineStr">
@@ -3442,7 +3573,11 @@
           <t>Se vince la presa, puoi prendere in mano una carta di valore 20 o meno catturata in questa presa, scartando una tua carta.</t>
         </is>
       </c>
-      <c r="M47" s="17" t="n"/>
+      <c r="M47" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
       <c r="N47" s="17" t="n"/>
       <c r="O47" s="17" t="n"/>
       <c r="P47" s="17" t="n"/>
@@ -3486,16 +3621,16 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I48" s="14" t="inlineStr"/>
-      <c r="J48" s="14" t="inlineStr"/>
-      <c r="K48" s="14" t="inlineStr"/>
-      <c r="L48" s="14" t="inlineStr"/>
+      <c r="I48" s="14" t="n"/>
+      <c r="J48" s="14" t="n"/>
+      <c r="K48" s="14" t="n"/>
+      <c r="L48" s="14" t="n"/>
       <c r="M48" s="17" t="n"/>
       <c r="N48" s="17" t="n"/>
       <c r="O48" s="17" t="n"/>
       <c r="P48" s="17" t="n"/>
     </row>
-    <row r="49" ht="58" customHeight="1">
+    <row r="49" ht="58.05" customHeight="1">
       <c r="A49" s="14" t="inlineStr">
         <is>
           <t>Reliquiae-5</t>
@@ -3534,7 +3669,7 @@
           <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
         </is>
       </c>
-      <c r="I49" s="14" t="inlineStr"/>
+      <c r="I49" s="14" t="n"/>
       <c r="J49" s="14" t="inlineStr">
         <is>
           <t>Gli 'scarti' oggi non esistono.</t>
@@ -3542,7 +3677,7 @@
       </c>
       <c r="K49" s="14" t="inlineStr">
         <is>
-          <t>C · Scarti e recuperi. Una regola generale sulle carte che escono o rientrano in mano (foglio 'Decisioni generali', punto 2).</t>
+          <t>Deciso il 28/10/2026: si programma insieme agli altri poteri di scarti e recuperi.</t>
         </is>
       </c>
       <c r="L49" s="14" t="inlineStr">
@@ -3550,66 +3685,70 @@
           <t>Quando la giochi, puoi darle il valore stampato di una carta che si trova negli scarti.</t>
         </is>
       </c>
-      <c r="M49" s="17" t="n"/>
+      <c r="M49" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
       <c r="N49" s="17" t="n"/>
       <c r="O49" s="17" t="n"/>
       <c r="P49" s="17" t="n"/>
     </row>
-    <row r="50" ht="71" customHeight="1">
-      <c r="A50" s="14" t="inlineStr">
+    <row r="50" ht="70.95" customHeight="1">
+      <c r="A50" s="19" t="inlineStr">
         <is>
           <t>Reliquiae-6</t>
         </is>
       </c>
-      <c r="B50" s="14" t="inlineStr">
+      <c r="B50" s="19" t="inlineStr">
         <is>
           <t>Reliquiae</t>
         </is>
       </c>
-      <c r="C50" s="15" t="inlineStr">
+      <c r="C50" s="24" t="inlineStr">
         <is>
           <t>Afterimage</t>
         </is>
       </c>
-      <c r="D50" s="14" t="n">
+      <c r="D50" s="19" t="n">
         <v>46</v>
       </c>
-      <c r="E50" s="14" t="inlineStr">
+      <c r="E50" s="19" t="inlineStr">
         <is>
           <t>Se la carta precedente era 70+, +20.</t>
         </is>
       </c>
-      <c r="F50" s="19" t="inlineStr">
+      <c r="F50" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G50" s="14" t="inlineStr">
+      <c r="G50" s="19" t="inlineStr">
         <is>
           <t>Alla giocata</t>
         </is>
       </c>
-      <c r="H50" s="14" t="inlineStr">
+      <c r="H50" s="19" t="inlineStr">
         <is>
           <t>Se l'ultima carta che TU hai giocato prima di questa (anche in una presa precedente) aveva valore stampato 70 o più, vale +20 (66).</t>
         </is>
       </c>
-      <c r="I50" s="14" t="inlineStr">
+      <c r="I50" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 22% delle giocate (2 giocatori: 22% · 4 giocatori: 19% · 8 giocatori: 21%). Vince il 20% delle prese in cui segue la fazione; le carte senza potere da 40–49 ne vincono il 14%.</t>
         </is>
       </c>
-      <c r="J50" s="14" t="inlineStr">
+      <c r="J50" s="19" t="inlineStr">
         <is>
           <t>Ambiguo: 'la carta precedente' potrebbe essere quella giocata subito prima nella stessa presa, da chiunque. Oggi è la tua carta precedente.</t>
         </is>
       </c>
-      <c r="K50" s="14" t="inlineStr">
+      <c r="K50" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L50" s="14" t="inlineStr">
+      <c r="L50" s="19" t="inlineStr">
         <is>
           <t>Decidi quale 'carta precedente' intendi (foglio 'Decisioni generali', punto 7); per il resto va bene.</t>
         </is>
@@ -3658,10 +3797,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I51" s="14" t="inlineStr"/>
-      <c r="J51" s="14" t="inlineStr"/>
-      <c r="K51" s="14" t="inlineStr"/>
-      <c r="L51" s="14" t="inlineStr"/>
+      <c r="I51" s="14" t="n"/>
+      <c r="J51" s="14" t="n"/>
+      <c r="K51" s="14" t="n"/>
+      <c r="L51" s="14" t="n"/>
       <c r="M51" s="17" t="n"/>
       <c r="N51" s="17" t="n"/>
       <c r="O51" s="17" t="n"/>
@@ -3706,10 +3845,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I52" s="14" t="inlineStr"/>
-      <c r="J52" s="14" t="inlineStr"/>
-      <c r="K52" s="14" t="inlineStr"/>
-      <c r="L52" s="14" t="inlineStr"/>
+      <c r="I52" s="14" t="n"/>
+      <c r="J52" s="14" t="n"/>
+      <c r="K52" s="14" t="n"/>
+      <c r="L52" s="14" t="n"/>
       <c r="M52" s="17" t="n"/>
       <c r="N52" s="17" t="n"/>
       <c r="O52" s="17" t="n"/>
@@ -3754,16 +3893,16 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I53" s="14" t="inlineStr"/>
-      <c r="J53" s="14" t="inlineStr"/>
-      <c r="K53" s="14" t="inlineStr"/>
-      <c r="L53" s="14" t="inlineStr"/>
+      <c r="I53" s="14" t="n"/>
+      <c r="J53" s="14" t="n"/>
+      <c r="K53" s="14" t="n"/>
+      <c r="L53" s="14" t="n"/>
       <c r="M53" s="17" t="n"/>
       <c r="N53" s="17" t="n"/>
       <c r="O53" s="17" t="n"/>
       <c r="P53" s="17" t="n"/>
     </row>
-    <row r="54" ht="58" customHeight="1">
+    <row r="54" ht="58.05" customHeight="1">
       <c r="A54" s="14" t="inlineStr">
         <is>
           <t>Reliquiae-10</t>
@@ -3802,7 +3941,7 @@
           <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
         </is>
       </c>
-      <c r="I54" s="14" t="inlineStr"/>
+      <c r="I54" s="14" t="n"/>
       <c r="J54" s="14" t="inlineStr">
         <is>
           <t>'Bonus' non definito; dipende dagli scarti.</t>
@@ -3810,7 +3949,7 @@
       </c>
       <c r="K54" s="14" t="inlineStr">
         <is>
-          <t>C · Scarti e recuperi. Una regola generale sulle carte che escono o rientrano in mano (foglio 'Decisioni generali', punto 2).</t>
+          <t>Deciso il 28/10/2026: si programma insieme agli altri poteri di scarti e recuperi.</t>
         </is>
       </c>
       <c r="L54" s="14" t="inlineStr">
@@ -3818,12 +3957,16 @@
           <t>Se viene scartata da un potere, chi la possedeva guadagna 2 punti Contratto.</t>
         </is>
       </c>
-      <c r="M54" s="17" t="n"/>
+      <c r="M54" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
       <c r="N54" s="17" t="n"/>
       <c r="O54" s="17" t="n"/>
       <c r="P54" s="17" t="n"/>
     </row>
-    <row r="55" ht="58" customHeight="1">
+    <row r="55" ht="58.05" customHeight="1">
       <c r="A55" s="14" t="inlineStr">
         <is>
           <t>Reliquiae-11</t>
@@ -3862,7 +4005,7 @@
           <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
         </is>
       </c>
-      <c r="I55" s="14" t="inlineStr"/>
+      <c r="I55" s="14" t="n"/>
       <c r="J55" s="14" t="inlineStr">
         <is>
           <t>Dipende dagli scarti.</t>
@@ -3870,7 +4013,7 @@
       </c>
       <c r="K55" s="14" t="inlineStr">
         <is>
-          <t>C · Scarti e recuperi. Una regola generale sulle carte che escono o rientrano in mano (foglio 'Decisioni generali', punto 2).</t>
+          <t>Deciso il 28/10/2026: si programma insieme agli altri poteri di scarti e recuperi.</t>
         </is>
       </c>
       <c r="L55" s="14" t="inlineStr">
@@ -3878,7 +4021,11 @@
           <t>Non può essere scartata dai poteri.</t>
         </is>
       </c>
-      <c r="M55" s="17" t="n"/>
+      <c r="M55" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
       <c r="N55" s="17" t="n"/>
       <c r="O55" s="17" t="n"/>
       <c r="P55" s="17" t="n"/>
@@ -3922,10 +4069,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I56" s="14" t="inlineStr"/>
-      <c r="J56" s="14" t="inlineStr"/>
-      <c r="K56" s="14" t="inlineStr"/>
-      <c r="L56" s="14" t="inlineStr"/>
+      <c r="I56" s="14" t="n"/>
+      <c r="J56" s="14" t="n"/>
+      <c r="K56" s="14" t="n"/>
+      <c r="L56" s="14" t="n"/>
       <c r="M56" s="17" t="n"/>
       <c r="N56" s="17" t="n"/>
       <c r="O56" s="17" t="n"/>
@@ -3970,10 +4117,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I57" s="14" t="inlineStr"/>
-      <c r="J57" s="14" t="inlineStr"/>
-      <c r="K57" s="14" t="inlineStr"/>
-      <c r="L57" s="14" t="inlineStr"/>
+      <c r="I57" s="14" t="n"/>
+      <c r="J57" s="14" t="n"/>
+      <c r="K57" s="14" t="n"/>
+      <c r="L57" s="14" t="n"/>
       <c r="M57" s="17" t="n"/>
       <c r="N57" s="17" t="n"/>
       <c r="O57" s="17" t="n"/>
@@ -4018,70 +4165,70 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I58" s="14" t="inlineStr"/>
-      <c r="J58" s="14" t="inlineStr"/>
-      <c r="K58" s="14" t="inlineStr"/>
-      <c r="L58" s="14" t="inlineStr"/>
+      <c r="I58" s="14" t="n"/>
+      <c r="J58" s="14" t="n"/>
+      <c r="K58" s="14" t="n"/>
+      <c r="L58" s="14" t="n"/>
       <c r="M58" s="17" t="n"/>
       <c r="N58" s="17" t="n"/>
       <c r="O58" s="17" t="n"/>
       <c r="P58" s="17" t="n"/>
     </row>
-    <row r="59" ht="71" customHeight="1">
-      <c r="A59" s="14" t="inlineStr">
+    <row r="59" ht="70.95" customHeight="1">
+      <c r="A59" s="19" t="inlineStr">
         <is>
           <t>Dominari-2</t>
         </is>
       </c>
-      <c r="B59" s="14" t="inlineStr">
+      <c r="B59" s="19" t="inlineStr">
         <is>
           <t>Dominari</t>
         </is>
       </c>
-      <c r="C59" s="15" t="inlineStr">
+      <c r="C59" s="24" t="inlineStr">
         <is>
           <t>Praetor</t>
         </is>
       </c>
-      <c r="D59" s="14" t="n">
+      <c r="D59" s="19" t="n">
         <v>82</v>
       </c>
-      <c r="E59" s="14" t="inlineStr">
+      <c r="E59" s="19" t="inlineStr">
         <is>
           <t>Se prende la presa, la prossima carta +10.</t>
         </is>
       </c>
-      <c r="F59" s="19" t="inlineStr">
+      <c r="F59" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G59" s="14" t="inlineStr">
+      <c r="G59" s="19" t="inlineStr">
         <is>
           <t>Dopo la presa</t>
         </is>
       </c>
-      <c r="H59" s="14" t="inlineStr">
+      <c r="H59" s="19" t="inlineStr">
         <is>
           <t>Se vince la presa, la prossima carta che giochi in questa mano vale +10.</t>
         </is>
       </c>
-      <c r="I59" s="14" t="inlineStr">
+      <c r="I59" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 35% delle giocate (2 giocatori: 67% · 4 giocatori: 45% · 8 giocatori: 24%). Vince il 49% delle prese in cui segue la fazione; le carte senza potere da 80–89 ne vincono il 63%.</t>
         </is>
       </c>
-      <c r="J59" s="14" t="inlineStr">
+      <c r="J59" s="19" t="inlineStr">
         <is>
           <t>Più forte con pochi giocatori: si attiva nel 67% dei casi in 2, nel 24% in 8.</t>
         </is>
       </c>
-      <c r="K59" s="14" t="inlineStr">
+      <c r="K59" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L59" s="14" t="inlineStr">
+      <c r="L59" s="19" t="inlineStr">
         <is>
           <t>Va bene così.</t>
         </is>
@@ -4092,60 +4239,60 @@
       <c r="P59" s="17" t="n"/>
     </row>
     <row r="60" ht="84" customHeight="1">
-      <c r="A60" s="14" t="inlineStr">
+      <c r="A60" s="19" t="inlineStr">
         <is>
           <t>Dominari-3</t>
         </is>
       </c>
-      <c r="B60" s="14" t="inlineStr">
+      <c r="B60" s="19" t="inlineStr">
         <is>
           <t>Dominari</t>
         </is>
       </c>
-      <c r="C60" s="15" t="inlineStr">
+      <c r="C60" s="24" t="inlineStr">
         <is>
           <t>Ravager</t>
         </is>
       </c>
-      <c r="D60" s="14" t="n">
+      <c r="D60" s="19" t="n">
         <v>74</v>
       </c>
-      <c r="E60" s="14" t="inlineStr">
+      <c r="E60" s="19" t="inlineStr">
         <is>
           <t>Se prende la presa, un avversario perde 1 punto Contratto.</t>
         </is>
       </c>
-      <c r="F60" s="19" t="inlineStr">
+      <c r="F60" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G60" s="14" t="inlineStr">
+      <c r="G60" s="19" t="inlineStr">
         <is>
           <t>Dopo la presa</t>
         </is>
       </c>
-      <c r="H60" s="14" t="inlineStr">
+      <c r="H60" s="19" t="inlineStr">
         <is>
           <t>Se vince la presa, l'avversario con più punti nella mano perde 1 punto Contratto.</t>
         </is>
       </c>
-      <c r="I60" s="14" t="inlineStr">
+      <c r="I60" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 24% delle giocate (2 giocatori: 64% · 4 giocatori: 35% · 8 giocatori: 11%). Vince il 34% delle prese in cui segue la fazione; le carte senza potere da 70–79 ne vincono il 43%. Effetto medio sui punti: -0,24 per giocata.</t>
         </is>
       </c>
-      <c r="J60" s="14" t="inlineStr">
+      <c r="J60" s="19" t="inlineStr">
         <is>
           <t>Il bersaglio lo sceglie il gioco, come per Vesper Null. Più forte con pochi giocatori.</t>
         </is>
       </c>
-      <c r="K60" s="14" t="inlineStr">
+      <c r="K60" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L60" s="14" t="inlineStr">
+      <c r="L60" s="19" t="inlineStr">
         <is>
           <t>Va bene così; oppure bersaglio scelto da chi gioca.</t>
         </is>
@@ -4194,10 +4341,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I61" s="14" t="inlineStr"/>
-      <c r="J61" s="14" t="inlineStr"/>
-      <c r="K61" s="14" t="inlineStr"/>
-      <c r="L61" s="14" t="inlineStr"/>
+      <c r="I61" s="14" t="n"/>
+      <c r="J61" s="14" t="n"/>
+      <c r="K61" s="14" t="n"/>
+      <c r="L61" s="14" t="n"/>
       <c r="M61" s="17" t="n"/>
       <c r="N61" s="17" t="n"/>
       <c r="O61" s="17" t="n"/>
@@ -4242,10 +4389,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I62" s="14" t="inlineStr"/>
-      <c r="J62" s="14" t="inlineStr"/>
-      <c r="K62" s="14" t="inlineStr"/>
-      <c r="L62" s="14" t="inlineStr"/>
+      <c r="I62" s="14" t="n"/>
+      <c r="J62" s="14" t="n"/>
+      <c r="K62" s="14" t="n"/>
+      <c r="L62" s="14" t="n"/>
       <c r="M62" s="17" t="n"/>
       <c r="N62" s="17" t="n"/>
       <c r="O62" s="17" t="n"/>
@@ -4290,130 +4437,130 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I63" s="14" t="inlineStr"/>
-      <c r="J63" s="14" t="inlineStr"/>
-      <c r="K63" s="14" t="inlineStr"/>
-      <c r="L63" s="14" t="inlineStr"/>
+      <c r="I63" s="14" t="n"/>
+      <c r="J63" s="14" t="n"/>
+      <c r="K63" s="14" t="n"/>
+      <c r="L63" s="14" t="n"/>
       <c r="M63" s="17" t="n"/>
       <c r="N63" s="17" t="n"/>
       <c r="O63" s="17" t="n"/>
       <c r="P63" s="17" t="n"/>
     </row>
     <row r="64" ht="45" customHeight="1">
-      <c r="A64" s="14" t="inlineStr">
+      <c r="A64" s="19" t="inlineStr">
         <is>
           <t>Dominari-7</t>
         </is>
       </c>
-      <c r="B64" s="14" t="inlineStr">
+      <c r="B64" s="19" t="inlineStr">
         <is>
           <t>Dominari</t>
         </is>
       </c>
-      <c r="C64" s="15" t="inlineStr">
+      <c r="C64" s="24" t="inlineStr">
         <is>
           <t>Usurper</t>
         </is>
       </c>
-      <c r="D64" s="14" t="n">
+      <c r="D64" s="19" t="n">
         <v>43</v>
       </c>
-      <c r="E64" s="14" t="inlineStr">
-        <is>
-          <t>Bonus se batte carte molto alte.</t>
-        </is>
-      </c>
-      <c r="F64" s="18" t="inlineStr">
-        <is>
-          <t>Non programmato</t>
-        </is>
-      </c>
-      <c r="G64" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H64" s="14" t="inlineStr">
-        <is>
-          <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
-        </is>
-      </c>
-      <c r="I64" s="14" t="inlineStr"/>
-      <c r="J64" s="14" t="inlineStr">
+      <c r="E64" s="19" t="inlineStr"/>
+      <c r="F64" s="25" t="inlineStr">
+        <is>
+          <t>Potere tolto</t>
+        </is>
+      </c>
+      <c r="G64" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H64" s="19" t="inlineStr">
+        <is>
+          <t>Nessun potere: tolto su tua decisione (versione 0.18.0). La carta resta, senza testo.</t>
+        </is>
+      </c>
+      <c r="I64" s="19" t="n"/>
+      <c r="J64" s="19" t="inlineStr">
         <is>
           <t>'Bonus' e 'carte molto alte' non sono definiti.</t>
         </is>
       </c>
-      <c r="K64" s="14" t="inlineStr">
-        <is>
-          <t>A · Serve solo la regola esatta. Nessuna meccanica nuova: basta approvare la regola.</t>
-        </is>
-      </c>
-      <c r="L64" s="14" t="inlineStr">
+      <c r="K64" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L64" s="19" t="inlineStr">
         <is>
           <t>Se nella presa c'è una carta avversaria di valore 85 o più, Usurper vale +30 (73).</t>
         </is>
       </c>
-      <c r="M64" s="17" t="n"/>
+      <c r="M64" s="17" t="inlineStr">
+        <is>
+          <t>Togli il potere</t>
+        </is>
+      </c>
       <c r="N64" s="17" t="n"/>
       <c r="O64" s="17" t="n"/>
       <c r="P64" s="17" t="n"/>
     </row>
-    <row r="65" ht="71" customHeight="1">
-      <c r="A65" s="14" t="inlineStr">
+    <row r="65" ht="70.95" customHeight="1">
+      <c r="A65" s="19" t="inlineStr">
         <is>
           <t>Dominari-8</t>
         </is>
       </c>
-      <c r="B65" s="14" t="inlineStr">
+      <c r="B65" s="19" t="inlineStr">
         <is>
           <t>Dominari</t>
         </is>
       </c>
-      <c r="C65" s="15" t="inlineStr">
+      <c r="C65" s="24" t="inlineStr">
         <is>
           <t>Bloodmark</t>
         </is>
       </c>
-      <c r="D65" s="14" t="n">
+      <c r="D65" s="19" t="n">
         <v>35</v>
       </c>
-      <c r="E65" s="14" t="inlineStr">
+      <c r="E65" s="19" t="inlineStr">
         <is>
           <t>Se perde contro 75+, prossima carta +15.</t>
         </is>
       </c>
-      <c r="F65" s="19" t="inlineStr">
+      <c r="F65" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G65" s="14" t="inlineStr">
+      <c r="G65" s="19" t="inlineStr">
         <is>
           <t>Dopo la presa</t>
         </is>
       </c>
-      <c r="H65" s="14" t="inlineStr">
+      <c r="H65" s="19" t="inlineStr">
         <is>
           <t>Se non vince e la carta vincente ha valore finale 75 o più, la tua prossima carta vale +15.</t>
         </is>
       </c>
-      <c r="I65" s="14" t="inlineStr">
+      <c r="I65" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 53% delle giocate (2 giocatori: 15% · 4 giocatori: 40% · 8 giocatori: 68%). Vince il 9% delle prese in cui segue la fazione; le carte senza potere da 30–39 ne vincono il 10%.</t>
         </is>
       </c>
-      <c r="J65" s="14" t="inlineStr">
+      <c r="J65" s="19" t="inlineStr">
         <is>
           <t>Nessun problema evidente; più frequente con tanti giocatori.</t>
         </is>
       </c>
-      <c r="K65" s="14" t="inlineStr">
+      <c r="K65" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L65" s="14" t="inlineStr">
+      <c r="L65" s="19" t="inlineStr">
         <is>
           <t>Va bene così.</t>
         </is>
@@ -4424,60 +4571,60 @@
       <c r="P65" s="17" t="n"/>
     </row>
     <row r="66" ht="84" customHeight="1">
-      <c r="A66" s="14" t="inlineStr">
+      <c r="A66" s="19" t="inlineStr">
         <is>
           <t>Dominari-9</t>
         </is>
       </c>
-      <c r="B66" s="14" t="inlineStr">
+      <c r="B66" s="19" t="inlineStr">
         <is>
           <t>Dominari</t>
         </is>
       </c>
-      <c r="C66" s="15" t="inlineStr">
+      <c r="C66" s="24" t="inlineStr">
         <is>
           <t>Challenger</t>
         </is>
       </c>
-      <c r="D66" s="14" t="n">
+      <c r="D66" s="19" t="n">
         <v>28</v>
       </c>
-      <c r="E66" s="14" t="inlineStr">
+      <c r="E66" s="19" t="inlineStr">
         <is>
           <t>Se affronta un 70+, diventa 68.</t>
         </is>
       </c>
-      <c r="F66" s="19" t="inlineStr">
+      <c r="F66" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G66" s="14" t="inlineStr">
+      <c r="G66" s="19" t="inlineStr">
         <is>
           <t>Alla giocata</t>
         </is>
       </c>
-      <c r="H66" s="14" t="inlineStr">
+      <c r="H66" s="19" t="inlineStr">
         <is>
           <t>Se tra le carte giocate PRIMA di lei in questa presa ce n'è una con valore stampato oltre 70 (cioè 71 o più), vale 68.</t>
         </is>
       </c>
-      <c r="I66" s="14" t="inlineStr">
+      <c r="I66" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 39% delle giocate (2 giocatori: 12% · 4 giocatori: 30% · 8 giocatori: 49%). Vince il 8% delle prese in cui segue la fazione; le carte senza potere da 20–29 ne vincono il 7%.</t>
         </is>
       </c>
-      <c r="J66" s="14" t="inlineStr">
+      <c r="J66" s="19" t="inlineStr">
         <is>
           <t>Si contraddice: diventa 68 proprio quando in tavola c'è già una carta più alta, che se segue la fazione vince comunque. Aiuta solo se la carta alta era fuori fazione. Il testo dice '70+', il gioco esclude il 70.</t>
         </is>
       </c>
-      <c r="K66" s="14" t="inlineStr">
+      <c r="K66" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L66" s="14" t="inlineStr">
+      <c r="L66" s="19" t="inlineStr">
         <is>
           <t>Alla rivelazione: se nella presa c'è una carta avversaria di valore 70 o più (giocata prima o dopo), Challenger vale 85.</t>
         </is>
@@ -4487,121 +4634,125 @@
       <c r="O66" s="17" t="n"/>
       <c r="P66" s="17" t="n"/>
     </row>
-    <row r="67" ht="58" customHeight="1">
-      <c r="A67" s="14" t="inlineStr">
+    <row r="67" ht="58.05" customHeight="1">
+      <c r="A67" s="19" t="inlineStr">
         <is>
           <t>Dominari-10</t>
         </is>
       </c>
-      <c r="B67" s="14" t="inlineStr">
+      <c r="B67" s="19" t="inlineStr">
         <is>
           <t>Dominari</t>
         </is>
       </c>
-      <c r="C67" s="15" t="inlineStr">
+      <c r="C67" s="24" t="inlineStr">
         <is>
           <t>Fury</t>
         </is>
       </c>
-      <c r="D67" s="14" t="n">
+      <c r="D67" s="19" t="n">
         <v>20</v>
       </c>
-      <c r="E67" s="14" t="inlineStr">
+      <c r="E67" s="19" t="inlineStr">
         <is>
           <t>Può aumentare pagando punti.</t>
         </is>
       </c>
-      <c r="F67" s="18" t="inlineStr">
-        <is>
-          <t>Non programmato</t>
-        </is>
-      </c>
-      <c r="G67" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H67" s="14" t="inlineStr">
-        <is>
-          <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
-        </is>
-      </c>
-      <c r="I67" s="14" t="inlineStr"/>
-      <c r="J67" s="14" t="inlineStr">
+      <c r="F67" s="25" t="inlineStr">
+        <is>
+          <t>Programmato</t>
+        </is>
+      </c>
+      <c r="G67" s="19" t="inlineStr">
+        <is>
+          <t>Alla giocata (scelta)</t>
+        </is>
+      </c>
+      <c r="H67" s="19" t="inlineStr">
+        <is>
+          <t>Quando la giochi puoi pagare 2 punti Contratto: vale 75 (pulsante 'Paga 2 punti: vale 75'). La CPU paga solo se vincere la presa le rende più di quanto spende.</t>
+        </is>
+      </c>
+      <c r="I67" s="19" t="n"/>
+      <c r="J67" s="19" t="inlineStr">
         <is>
           <t>Oggi ha lo stesso testo di Ashen.</t>
         </is>
       </c>
-      <c r="K67" s="14" t="inlineStr">
-        <is>
-          <t>B · Scelta del giocatore. Una finestra in cui il giocatore sceglie quando gioca la carta, più la logica per la CPU.</t>
-        </is>
-      </c>
-      <c r="L67" s="14" t="inlineStr">
+      <c r="K67" s="19" t="inlineStr">
+        <is>
+          <t>Programmato nella versione 0.19.0.</t>
+        </is>
+      </c>
+      <c r="L67" s="19" t="inlineStr">
         <is>
           <t>Quando la giochi puoi pagare 2 punti Contratto: vale 75.</t>
         </is>
       </c>
-      <c r="M67" s="17" t="n"/>
+      <c r="M67" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
       <c r="N67" s="17" t="n"/>
       <c r="O67" s="17" t="n"/>
       <c r="P67" s="17" t="n"/>
     </row>
     <row r="68" ht="84" customHeight="1">
-      <c r="A68" s="14" t="inlineStr">
+      <c r="A68" s="19" t="inlineStr">
         <is>
           <t>Dominari-11</t>
         </is>
       </c>
-      <c r="B68" s="14" t="inlineStr">
+      <c r="B68" s="19" t="inlineStr">
         <is>
           <t>Dominari</t>
         </is>
       </c>
-      <c r="C68" s="15" t="inlineStr">
+      <c r="C68" s="24" t="inlineStr">
         <is>
           <t>Rebel</t>
         </is>
       </c>
-      <c r="D68" s="14" t="n">
+      <c r="D68" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="E68" s="14" t="inlineStr">
+      <c r="E68" s="19" t="inlineStr">
         <is>
           <t>Punisce un vincitore 80+.</t>
         </is>
       </c>
-      <c r="F68" s="19" t="inlineStr">
+      <c r="F68" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G68" s="14" t="inlineStr">
+      <c r="G68" s="19" t="inlineStr">
         <is>
           <t>Dopo la presa</t>
         </is>
       </c>
-      <c r="H68" s="14" t="inlineStr">
+      <c r="H68" s="19" t="inlineStr">
         <is>
           <t>Se non vince e la carta vincente ha valore finale 80 o più, chi ha vinto perde 1 punto Contratto.</t>
         </is>
       </c>
-      <c r="I68" s="14" t="inlineStr">
+      <c r="I68" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 44% delle giocate (2 giocatori: 10% · 4 giocatori: 30% · 8 giocatori: 57%). Vince il 4% delle prese in cui segue la fazione; le carte senza potere da 10–19 ne vincono il 6%. Effetto medio sui punti: -0,44 per giocata.</t>
         </is>
       </c>
-      <c r="J68" s="14" t="inlineStr">
+      <c r="J68" s="19" t="inlineStr">
         <is>
           <t>Forte sui punti (in media −0,44 a giocata) e molto più frequente con tanti giocatori.</t>
         </is>
       </c>
-      <c r="K68" s="14" t="inlineStr">
+      <c r="K68" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L68" s="14" t="inlineStr">
+      <c r="L68" s="19" t="inlineStr">
         <is>
           <t>Va bene così.</t>
         </is>
@@ -4611,61 +4762,61 @@
       <c r="O68" s="17" t="n"/>
       <c r="P68" s="17" t="n"/>
     </row>
-    <row r="69" ht="71" customHeight="1">
-      <c r="A69" s="14" t="inlineStr">
+    <row r="69" ht="70.95" customHeight="1">
+      <c r="A69" s="19" t="inlineStr">
         <is>
           <t>Dominari-12</t>
         </is>
       </c>
-      <c r="B69" s="14" t="inlineStr">
+      <c r="B69" s="19" t="inlineStr">
         <is>
           <t>Dominari</t>
         </is>
       </c>
-      <c r="C69" s="15" t="inlineStr">
+      <c r="C69" s="24" t="inlineStr">
         <is>
           <t>Ascendant</t>
         </is>
       </c>
-      <c r="D69" s="14" t="n">
+      <c r="D69" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="E69" s="14" t="inlineStr">
+      <c r="E69" s="19" t="inlineStr">
         <is>
           <t>Dopo due prese perse può diventare 74.</t>
         </is>
       </c>
-      <c r="F69" s="19" t="inlineStr">
+      <c r="F69" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G69" s="14" t="inlineStr">
+      <c r="G69" s="19" t="inlineStr">
         <is>
           <t>Alla giocata</t>
         </is>
       </c>
-      <c r="H69" s="14" t="inlineStr">
+      <c r="H69" s="19" t="inlineStr">
         <is>
           <t>Se hai perso le ultime due prese in cui hai giocato, vale 74 invece di 4. È automatico: non lo scegli tu.</t>
         </is>
       </c>
-      <c r="I69" s="14" t="inlineStr">
+      <c r="I69" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 54% delle giocate (2 giocatori: 26% · 4 giocatori: 47% · 8 giocatori: 61%). Vince il 23% delle prese in cui segue la fazione; le carte senza potere da 0–9 ne vincono il 3%.</t>
         </is>
       </c>
-      <c r="J69" s="14" t="inlineStr">
+      <c r="J69" s="19" t="inlineStr">
         <is>
           <t>Molto forte: vince il 23% delle prese contro il 3% delle carte simili. Il testo dice 'può diventare' (come una scelta), il gioco lo applica sempre.</t>
         </is>
       </c>
-      <c r="K69" s="14" t="inlineStr">
+      <c r="K69" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L69" s="14" t="inlineStr">
+      <c r="L69" s="19" t="inlineStr">
         <is>
           <t>Va bene così (automatico).</t>
         </is>
@@ -4714,10 +4865,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I70" s="14" t="inlineStr"/>
-      <c r="J70" s="14" t="inlineStr"/>
-      <c r="K70" s="14" t="inlineStr"/>
-      <c r="L70" s="14" t="inlineStr"/>
+      <c r="I70" s="14" t="n"/>
+      <c r="J70" s="14" t="n"/>
+      <c r="K70" s="14" t="n"/>
+      <c r="L70" s="14" t="n"/>
       <c r="M70" s="17" t="n"/>
       <c r="N70" s="17" t="n"/>
       <c r="O70" s="17" t="n"/>
@@ -4762,10 +4913,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I71" s="14" t="inlineStr"/>
-      <c r="J71" s="14" t="inlineStr"/>
-      <c r="K71" s="14" t="inlineStr"/>
-      <c r="L71" s="14" t="inlineStr"/>
+      <c r="I71" s="14" t="n"/>
+      <c r="J71" s="14" t="n"/>
+      <c r="K71" s="14" t="n"/>
+      <c r="L71" s="14" t="n"/>
       <c r="M71" s="17" t="n"/>
       <c r="N71" s="17" t="n"/>
       <c r="O71" s="17" t="n"/>
@@ -4810,71 +4961,75 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I72" s="14" t="inlineStr"/>
-      <c r="J72" s="14" t="inlineStr"/>
-      <c r="K72" s="14" t="inlineStr"/>
-      <c r="L72" s="14" t="inlineStr"/>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="14" t="n"/>
+      <c r="L72" s="14" t="n"/>
       <c r="M72" s="17" t="n"/>
       <c r="N72" s="17" t="n"/>
       <c r="O72" s="17" t="n"/>
       <c r="P72" s="17" t="n"/>
     </row>
     <row r="73" ht="45" customHeight="1">
-      <c r="A73" s="14" t="inlineStr">
+      <c r="A73" s="19" t="inlineStr">
         <is>
           <t>Concordia-3</t>
         </is>
       </c>
-      <c r="B73" s="14" t="inlineStr">
+      <c r="B73" s="19" t="inlineStr">
         <is>
           <t>Concordia</t>
         </is>
       </c>
-      <c r="C73" s="15" t="inlineStr">
+      <c r="C73" s="24" t="inlineStr">
         <is>
           <t>Balancer</t>
         </is>
       </c>
-      <c r="D73" s="14" t="n">
+      <c r="D73" s="19" t="n">
         <v>71</v>
       </c>
-      <c r="E73" s="14" t="inlineStr">
+      <c r="E73" s="19" t="inlineStr">
         <is>
           <t>Se sei unico ultimo in classifica, +15.</t>
         </is>
       </c>
-      <c r="F73" s="18" t="inlineStr">
-        <is>
-          <t>Non programmato</t>
-        </is>
-      </c>
-      <c r="G73" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H73" s="14" t="inlineStr">
-        <is>
-          <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
-        </is>
-      </c>
-      <c r="I73" s="14" t="inlineStr"/>
-      <c r="J73" s="14" t="inlineStr">
+      <c r="F73" s="25" t="inlineStr">
+        <is>
+          <t>Programmato</t>
+        </is>
+      </c>
+      <c r="G73" s="19" t="inlineStr">
+        <is>
+          <t>Alla giocata</t>
+        </is>
+      </c>
+      <c r="H73" s="19" t="inlineStr">
+        <is>
+          <t>+15 (vale 86) se quando la giochi sei l'unico ultimo nei punti della mano in corso.</t>
+        </is>
+      </c>
+      <c r="I73" s="19" t="n"/>
+      <c r="J73" s="19" t="inlineStr">
         <is>
           <t>'Classifica': quella della mano o quella della serie?</t>
         </is>
       </c>
-      <c r="K73" s="14" t="inlineStr">
-        <is>
-          <t>A · Serve solo la regola esatta. Nessuna meccanica nuova: basta approvare la regola.</t>
-        </is>
-      </c>
-      <c r="L73" s="14" t="inlineStr">
+      <c r="K73" s="19" t="inlineStr">
+        <is>
+          <t>Programmato nella versione 0.18.0.</t>
+        </is>
+      </c>
+      <c r="L73" s="19" t="inlineStr">
         <is>
           <t>Se sei l'unico ultimo nei punti della mano in corso, vale 86.</t>
         </is>
       </c>
-      <c r="M73" s="17" t="n"/>
+      <c r="M73" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
       <c r="N73" s="17" t="n"/>
       <c r="O73" s="17" t="n"/>
       <c r="P73" s="17" t="n"/>
@@ -4918,10 +5073,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I74" s="14" t="inlineStr"/>
-      <c r="J74" s="14" t="inlineStr"/>
-      <c r="K74" s="14" t="inlineStr"/>
-      <c r="L74" s="14" t="inlineStr"/>
+      <c r="I74" s="14" t="n"/>
+      <c r="J74" s="14" t="n"/>
+      <c r="K74" s="14" t="n"/>
+      <c r="L74" s="14" t="n"/>
       <c r="M74" s="17" t="n"/>
       <c r="N74" s="17" t="n"/>
       <c r="O74" s="17" t="n"/>
@@ -4966,131 +5121,139 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I75" s="14" t="inlineStr"/>
-      <c r="J75" s="14" t="inlineStr"/>
-      <c r="K75" s="14" t="inlineStr"/>
-      <c r="L75" s="14" t="inlineStr"/>
+      <c r="I75" s="14" t="n"/>
+      <c r="J75" s="14" t="n"/>
+      <c r="K75" s="14" t="n"/>
+      <c r="L75" s="14" t="n"/>
       <c r="M75" s="17" t="n"/>
       <c r="N75" s="17" t="n"/>
       <c r="O75" s="17" t="n"/>
       <c r="P75" s="17" t="n"/>
     </row>
     <row r="76" ht="45" customHeight="1">
-      <c r="A76" s="14" t="inlineStr">
+      <c r="A76" s="19" t="inlineStr">
         <is>
           <t>Concordia-6</t>
         </is>
       </c>
-      <c r="B76" s="14" t="inlineStr">
+      <c r="B76" s="19" t="inlineStr">
         <is>
           <t>Concordia</t>
         </is>
       </c>
-      <c r="C76" s="15" t="inlineStr">
+      <c r="C76" s="24" t="inlineStr">
         <is>
           <t>Evenhand</t>
         </is>
       </c>
-      <c r="D76" s="14" t="n">
+      <c r="D76" s="19" t="n">
         <v>47</v>
       </c>
-      <c r="E76" s="14" t="inlineStr">
+      <c r="E76" s="19" t="inlineStr">
         <is>
           <t>Se sei a pari merito ultimo, +15.</t>
         </is>
       </c>
-      <c r="F76" s="18" t="inlineStr">
-        <is>
-          <t>Non programmato</t>
-        </is>
-      </c>
-      <c r="G76" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H76" s="14" t="inlineStr">
-        <is>
-          <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
-        </is>
-      </c>
-      <c r="I76" s="14" t="inlineStr"/>
-      <c r="J76" s="14" t="inlineStr">
+      <c r="F76" s="25" t="inlineStr">
+        <is>
+          <t>Programmato</t>
+        </is>
+      </c>
+      <c r="G76" s="19" t="inlineStr">
+        <is>
+          <t>Alla giocata</t>
+        </is>
+      </c>
+      <c r="H76" s="19" t="inlineStr">
+        <is>
+          <t>+15 (vale 62) se quando la giochi sei ultimo nei punti della mano in corso a pari merito con almeno un altro giocatore. A inizio mano, con tutti a 0, vale sempre.</t>
+        </is>
+      </c>
+      <c r="I76" s="19" t="n"/>
+      <c r="J76" s="19" t="inlineStr">
         <is>
           <t>'Classifica': quella della mano o quella della serie?</t>
         </is>
       </c>
-      <c r="K76" s="14" t="inlineStr">
-        <is>
-          <t>A · Serve solo la regola esatta. Nessuna meccanica nuova: basta approvare la regola.</t>
-        </is>
-      </c>
-      <c r="L76" s="14" t="inlineStr">
+      <c r="K76" s="19" t="inlineStr">
+        <is>
+          <t>Programmato nella versione 0.18.0.</t>
+        </is>
+      </c>
+      <c r="L76" s="19" t="inlineStr">
         <is>
           <t>Se sei ultimo a pari merito con almeno un altro giocatore, vale 62.</t>
         </is>
       </c>
-      <c r="M76" s="17" t="n"/>
+      <c r="M76" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
       <c r="N76" s="17" t="n"/>
       <c r="O76" s="17" t="n"/>
       <c r="P76" s="17" t="n"/>
     </row>
     <row r="77" ht="45" customHeight="1">
-      <c r="A77" s="14" t="inlineStr">
+      <c r="A77" s="19" t="inlineStr">
         <is>
           <t>Concordia-7</t>
         </is>
       </c>
-      <c r="B77" s="14" t="inlineStr">
+      <c r="B77" s="19" t="inlineStr">
         <is>
           <t>Concordia</t>
         </is>
       </c>
-      <c r="C77" s="15" t="inlineStr">
+      <c r="C77" s="24" t="inlineStr">
         <is>
           <t>Symmetra</t>
         </is>
       </c>
-      <c r="D77" s="14" t="n">
+      <c r="D77" s="19" t="n">
         <v>39</v>
       </c>
-      <c r="E77" s="14" t="inlineStr">
+      <c r="E77" s="19" t="inlineStr">
         <is>
           <t>Se il range è 40+, diventa 69.</t>
         </is>
       </c>
-      <c r="F77" s="18" t="inlineStr">
-        <is>
-          <t>Non programmato</t>
-        </is>
-      </c>
-      <c r="G77" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H77" s="14" t="inlineStr">
-        <is>
-          <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
-        </is>
-      </c>
-      <c r="I77" s="14" t="inlineStr"/>
-      <c r="J77" s="14" t="inlineStr">
+      <c r="F77" s="25" t="inlineStr">
+        <is>
+          <t>Programmato</t>
+        </is>
+      </c>
+      <c r="G77" s="19" t="inlineStr">
+        <is>
+          <t>Alla rivelazione</t>
+        </is>
+      </c>
+      <c r="H77" s="19" t="inlineStr">
+        <is>
+          <t>Vale 69 se tra il valore finale più alto e il più basso della presa ci sono almeno 40 punti (guardando i valori prima degli altri poteri della rivelazione).</t>
+        </is>
+      </c>
+      <c r="I77" s="19" t="n"/>
+      <c r="J77" s="19" t="inlineStr">
         <is>
           <t>'Range' va definito.</t>
         </is>
       </c>
-      <c r="K77" s="14" t="inlineStr">
-        <is>
-          <t>A · Serve solo la regola esatta. Nessuna meccanica nuova: basta approvare la regola.</t>
-        </is>
-      </c>
-      <c r="L77" s="14" t="inlineStr">
+      <c r="K77" s="19" t="inlineStr">
+        <is>
+          <t>Programmato nella versione 0.18.0.</t>
+        </is>
+      </c>
+      <c r="L77" s="19" t="inlineStr">
         <is>
           <t>Se tra il valore finale più alto e il più basso della presa ci sono almeno 40 punti, vale 69 (l'opposto di Equalis).</t>
         </is>
       </c>
-      <c r="M77" s="17" t="n"/>
+      <c r="M77" s="17" t="inlineStr">
+        <is>
+          <t>Usa la proposta</t>
+        </is>
+      </c>
       <c r="N77" s="17" t="n"/>
       <c r="O77" s="17" t="n"/>
       <c r="P77" s="17" t="n"/>
@@ -5134,10 +5297,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I78" s="14" t="inlineStr"/>
-      <c r="J78" s="14" t="inlineStr"/>
-      <c r="K78" s="14" t="inlineStr"/>
-      <c r="L78" s="14" t="inlineStr"/>
+      <c r="I78" s="14" t="n"/>
+      <c r="J78" s="14" t="n"/>
+      <c r="K78" s="14" t="n"/>
+      <c r="L78" s="14" t="n"/>
       <c r="M78" s="17" t="n"/>
       <c r="N78" s="17" t="n"/>
       <c r="O78" s="17" t="n"/>
@@ -5182,10 +5345,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I79" s="14" t="inlineStr"/>
-      <c r="J79" s="14" t="inlineStr"/>
-      <c r="K79" s="14" t="inlineStr"/>
-      <c r="L79" s="14" t="inlineStr"/>
+      <c r="I79" s="14" t="n"/>
+      <c r="J79" s="14" t="n"/>
+      <c r="K79" s="14" t="n"/>
+      <c r="L79" s="14" t="n"/>
       <c r="M79" s="17" t="n"/>
       <c r="N79" s="17" t="n"/>
       <c r="O79" s="17" t="n"/>
@@ -5230,7 +5393,7 @@
           <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
         </is>
       </c>
-      <c r="I80" s="14" t="inlineStr"/>
+      <c r="I80" s="14" t="n"/>
       <c r="J80" s="14" t="inlineStr">
         <is>
           <t>'Perdite di punti carta' non è definito.</t>
@@ -5251,61 +5414,61 @@
       <c r="O80" s="17" t="n"/>
       <c r="P80" s="17" t="n"/>
     </row>
-    <row r="81" ht="71" customHeight="1">
-      <c r="A81" s="14" t="inlineStr">
+    <row r="81" ht="70.95" customHeight="1">
+      <c r="A81" s="19" t="inlineStr">
         <is>
           <t>Concordia-11</t>
         </is>
       </c>
-      <c r="B81" s="14" t="inlineStr">
+      <c r="B81" s="19" t="inlineStr">
         <is>
           <t>Concordia</t>
         </is>
       </c>
-      <c r="C81" s="15" t="inlineStr">
+      <c r="C81" s="24" t="inlineStr">
         <is>
           <t>Equalis</t>
         </is>
       </c>
-      <c r="D81" s="14" t="n">
+      <c r="D81" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="E81" s="14" t="inlineStr">
+      <c r="E81" s="19" t="inlineStr">
         <is>
           <t>Se il range è ≤20, diventa 77.</t>
         </is>
       </c>
-      <c r="F81" s="19" t="inlineStr">
+      <c r="F81" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G81" s="14" t="inlineStr">
+      <c r="G81" s="19" t="inlineStr">
         <is>
           <t>Alla rivelazione</t>
         </is>
       </c>
-      <c r="H81" s="14" t="inlineStr">
+      <c r="H81" s="19" t="inlineStr">
         <is>
           <t>Se la differenza tra il valore finale più alto e il più basso della presa è 20 o meno, Equalis vale 77.</t>
         </is>
       </c>
-      <c r="I81" s="14" t="inlineStr">
+      <c r="I81" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 6% delle giocate (2 giocatori: 51% · 4 giocatori: 6% · 8 giocatori: 1%). Vince il 9% delle prese in cui segue la fazione; le carte senza potere da 0–9 ne vincono il 3%.</t>
         </is>
       </c>
-      <c r="J81" s="14" t="inlineStr">
+      <c r="J81" s="19" t="inlineStr">
         <is>
           <t>Funziona solo in 2 giocatori (51% delle volte). Con 4 giocatori scende al 6%, con 8 all'1%.</t>
         </is>
       </c>
-      <c r="K81" s="14" t="inlineStr">
+      <c r="K81" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L81" s="14" t="inlineStr">
+      <c r="L81" s="19" t="inlineStr">
         <is>
           <t>Soglia che cresce con i giocatori: differenza ≤ 20 × (giocatori − 1). Oppure una soglia fissa ≤ 40.</t>
         </is>
@@ -5354,10 +5517,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I82" s="14" t="inlineStr"/>
-      <c r="J82" s="14" t="inlineStr"/>
-      <c r="K82" s="14" t="inlineStr"/>
-      <c r="L82" s="14" t="inlineStr"/>
+      <c r="I82" s="14" t="n"/>
+      <c r="J82" s="14" t="n"/>
+      <c r="K82" s="14" t="n"/>
+      <c r="L82" s="14" t="n"/>
       <c r="M82" s="17" t="n"/>
       <c r="N82" s="17" t="n"/>
       <c r="O82" s="17" t="n"/>
@@ -5402,10 +5565,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I83" s="14" t="inlineStr"/>
-      <c r="J83" s="14" t="inlineStr"/>
-      <c r="K83" s="14" t="inlineStr"/>
-      <c r="L83" s="14" t="inlineStr"/>
+      <c r="I83" s="14" t="n"/>
+      <c r="J83" s="14" t="n"/>
+      <c r="K83" s="14" t="n"/>
+      <c r="L83" s="14" t="n"/>
       <c r="M83" s="17" t="n"/>
       <c r="N83" s="17" t="n"/>
       <c r="O83" s="17" t="n"/>
@@ -5450,70 +5613,70 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I84" s="14" t="inlineStr"/>
-      <c r="J84" s="14" t="inlineStr"/>
-      <c r="K84" s="14" t="inlineStr"/>
-      <c r="L84" s="14" t="inlineStr"/>
+      <c r="I84" s="14" t="n"/>
+      <c r="J84" s="14" t="n"/>
+      <c r="K84" s="14" t="n"/>
+      <c r="L84" s="14" t="n"/>
       <c r="M84" s="17" t="n"/>
       <c r="N84" s="17" t="n"/>
       <c r="O84" s="17" t="n"/>
       <c r="P84" s="17" t="n"/>
     </row>
-    <row r="85" ht="71" customHeight="1">
-      <c r="A85" s="14" t="inlineStr">
+    <row r="85" ht="70.95" customHeight="1">
+      <c r="A85" s="19" t="inlineStr">
         <is>
           <t>Axiomata-2</t>
         </is>
       </c>
-      <c r="B85" s="14" t="inlineStr">
+      <c r="B85" s="19" t="inlineStr">
         <is>
           <t>Axiomata</t>
         </is>
       </c>
-      <c r="C85" s="15" t="inlineStr">
+      <c r="C85" s="24" t="inlineStr">
         <is>
           <t>Veritas</t>
         </is>
       </c>
-      <c r="D85" s="14" t="n">
+      <c r="D85" s="19" t="n">
         <v>80</v>
       </c>
-      <c r="E85" s="14" t="inlineStr">
+      <c r="E85" s="19" t="inlineStr">
         <is>
           <t>Il valore resta sempre 80.</t>
         </is>
       </c>
-      <c r="F85" s="19" t="inlineStr">
+      <c r="F85" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G85" s="14" t="inlineStr">
+      <c r="G85" s="19" t="inlineStr">
         <is>
           <t>Alla giocata</t>
         </is>
       </c>
-      <c r="H85" s="14" t="inlineStr">
+      <c r="H85" s="19" t="inlineStr">
         <is>
           <t>Vale sempre 80, anche se hai un bonus o un malus in sospeso (da Praetor, Bloodmark o Vesper Null). Se nella presa c'è Axiom resta comunque 80, il suo valore stampato.</t>
         </is>
       </c>
-      <c r="I85" s="14" t="inlineStr">
+      <c r="I85" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 1% delle giocate (2 giocatori: 1% · 4 giocatori: 0% · 8 giocatori: 1%). Vince il 48% delle prese in cui segue la fazione; le carte senza potere da 80–89 ne vincono il 63%.</t>
         </is>
       </c>
-      <c r="J85" s="14" t="inlineStr">
+      <c r="J85" s="19" t="inlineStr">
         <is>
           <t>Vale già 80 stampato: il potere cambia qualcosa solo nell'1% delle giocate. In pratica è un 80 normale.</t>
         </is>
       </c>
-      <c r="K85" s="14" t="inlineStr">
+      <c r="K85" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L85" s="14" t="inlineStr">
+      <c r="L85" s="19" t="inlineStr">
         <is>
           <t>Se Veritas è nella presa, nessuna carta può valere più di 80: i valori sopra 80 scendono a 80.</t>
         </is>
@@ -5562,10 +5725,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I86" s="14" t="inlineStr"/>
-      <c r="J86" s="14" t="inlineStr"/>
-      <c r="K86" s="14" t="inlineStr"/>
-      <c r="L86" s="14" t="inlineStr"/>
+      <c r="I86" s="14" t="n"/>
+      <c r="J86" s="14" t="n"/>
+      <c r="K86" s="14" t="n"/>
+      <c r="L86" s="14" t="n"/>
       <c r="M86" s="17" t="n"/>
       <c r="N86" s="17" t="n"/>
       <c r="O86" s="17" t="n"/>
@@ -5610,70 +5773,70 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I87" s="14" t="inlineStr"/>
-      <c r="J87" s="14" t="inlineStr"/>
-      <c r="K87" s="14" t="inlineStr"/>
-      <c r="L87" s="14" t="inlineStr"/>
+      <c r="I87" s="14" t="n"/>
+      <c r="J87" s="14" t="n"/>
+      <c r="K87" s="14" t="n"/>
+      <c r="L87" s="14" t="n"/>
       <c r="M87" s="17" t="n"/>
       <c r="N87" s="17" t="n"/>
       <c r="O87" s="17" t="n"/>
       <c r="P87" s="17" t="n"/>
     </row>
-    <row r="88" ht="97" customHeight="1">
-      <c r="A88" s="14" t="inlineStr">
+    <row r="88" ht="97.05" customHeight="1">
+      <c r="A88" s="19" t="inlineStr">
         <is>
           <t>Axiomata-5</t>
         </is>
       </c>
-      <c r="B88" s="14" t="inlineStr">
+      <c r="B88" s="19" t="inlineStr">
         <is>
           <t>Axiomata</t>
         </is>
       </c>
-      <c r="C88" s="15" t="inlineStr">
+      <c r="C88" s="24" t="inlineStr">
         <is>
           <t>Axiom</t>
         </is>
       </c>
-      <c r="D88" s="14" t="n">
+      <c r="D88" s="19" t="n">
         <v>55</v>
       </c>
-      <c r="E88" s="14" t="inlineStr">
+      <c r="E88" s="19" t="inlineStr">
         <is>
           <t>Annulla gli altri effetti nella presa.</t>
         </is>
       </c>
-      <c r="F88" s="19" t="inlineStr">
+      <c r="F88" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G88" s="14" t="inlineStr">
+      <c r="G88" s="19" t="inlineStr">
         <is>
           <t>Alla rivelazione (prima di ogni altro potere)</t>
         </is>
       </c>
-      <c r="H88" s="14" t="inlineStr">
+      <c r="H88" s="19" t="inlineStr">
         <is>
           <t>Quando tutte le carte sono sul tavolo, ogni carta della presa torna al suo valore stampato: annulla bonus e malus in sospeso e tutti i poteri che cambiano valore (Invariant, Veritas, Ascendant, Switch, Equalis, Wildcard, Measure…), anche quelli degli avversari. Non blocca i poteri 'dopo la presa' (punti e bonus futuri).</t>
         </is>
       </c>
-      <c r="I88" s="14" t="inlineStr">
+      <c r="I88" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 69% delle giocate (2 giocatori: 27% · 4 giocatori: 53% · 8 giocatori: 82%). Vince il 24% delle prese in cui segue la fazione; le carte senza potere da 50–59 ne vincono il 20%.</t>
         </is>
       </c>
-      <c r="J88" s="14" t="inlineStr">
+      <c r="J88" s="19" t="inlineStr">
         <is>
           <t>Più forte con tanti giocatori: si attiva nel 27% dei casi in 2, nell'82% in 8.</t>
         </is>
       </c>
-      <c r="K88" s="14" t="inlineStr">
+      <c r="K88" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L88" s="14" t="inlineStr">
+      <c r="L88" s="19" t="inlineStr">
         <is>
           <t>Va bene così.</t>
         </is>
@@ -5722,70 +5885,70 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I89" s="14" t="inlineStr"/>
-      <c r="J89" s="14" t="inlineStr"/>
-      <c r="K89" s="14" t="inlineStr"/>
-      <c r="L89" s="14" t="inlineStr"/>
+      <c r="I89" s="14" t="n"/>
+      <c r="J89" s="14" t="n"/>
+      <c r="K89" s="14" t="n"/>
+      <c r="L89" s="14" t="n"/>
       <c r="M89" s="17" t="n"/>
       <c r="N89" s="17" t="n"/>
       <c r="O89" s="17" t="n"/>
       <c r="P89" s="17" t="n"/>
     </row>
-    <row r="90" ht="71" customHeight="1">
-      <c r="A90" s="14" t="inlineStr">
+    <row r="90" ht="70.95" customHeight="1">
+      <c r="A90" s="19" t="inlineStr">
         <is>
           <t>Axiomata-7</t>
         </is>
       </c>
-      <c r="B90" s="14" t="inlineStr">
+      <c r="B90" s="19" t="inlineStr">
         <is>
           <t>Axiomata</t>
         </is>
       </c>
-      <c r="C90" s="15" t="inlineStr">
+      <c r="C90" s="24" t="inlineStr">
         <is>
           <t>Measure</t>
         </is>
       </c>
-      <c r="D90" s="14" t="n">
+      <c r="D90" s="19" t="n">
         <v>39</v>
       </c>
-      <c r="E90" s="14" t="inlineStr">
+      <c r="E90" s="19" t="inlineStr">
         <is>
           <t>Limita i valori tra 10 e 90.</t>
         </is>
       </c>
-      <c r="F90" s="19" t="inlineStr">
+      <c r="F90" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G90" s="14" t="inlineStr">
+      <c r="G90" s="19" t="inlineStr">
         <is>
           <t>Alla rivelazione (dopo Switch, Equalis e Wildcard)</t>
         </is>
       </c>
-      <c r="H90" s="14" t="inlineStr">
+      <c r="H90" s="19" t="inlineStr">
         <is>
           <t>Tutti i valori finali della presa vengono portati tra 10 e 90: sotto 10 diventano 10, sopra 90 diventano 90.</t>
         </is>
       </c>
-      <c r="I90" s="14" t="inlineStr">
+      <c r="I90" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 51% delle giocate (2 giocatori: 20% · 4 giocatori: 47% · 8 giocatori: 60%). Vince il 9% delle prese in cui segue la fazione; le carte senza potere da 30–39 ne vincono il 10%.</t>
         </is>
       </c>
-      <c r="J90" s="14" t="inlineStr">
+      <c r="J90" s="19" t="inlineStr">
         <is>
           <t>Effetto collaterale: le carte da 91 a 99 diventano 90 e a parità vince il valore stampato più basso. Con Measure in presa, quindi, un 90 batte un 99.</t>
         </is>
       </c>
-      <c r="K90" s="14" t="inlineStr">
+      <c r="K90" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L90" s="14" t="inlineStr">
+      <c r="L90" s="19" t="inlineStr">
         <is>
           <t>Va bene così se l'effetto è voluto; altrimenti, nei pareggi creati da Measure vince il valore stampato più alto.</t>
         </is>
@@ -5834,10 +5997,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I91" s="14" t="inlineStr"/>
-      <c r="J91" s="14" t="inlineStr"/>
-      <c r="K91" s="14" t="inlineStr"/>
-      <c r="L91" s="14" t="inlineStr"/>
+      <c r="I91" s="14" t="n"/>
+      <c r="J91" s="14" t="n"/>
+      <c r="K91" s="14" t="n"/>
+      <c r="L91" s="14" t="n"/>
       <c r="M91" s="17" t="n"/>
       <c r="N91" s="17" t="n"/>
       <c r="O91" s="17" t="n"/>
@@ -5882,10 +6045,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I92" s="14" t="inlineStr"/>
-      <c r="J92" s="14" t="inlineStr"/>
-      <c r="K92" s="14" t="inlineStr"/>
-      <c r="L92" s="14" t="inlineStr"/>
+      <c r="I92" s="14" t="n"/>
+      <c r="J92" s="14" t="n"/>
+      <c r="K92" s="14" t="n"/>
+      <c r="L92" s="14" t="n"/>
       <c r="M92" s="17" t="n"/>
       <c r="N92" s="17" t="n"/>
       <c r="O92" s="17" t="n"/>
@@ -5930,70 +6093,70 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I93" s="14" t="inlineStr"/>
-      <c r="J93" s="14" t="inlineStr"/>
-      <c r="K93" s="14" t="inlineStr"/>
-      <c r="L93" s="14" t="inlineStr"/>
+      <c r="I93" s="14" t="n"/>
+      <c r="J93" s="14" t="n"/>
+      <c r="K93" s="14" t="n"/>
+      <c r="L93" s="14" t="n"/>
       <c r="M93" s="17" t="n"/>
       <c r="N93" s="17" t="n"/>
       <c r="O93" s="17" t="n"/>
       <c r="P93" s="17" t="n"/>
     </row>
-    <row r="94" ht="71" customHeight="1">
-      <c r="A94" s="14" t="inlineStr">
+    <row r="94" ht="70.95" customHeight="1">
+      <c r="A94" s="19" t="inlineStr">
         <is>
           <t>Axiomata-11</t>
         </is>
       </c>
-      <c r="B94" s="14" t="inlineStr">
+      <c r="B94" s="19" t="inlineStr">
         <is>
           <t>Axiomata</t>
         </is>
       </c>
-      <c r="C94" s="15" t="inlineStr">
+      <c r="C94" s="24" t="inlineStr">
         <is>
           <t>Invariant</t>
         </is>
       </c>
-      <c r="D94" s="14" t="n">
+      <c r="D94" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="E94" s="14" t="inlineStr">
+      <c r="E94" s="19" t="inlineStr">
         <is>
           <t>Per il confronto vale sempre 50.</t>
         </is>
       </c>
-      <c r="F94" s="19" t="inlineStr">
+      <c r="F94" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G94" s="14" t="inlineStr">
+      <c r="G94" s="19" t="inlineStr">
         <is>
           <t>Alla giocata</t>
         </is>
       </c>
-      <c r="H94" s="14" t="inlineStr">
+      <c r="H94" s="19" t="inlineStr">
         <is>
           <t>Vale 50 invece di 8, anche con un bonus o un malus in sospeso. Se nella presa c'è Axiom torna a 8.</t>
         </is>
       </c>
-      <c r="I94" s="14" t="inlineStr">
+      <c r="I94" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 80% delle giocate (2 giocatori: 94% · 4 giocatori: 88% · 8 giocatori: 73%). Vince il 27% delle prese in cui segue la fazione; le carte senza potere da 0–9 ne vincono il 3%.</t>
         </is>
       </c>
-      <c r="J94" s="14" t="inlineStr">
+      <c r="J94" s="19" t="inlineStr">
         <is>
           <t>Fortissimo: vince il 27% delle prese in cui segue la fazione, contro il 3% delle carte normali di valore simile. Forse è voluto: da valutare.</t>
         </is>
       </c>
-      <c r="K94" s="14" t="inlineStr">
+      <c r="K94" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L94" s="14" t="inlineStr">
+      <c r="L94" s="19" t="inlineStr">
         <is>
           <t>Va bene così; se lo trovi troppo forte, 40 invece di 50.</t>
         </is>
@@ -6042,10 +6205,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I95" s="14" t="inlineStr"/>
-      <c r="J95" s="14" t="inlineStr"/>
-      <c r="K95" s="14" t="inlineStr"/>
-      <c r="L95" s="14" t="inlineStr"/>
+      <c r="I95" s="14" t="n"/>
+      <c r="J95" s="14" t="n"/>
+      <c r="K95" s="14" t="n"/>
+      <c r="L95" s="14" t="n"/>
       <c r="M95" s="17" t="n"/>
       <c r="N95" s="17" t="n"/>
       <c r="O95" s="17" t="n"/>
@@ -6090,10 +6253,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I96" s="14" t="inlineStr"/>
-      <c r="J96" s="14" t="inlineStr"/>
-      <c r="K96" s="14" t="inlineStr"/>
-      <c r="L96" s="14" t="inlineStr"/>
+      <c r="I96" s="14" t="n"/>
+      <c r="J96" s="14" t="n"/>
+      <c r="K96" s="14" t="n"/>
+      <c r="L96" s="14" t="n"/>
       <c r="M96" s="17" t="n"/>
       <c r="N96" s="17" t="n"/>
       <c r="O96" s="17" t="n"/>
@@ -6138,16 +6301,16 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I97" s="14" t="inlineStr"/>
-      <c r="J97" s="14" t="inlineStr"/>
-      <c r="K97" s="14" t="inlineStr"/>
-      <c r="L97" s="14" t="inlineStr"/>
+      <c r="I97" s="14" t="n"/>
+      <c r="J97" s="14" t="n"/>
+      <c r="K97" s="14" t="n"/>
+      <c r="L97" s="14" t="n"/>
       <c r="M97" s="17" t="n"/>
       <c r="N97" s="17" t="n"/>
       <c r="O97" s="17" t="n"/>
       <c r="P97" s="17" t="n"/>
     </row>
-    <row r="98" ht="58" customHeight="1">
+    <row r="98" ht="58.05" customHeight="1">
       <c r="A98" s="14" t="inlineStr">
         <is>
           <t>Conflux-2</t>
@@ -6186,7 +6349,7 @@
           <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
         </is>
       </c>
-      <c r="I98" s="14" t="inlineStr"/>
+      <c r="I98" s="14" t="n"/>
       <c r="J98" s="14" t="inlineStr">
         <is>
           <t>Non dice quando si sceglie.</t>
@@ -6207,7 +6370,7 @@
       <c r="O98" s="17" t="n"/>
       <c r="P98" s="17" t="n"/>
     </row>
-    <row r="99" ht="58" customHeight="1">
+    <row r="99" ht="58.05" customHeight="1">
       <c r="A99" s="14" t="inlineStr">
         <is>
           <t>Conflux-3</t>
@@ -6246,7 +6409,7 @@
           <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
         </is>
       </c>
-      <c r="I99" s="14" t="inlineStr"/>
+      <c r="I99" s="14" t="n"/>
       <c r="J99" s="14" t="inlineStr">
         <is>
           <t>Non dice quando si sceglie.</t>
@@ -6306,10 +6469,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I100" s="14" t="inlineStr"/>
-      <c r="J100" s="14" t="inlineStr"/>
-      <c r="K100" s="14" t="inlineStr"/>
-      <c r="L100" s="14" t="inlineStr"/>
+      <c r="I100" s="14" t="n"/>
+      <c r="J100" s="14" t="n"/>
+      <c r="K100" s="14" t="n"/>
+      <c r="L100" s="14" t="n"/>
       <c r="M100" s="17" t="n"/>
       <c r="N100" s="17" t="n"/>
       <c r="O100" s="17" t="n"/>
@@ -6354,70 +6517,70 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I101" s="14" t="inlineStr"/>
-      <c r="J101" s="14" t="inlineStr"/>
-      <c r="K101" s="14" t="inlineStr"/>
-      <c r="L101" s="14" t="inlineStr"/>
+      <c r="I101" s="14" t="n"/>
+      <c r="J101" s="14" t="n"/>
+      <c r="K101" s="14" t="n"/>
+      <c r="L101" s="14" t="n"/>
       <c r="M101" s="17" t="n"/>
       <c r="N101" s="17" t="n"/>
       <c r="O101" s="17" t="n"/>
       <c r="P101" s="17" t="n"/>
     </row>
-    <row r="102" ht="71" customHeight="1">
-      <c r="A102" s="14" t="inlineStr">
+    <row r="102" ht="70.95" customHeight="1">
+      <c r="A102" s="19" t="inlineStr">
         <is>
           <t>Conflux-6</t>
         </is>
       </c>
-      <c r="B102" s="14" t="inlineStr">
+      <c r="B102" s="19" t="inlineStr">
         <is>
           <t>Conflux</t>
         </is>
       </c>
-      <c r="C102" s="15" t="inlineStr">
+      <c r="C102" s="24" t="inlineStr">
         <is>
           <t>Switch</t>
         </is>
       </c>
-      <c r="D102" s="14" t="n">
+      <c r="D102" s="19" t="n">
         <v>51</v>
       </c>
-      <c r="E102" s="14" t="inlineStr">
+      <c r="E102" s="19" t="inlineStr">
         <is>
           <t>Se ci sono un 80+ e un ≤20, diventa 91.</t>
         </is>
       </c>
-      <c r="F102" s="19" t="inlineStr">
+      <c r="F102" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G102" s="14" t="inlineStr">
+      <c r="G102" s="19" t="inlineStr">
         <is>
           <t>Alla rivelazione</t>
         </is>
       </c>
-      <c r="H102" s="14" t="inlineStr">
+      <c r="H102" s="19" t="inlineStr">
         <is>
           <t>Se nella presa c'è almeno una carta con valore finale 80 o più E una con valore finale 20 o meno, Switch vale 91.</t>
         </is>
       </c>
-      <c r="I102" s="14" t="inlineStr">
+      <c r="I102" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 32% delle giocate (2 giocatori: 0% · 4 giocatori: 12% · 8 giocatori: 51%). Vince il 36% delle prese in cui segue la fazione; le carte senza potere da 50–59 ne vincono il 20%.</t>
         </is>
       </c>
-      <c r="J102" s="14" t="inlineStr">
+      <c r="J102" s="19" t="inlineStr">
         <is>
           <t>Non si attiva mai in 2 giocatori, si attiva nel 51% dei casi in 8: dipende moltissimo dal numero di giocatori.</t>
         </is>
       </c>
-      <c r="K102" s="14" t="inlineStr">
+      <c r="K102" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L102" s="14" t="inlineStr">
+      <c r="L102" s="19" t="inlineStr">
         <is>
           <t>Va bene così; in alternativa, in 2 giocatori basta una delle due condizioni.</t>
         </is>
@@ -6466,10 +6629,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I103" s="14" t="inlineStr"/>
-      <c r="J103" s="14" t="inlineStr"/>
-      <c r="K103" s="14" t="inlineStr"/>
-      <c r="L103" s="14" t="inlineStr"/>
+      <c r="I103" s="14" t="n"/>
+      <c r="J103" s="14" t="n"/>
+      <c r="K103" s="14" t="n"/>
+      <c r="L103" s="14" t="n"/>
       <c r="M103" s="17" t="n"/>
       <c r="N103" s="17" t="n"/>
       <c r="O103" s="17" t="n"/>
@@ -6514,10 +6677,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I104" s="14" t="inlineStr"/>
-      <c r="J104" s="14" t="inlineStr"/>
-      <c r="K104" s="14" t="inlineStr"/>
-      <c r="L104" s="14" t="inlineStr"/>
+      <c r="I104" s="14" t="n"/>
+      <c r="J104" s="14" t="n"/>
+      <c r="K104" s="14" t="n"/>
+      <c r="L104" s="14" t="n"/>
       <c r="M104" s="17" t="n"/>
       <c r="N104" s="17" t="n"/>
       <c r="O104" s="17" t="n"/>
@@ -6562,7 +6725,7 @@
           <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
         </is>
       </c>
-      <c r="I105" s="14" t="inlineStr"/>
+      <c r="I105" s="14" t="n"/>
       <c r="J105" s="14" t="inlineStr">
         <is>
           <t>'Carta precedente' va definita.</t>
@@ -6583,7 +6746,7 @@
       <c r="O105" s="17" t="n"/>
       <c r="P105" s="17" t="n"/>
     </row>
-    <row r="106" ht="58" customHeight="1">
+    <row r="106" ht="58.05" customHeight="1">
       <c r="A106" s="14" t="inlineStr">
         <is>
           <t>Conflux-10</t>
@@ -6622,7 +6785,7 @@
           <t>Niente: il testo si vede sulla carta, ma il gioco non lo applica (la carta mostra 'potere non ancora attivo').</t>
         </is>
       </c>
-      <c r="I106" s="14" t="inlineStr"/>
+      <c r="I106" s="14" t="n"/>
       <c r="J106" s="14" t="inlineStr">
         <is>
           <t>Non dice quando si sceglie.</t>
@@ -6643,61 +6806,61 @@
       <c r="O106" s="17" t="n"/>
       <c r="P106" s="17" t="n"/>
     </row>
-    <row r="107" ht="71" customHeight="1">
-      <c r="A107" s="14" t="inlineStr">
+    <row r="107" ht="70.95" customHeight="1">
+      <c r="A107" s="19" t="inlineStr">
         <is>
           <t>Conflux-11</t>
         </is>
       </c>
-      <c r="B107" s="14" t="inlineStr">
+      <c r="B107" s="19" t="inlineStr">
         <is>
           <t>Conflux</t>
         </is>
       </c>
-      <c r="C107" s="15" t="inlineStr">
+      <c r="C107" s="24" t="inlineStr">
         <is>
           <t>Wildcard</t>
         </is>
       </c>
-      <c r="D107" s="14" t="n">
+      <c r="D107" s="19" t="n">
         <v>11</v>
       </c>
-      <c r="E107" s="14" t="inlineStr">
+      <c r="E107" s="19" t="inlineStr">
         <is>
           <t>Diventa il valore avversario più basso +1.</t>
         </is>
       </c>
-      <c r="F107" s="19" t="inlineStr">
+      <c r="F107" s="25" t="inlineStr">
         <is>
           <t>Programmato</t>
         </is>
       </c>
-      <c r="G107" s="14" t="inlineStr">
+      <c r="G107" s="19" t="inlineStr">
         <is>
           <t>Alla rivelazione</t>
         </is>
       </c>
-      <c r="H107" s="14" t="inlineStr">
+      <c r="H107" s="19" t="inlineStr">
         <is>
           <t>Vale il valore stampato più basso tra le carte degli avversari nella presa, +1.</t>
         </is>
       </c>
-      <c r="I107" s="14" t="inlineStr">
+      <c r="I107" s="19" t="inlineStr">
         <is>
           <t>Si attiva nel 98% delle giocate (2 giocatori: 100% · 4 giocatori: 99% · 8 giocatori: 96%). Vince il 11% delle prese in cui segue la fazione; le carte senza potere da 10–19 ne vincono il 6%.</t>
         </is>
       </c>
-      <c r="J107" s="14" t="inlineStr">
+      <c r="J107" s="19" t="inlineStr">
         <is>
           <t>Si attiva quasi sempre, ma spesso resta un valore basso. Usa i valori stampati degli avversari, non quelli finali.</t>
         </is>
       </c>
-      <c r="K107" s="14" t="inlineStr">
+      <c r="K107" s="19" t="inlineStr">
         <is>
           <t>Già programmato.</t>
         </is>
       </c>
-      <c r="L107" s="14" t="inlineStr">
+      <c r="L107" s="19" t="inlineStr">
         <is>
           <t>Va bene così; decidi solo se usare i valori stampati o quelli finali.</t>
         </is>
@@ -6746,10 +6909,10 @@
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I108" s="14" t="inlineStr"/>
-      <c r="J108" s="14" t="inlineStr"/>
-      <c r="K108" s="14" t="inlineStr"/>
-      <c r="L108" s="14" t="inlineStr"/>
+      <c r="I108" s="14" t="n"/>
+      <c r="J108" s="14" t="n"/>
+      <c r="K108" s="14" t="n"/>
+      <c r="L108" s="14" t="n"/>
       <c r="M108" s="17" t="n"/>
       <c r="N108" s="17" t="n"/>
       <c r="O108" s="17" t="n"/>
@@ -6773,18 +6936,17 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="36" customWidth="1" min="3" max="3"/>
     <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="5" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Decisioni generali</t>
@@ -7091,19 +7253,20 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Come il gioco applica i poteri</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="20" t="inlineStr">
         <is>
@@ -7112,11 +7275,11 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Appena la carta viene giocata si calcola il suo valore: valore stampato + eventuale bonus o malus in sospeso, poi i poteri 'alla giocata' (Veritas, Invariant, Ascendant, Challenger, Gravemind, Afterimage). Il valore resta tra 0 e 100.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="32" customHeight="1">
+          <t>Appena la carta viene giocata si calcola il suo valore: valore stampato + eventuale bonus o malus in sospeso, poi i poteri 'alla giocata' (Veritas, Invariant, Ascendant, Challenger, Gravemind, Afterimage, Balancer, Evenhand) e i pagamenti scelti per Fury e Ashen. Palimpsest prende qui il potere che copia. Il valore resta tra 0 e 100. Vigil: se apre la presa, chi segue deve giocare la sua carta più alta di quella fazione.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="31.95" customHeight="1">
       <c r="A4" s="20" t="inlineStr">
         <is>
           <t>2 · Alla rivelazione</t>
@@ -7124,11 +7287,11 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Quando tutti hanno giocato: se c'è Axiom, tutte le carte tornano al valore stampato e ci si ferma qui. Altrimenti si applicano Switch, Equalis e Wildcard (guardando i valori prima di queste modifiche), poi Measure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="32" customHeight="1">
+          <t>Quando tutti hanno giocato: se c'è Axiom, tutte le carte tornano al valore stampato e ci si ferma qui. Altrimenti si applicano Switch, Equalis, Symmetra e Wildcard (guardando i valori prima di queste modifiche), poi Paradox, poi Measure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31.95" customHeight="1">
       <c r="A5" s="20" t="inlineStr">
         <is>
           <t>3 · Chi vince</t>
@@ -7140,7 +7303,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1">
+    <row r="6" ht="19.95" customHeight="1">
       <c r="A6" s="20" t="inlineStr">
         <is>
           <t>4 · Punti del Contratto</t>
@@ -7152,7 +7315,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1">
+    <row r="7" ht="31.95" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
           <t>5 · Dopo la presa</t>
@@ -7160,11 +7323,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Nell'ordine in cui sono state giocate: Origin, Zero, Praetor, Bloodmark, Vesper Null, Maledict, Rebel, Ravager.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
+          <t>Nell'ordine in cui sono state giocate: Origin, Zero, Praetor, Bloodmark, Vesper Null, Maledict, Rebel, Ravager, Morrowshade, Nullchild. Poi, se c'è Reversal e la presa ha dato o tolto punti, chi l'ha catturata decide se annullarli.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9" ht="16.8" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Parole usate nel file</t>
@@ -7231,7 +7395,8 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="15"/>
+    <row r="16" ht="16.8" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Prese vinte dalle carte senza potere</t>

</xml_diff>

<commit_message>
File dei poteri: in verde anche le carte senza potere
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/NEXUM_poteri.xlsx
+++ b/docs/NEXUM_poteri.xlsx
@@ -781,7 +781,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Riga verde: carta a posto. Il potere è programmato (il gioco lo applica) oppure è stato tolto su tua decisione. Puoi sempre cambiarla: compila le colonne gialle.</t>
+          <t>Riga verde: carta a posto. Il potere è programmato (il gioco lo applica), è stato tolto su tua decisione, oppure la carta non ha poteri. Puoi sempre cambiarla: compila le colonne gialle.</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Carta senza potere.</t>
+          <t>Non più usato: anche le carte senza potere sono verdi.</t>
         </is>
       </c>
     </row>
@@ -980,7 +980,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Aggiornato il 28/10/2026 con il gioco alla versione 0.19.0 · 104 carte · righe verdi = carte a posto (potere programmato o tolto) · colonne gialle (M–P) = da compilare. Filtri e menu nella riga delle intestazioni.</t>
+          <t>Aggiornato il 28/10/2026 con il gioco alla versione 0.19.0 · 104 carte · righe verdi = carte a posto (potere programmato, potere tolto o carta senza potere) · colonne gialle (M–P) = da compilare. Filtri e menu nella riga delle intestazioni.</t>
         </is>
       </c>
     </row>
@@ -1067,48 +1067,48 @@
       </c>
     </row>
     <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Custodes-0</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Custodes</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="C5" s="24" t="inlineStr">
         <is>
           <t>Meridianis</t>
         </is>
       </c>
-      <c r="D5" s="14" t="n">
+      <c r="D5" s="19" t="n">
         <v>91</v>
       </c>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F5" s="16" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F5" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H5" s="14" t="inlineStr">
+      <c r="G5" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I5" s="14" t="n"/>
-      <c r="J5" s="14" t="n"/>
-      <c r="K5" s="14" t="n"/>
-      <c r="L5" s="14" t="n"/>
+      <c r="I5" s="19" t="n"/>
+      <c r="J5" s="19" t="n"/>
+      <c r="K5" s="19" t="n"/>
+      <c r="L5" s="19" t="n"/>
       <c r="M5" s="17" t="n"/>
       <c r="N5" s="17" t="n"/>
       <c r="O5" s="17" t="n"/>
@@ -1243,48 +1243,48 @@
       <c r="P7" s="17" t="n"/>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Custodes-3</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="19" t="inlineStr">
         <is>
           <t>Custodes</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C8" s="24" t="inlineStr">
         <is>
           <t>Caelia Vorn</t>
         </is>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="19" t="n">
         <v>69</v>
       </c>
-      <c r="E8" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F8" s="16" t="inlineStr">
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F8" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H8" s="14" t="inlineStr">
+      <c r="G8" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I8" s="14" t="n"/>
-      <c r="J8" s="14" t="n"/>
-      <c r="K8" s="14" t="n"/>
-      <c r="L8" s="14" t="n"/>
+      <c r="I8" s="19" t="n"/>
+      <c r="J8" s="19" t="n"/>
+      <c r="K8" s="19" t="n"/>
+      <c r="L8" s="19" t="n"/>
       <c r="M8" s="17" t="n"/>
       <c r="N8" s="17" t="n"/>
       <c r="O8" s="17" t="n"/>
@@ -1411,48 +1411,48 @@
       <c r="P10" s="17" t="n"/>
     </row>
     <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Custodes-6</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>Custodes</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="C11" s="24" t="inlineStr">
         <is>
           <t>Sentry-7</t>
         </is>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="D11" s="19" t="n">
         <v>51</v>
       </c>
-      <c r="E11" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F11" s="16" t="inlineStr">
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H11" s="14" t="inlineStr">
+      <c r="G11" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I11" s="14" t="n"/>
-      <c r="J11" s="14" t="n"/>
-      <c r="K11" s="14" t="n"/>
-      <c r="L11" s="14" t="n"/>
+      <c r="I11" s="19" t="n"/>
+      <c r="J11" s="19" t="n"/>
+      <c r="K11" s="19" t="n"/>
+      <c r="L11" s="19" t="n"/>
       <c r="M11" s="17" t="n"/>
       <c r="N11" s="17" t="n"/>
       <c r="O11" s="17" t="n"/>
@@ -1531,48 +1531,48 @@
       <c r="P12" s="17" t="n"/>
     </row>
     <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>Custodes-8</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="19" t="inlineStr">
         <is>
           <t>Custodes</t>
         </is>
       </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="C13" s="24" t="inlineStr">
         <is>
           <t>Greyline</t>
         </is>
       </c>
-      <c r="D13" s="14" t="n">
+      <c r="D13" s="19" t="n">
         <v>37</v>
       </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F13" s="16" t="inlineStr">
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G13" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="G13" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I13" s="14" t="n"/>
-      <c r="J13" s="14" t="n"/>
-      <c r="K13" s="14" t="n"/>
-      <c r="L13" s="14" t="n"/>
+      <c r="I13" s="19" t="n"/>
+      <c r="J13" s="19" t="n"/>
+      <c r="K13" s="19" t="n"/>
+      <c r="L13" s="19" t="n"/>
       <c r="M13" s="17" t="n"/>
       <c r="N13" s="17" t="n"/>
       <c r="O13" s="17" t="n"/>
@@ -1835,48 +1835,48 @@
       <c r="P17" s="17" t="n"/>
     </row>
     <row r="18" ht="42" customHeight="1">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>Nullarii-0</t>
         </is>
       </c>
-      <c r="B18" s="14" t="inlineStr">
+      <c r="B18" s="19" t="inlineStr">
         <is>
           <t>Nullarii</t>
         </is>
       </c>
-      <c r="C18" s="15" t="inlineStr">
+      <c r="C18" s="24" t="inlineStr">
         <is>
           <t>The Unmade</t>
         </is>
       </c>
-      <c r="D18" s="14" t="n">
+      <c r="D18" s="19" t="n">
         <v>98</v>
       </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F18" s="16" t="inlineStr">
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F18" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G18" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H18" s="14" t="inlineStr">
+      <c r="G18" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I18" s="14" t="n"/>
-      <c r="J18" s="14" t="n"/>
-      <c r="K18" s="14" t="n"/>
-      <c r="L18" s="14" t="n"/>
+      <c r="I18" s="19" t="n"/>
+      <c r="J18" s="19" t="n"/>
+      <c r="K18" s="19" t="n"/>
+      <c r="L18" s="19" t="n"/>
       <c r="M18" s="17" t="n"/>
       <c r="N18" s="17" t="n"/>
       <c r="O18" s="17" t="n"/>
@@ -2151,48 +2151,48 @@
       <c r="P22" s="17" t="n"/>
     </row>
     <row r="23" ht="42" customHeight="1">
-      <c r="A23" s="14" t="inlineStr">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>Nullarii-5</t>
         </is>
       </c>
-      <c r="B23" s="14" t="inlineStr">
+      <c r="B23" s="19" t="inlineStr">
         <is>
           <t>Nullarii</t>
         </is>
       </c>
-      <c r="C23" s="15" t="inlineStr">
+      <c r="C23" s="24" t="inlineStr">
         <is>
           <t>Ruinborn</t>
         </is>
       </c>
-      <c r="D23" s="14" t="n">
+      <c r="D23" s="19" t="n">
         <v>58</v>
       </c>
-      <c r="E23" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F23" s="16" t="inlineStr">
+      <c r="E23" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F23" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G23" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H23" s="14" t="inlineStr">
+      <c r="G23" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H23" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I23" s="14" t="n"/>
-      <c r="J23" s="14" t="n"/>
-      <c r="K23" s="14" t="n"/>
-      <c r="L23" s="14" t="n"/>
+      <c r="I23" s="19" t="n"/>
+      <c r="J23" s="19" t="n"/>
+      <c r="K23" s="19" t="n"/>
+      <c r="L23" s="19" t="n"/>
       <c r="M23" s="17" t="n"/>
       <c r="N23" s="17" t="n"/>
       <c r="O23" s="17" t="n"/>
@@ -2339,48 +2339,48 @@
       <c r="P25" s="17" t="n"/>
     </row>
     <row r="26" ht="42" customHeight="1">
-      <c r="A26" s="14" t="inlineStr">
+      <c r="A26" s="19" t="inlineStr">
         <is>
           <t>Nullarii-8</t>
         </is>
       </c>
-      <c r="B26" s="14" t="inlineStr">
+      <c r="B26" s="19" t="inlineStr">
         <is>
           <t>Nullarii</t>
         </is>
       </c>
-      <c r="C26" s="15" t="inlineStr">
+      <c r="C26" s="24" t="inlineStr">
         <is>
           <t>Hollow</t>
         </is>
       </c>
-      <c r="D26" s="14" t="n">
+      <c r="D26" s="19" t="n">
         <v>33</v>
       </c>
-      <c r="E26" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F26" s="16" t="inlineStr">
+      <c r="E26" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F26" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G26" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H26" s="14" t="inlineStr">
+      <c r="G26" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H26" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I26" s="14" t="n"/>
-      <c r="J26" s="14" t="n"/>
-      <c r="K26" s="14" t="n"/>
-      <c r="L26" s="14" t="n"/>
+      <c r="I26" s="19" t="n"/>
+      <c r="J26" s="19" t="n"/>
+      <c r="K26" s="19" t="n"/>
+      <c r="L26" s="19" t="n"/>
       <c r="M26" s="17" t="n"/>
       <c r="N26" s="17" t="n"/>
       <c r="O26" s="17" t="n"/>
@@ -2651,48 +2651,48 @@
       <c r="P30" s="17" t="n"/>
     </row>
     <row r="31" ht="45" customHeight="1">
-      <c r="A31" s="14" t="inlineStr">
+      <c r="A31" s="19" t="inlineStr">
         <is>
           <t>Auguria-0</t>
         </is>
       </c>
-      <c r="B31" s="14" t="inlineStr">
+      <c r="B31" s="19" t="inlineStr">
         <is>
           <t>Auguria</t>
         </is>
       </c>
-      <c r="C31" s="15" t="inlineStr">
+      <c r="C31" s="24" t="inlineStr">
         <is>
           <t>Fortuna</t>
         </is>
       </c>
-      <c r="D31" s="14" t="n">
+      <c r="D31" s="19" t="n">
         <v>94</v>
       </c>
-      <c r="E31" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F31" s="16" t="inlineStr">
+      <c r="E31" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F31" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G31" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H31" s="14" t="inlineStr">
+      <c r="G31" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H31" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I31" s="14" t="n"/>
-      <c r="J31" s="14" t="n"/>
-      <c r="K31" s="14" t="n"/>
-      <c r="L31" s="14" t="inlineStr">
+      <c r="I31" s="19" t="n"/>
+      <c r="J31" s="19" t="n"/>
+      <c r="K31" s="19" t="n"/>
+      <c r="L31" s="19" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
         </is>
@@ -2703,48 +2703,48 @@
       <c r="P31" s="17" t="n"/>
     </row>
     <row r="32" ht="45" customHeight="1">
-      <c r="A32" s="14" t="inlineStr">
+      <c r="A32" s="19" t="inlineStr">
         <is>
           <t>Auguria-1</t>
         </is>
       </c>
-      <c r="B32" s="14" t="inlineStr">
+      <c r="B32" s="19" t="inlineStr">
         <is>
           <t>Auguria</t>
         </is>
       </c>
-      <c r="C32" s="15" t="inlineStr">
+      <c r="C32" s="24" t="inlineStr">
         <is>
           <t>Praevis</t>
         </is>
       </c>
-      <c r="D32" s="14" t="n">
+      <c r="D32" s="19" t="n">
         <v>86</v>
       </c>
-      <c r="E32" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F32" s="16" t="inlineStr">
+      <c r="E32" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F32" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G32" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H32" s="14" t="inlineStr">
+      <c r="G32" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H32" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I32" s="14" t="n"/>
-      <c r="J32" s="14" t="n"/>
-      <c r="K32" s="14" t="n"/>
-      <c r="L32" s="14" t="inlineStr">
+      <c r="I32" s="19" t="n"/>
+      <c r="J32" s="19" t="n"/>
+      <c r="K32" s="19" t="n"/>
+      <c r="L32" s="19" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
         </is>
@@ -2875,48 +2875,48 @@
       <c r="P34" s="17" t="n"/>
     </row>
     <row r="35" ht="45" customHeight="1">
-      <c r="A35" s="14" t="inlineStr">
+      <c r="A35" s="19" t="inlineStr">
         <is>
           <t>Auguria-4</t>
         </is>
       </c>
-      <c r="B35" s="14" t="inlineStr">
+      <c r="B35" s="19" t="inlineStr">
         <is>
           <t>Auguria</t>
         </is>
       </c>
-      <c r="C35" s="15" t="inlineStr">
+      <c r="C35" s="24" t="inlineStr">
         <is>
           <t>Kairon</t>
         </is>
       </c>
-      <c r="D35" s="14" t="n">
+      <c r="D35" s="19" t="n">
         <v>62</v>
       </c>
-      <c r="E35" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F35" s="16" t="inlineStr">
+      <c r="E35" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F35" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G35" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H35" s="14" t="inlineStr">
+      <c r="G35" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I35" s="14" t="n"/>
-      <c r="J35" s="14" t="n"/>
-      <c r="K35" s="14" t="n"/>
-      <c r="L35" s="14" t="inlineStr">
+      <c r="I35" s="19" t="n"/>
+      <c r="J35" s="19" t="n"/>
+      <c r="K35" s="19" t="n"/>
+      <c r="L35" s="19" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
         </is>
@@ -2927,48 +2927,48 @@
       <c r="P35" s="17" t="n"/>
     </row>
     <row r="36" ht="45" customHeight="1">
-      <c r="A36" s="14" t="inlineStr">
+      <c r="A36" s="19" t="inlineStr">
         <is>
           <t>Auguria-5</t>
         </is>
       </c>
-      <c r="B36" s="14" t="inlineStr">
+      <c r="B36" s="19" t="inlineStr">
         <is>
           <t>Auguria</t>
         </is>
       </c>
-      <c r="C36" s="15" t="inlineStr">
+      <c r="C36" s="24" t="inlineStr">
         <is>
           <t>Lucent</t>
         </is>
       </c>
-      <c r="D36" s="14" t="n">
+      <c r="D36" s="19" t="n">
         <v>55</v>
       </c>
-      <c r="E36" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F36" s="16" t="inlineStr">
+      <c r="E36" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F36" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G36" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H36" s="14" t="inlineStr">
+      <c r="G36" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H36" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I36" s="14" t="n"/>
-      <c r="J36" s="14" t="n"/>
-      <c r="K36" s="14" t="n"/>
-      <c r="L36" s="14" t="inlineStr">
+      <c r="I36" s="19" t="n"/>
+      <c r="J36" s="19" t="n"/>
+      <c r="K36" s="19" t="n"/>
+      <c r="L36" s="19" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
         </is>
@@ -2979,48 +2979,48 @@
       <c r="P36" s="17" t="n"/>
     </row>
     <row r="37" ht="45" customHeight="1">
-      <c r="A37" s="14" t="inlineStr">
+      <c r="A37" s="19" t="inlineStr">
         <is>
           <t>Auguria-6</t>
         </is>
       </c>
-      <c r="B37" s="14" t="inlineStr">
+      <c r="B37" s="19" t="inlineStr">
         <is>
           <t>Auguria</t>
         </is>
       </c>
-      <c r="C37" s="15" t="inlineStr">
+      <c r="C37" s="24" t="inlineStr">
         <is>
           <t>Morrow</t>
         </is>
       </c>
-      <c r="D37" s="14" t="n">
+      <c r="D37" s="19" t="n">
         <v>47</v>
       </c>
-      <c r="E37" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F37" s="16" t="inlineStr">
+      <c r="E37" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F37" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G37" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H37" s="14" t="inlineStr">
+      <c r="G37" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H37" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I37" s="14" t="n"/>
-      <c r="J37" s="14" t="n"/>
-      <c r="K37" s="14" t="n"/>
-      <c r="L37" s="14" t="inlineStr">
+      <c r="I37" s="19" t="n"/>
+      <c r="J37" s="19" t="n"/>
+      <c r="K37" s="19" t="n"/>
+      <c r="L37" s="19" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
         </is>
@@ -3031,48 +3031,48 @@
       <c r="P37" s="17" t="n"/>
     </row>
     <row r="38" ht="45" customHeight="1">
-      <c r="A38" s="14" t="inlineStr">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>Auguria-7</t>
         </is>
       </c>
-      <c r="B38" s="14" t="inlineStr">
+      <c r="B38" s="19" t="inlineStr">
         <is>
           <t>Auguria</t>
         </is>
       </c>
-      <c r="C38" s="15" t="inlineStr">
+      <c r="C38" s="24" t="inlineStr">
         <is>
           <t>Threadseer</t>
         </is>
       </c>
-      <c r="D38" s="14" t="n">
+      <c r="D38" s="19" t="n">
         <v>39</v>
       </c>
-      <c r="E38" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F38" s="16" t="inlineStr">
+      <c r="E38" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F38" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G38" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H38" s="14" t="inlineStr">
+      <c r="G38" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H38" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I38" s="14" t="n"/>
-      <c r="J38" s="14" t="n"/>
-      <c r="K38" s="14" t="n"/>
-      <c r="L38" s="14" t="inlineStr">
+      <c r="I38" s="19" t="n"/>
+      <c r="J38" s="19" t="n"/>
+      <c r="K38" s="19" t="n"/>
+      <c r="L38" s="19" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
         </is>
@@ -3083,48 +3083,48 @@
       <c r="P38" s="17" t="n"/>
     </row>
     <row r="39" ht="45" customHeight="1">
-      <c r="A39" s="14" t="inlineStr">
+      <c r="A39" s="19" t="inlineStr">
         <is>
           <t>Auguria-8</t>
         </is>
       </c>
-      <c r="B39" s="14" t="inlineStr">
+      <c r="B39" s="19" t="inlineStr">
         <is>
           <t>Auguria</t>
         </is>
       </c>
-      <c r="C39" s="15" t="inlineStr">
+      <c r="C39" s="24" t="inlineStr">
         <is>
           <t>Auspice</t>
         </is>
       </c>
-      <c r="D39" s="14" t="n">
+      <c r="D39" s="19" t="n">
         <v>31</v>
       </c>
-      <c r="E39" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F39" s="16" t="inlineStr">
+      <c r="E39" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F39" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G39" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H39" s="14" t="inlineStr">
+      <c r="G39" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H39" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I39" s="14" t="n"/>
-      <c r="J39" s="14" t="n"/>
-      <c r="K39" s="14" t="n"/>
-      <c r="L39" s="14" t="inlineStr">
+      <c r="I39" s="19" t="n"/>
+      <c r="J39" s="19" t="n"/>
+      <c r="K39" s="19" t="n"/>
+      <c r="L39" s="19" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
         </is>
@@ -3135,48 +3135,48 @@
       <c r="P39" s="17" t="n"/>
     </row>
     <row r="40" ht="45" customHeight="1">
-      <c r="A40" s="14" t="inlineStr">
+      <c r="A40" s="19" t="inlineStr">
         <is>
           <t>Auguria-9</t>
         </is>
       </c>
-      <c r="B40" s="14" t="inlineStr">
+      <c r="B40" s="19" t="inlineStr">
         <is>
           <t>Auguria</t>
         </is>
       </c>
-      <c r="C40" s="15" t="inlineStr">
+      <c r="C40" s="24" t="inlineStr">
         <is>
           <t>Chanceborn</t>
         </is>
       </c>
-      <c r="D40" s="14" t="n">
+      <c r="D40" s="19" t="n">
         <v>23</v>
       </c>
-      <c r="E40" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F40" s="16" t="inlineStr">
+      <c r="E40" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F40" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G40" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H40" s="14" t="inlineStr">
+      <c r="G40" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H40" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I40" s="14" t="n"/>
-      <c r="J40" s="14" t="n"/>
-      <c r="K40" s="14" t="n"/>
-      <c r="L40" s="14" t="inlineStr">
+      <c r="I40" s="19" t="n"/>
+      <c r="J40" s="19" t="n"/>
+      <c r="K40" s="19" t="n"/>
+      <c r="L40" s="19" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
         </is>
@@ -3187,48 +3187,48 @@
       <c r="P40" s="17" t="n"/>
     </row>
     <row r="41" ht="45" customHeight="1">
-      <c r="A41" s="14" t="inlineStr">
+      <c r="A41" s="19" t="inlineStr">
         <is>
           <t>Auguria-10</t>
         </is>
       </c>
-      <c r="B41" s="14" t="inlineStr">
+      <c r="B41" s="19" t="inlineStr">
         <is>
           <t>Auguria</t>
         </is>
       </c>
-      <c r="C41" s="15" t="inlineStr">
+      <c r="C41" s="24" t="inlineStr">
         <is>
           <t>Tertia</t>
         </is>
       </c>
-      <c r="D41" s="14" t="n">
+      <c r="D41" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="E41" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F41" s="16" t="inlineStr">
+      <c r="E41" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F41" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G41" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H41" s="14" t="inlineStr">
+      <c r="G41" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H41" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I41" s="14" t="n"/>
-      <c r="J41" s="14" t="n"/>
-      <c r="K41" s="14" t="n"/>
-      <c r="L41" s="14" t="inlineStr">
+      <c r="I41" s="19" t="n"/>
+      <c r="J41" s="19" t="n"/>
+      <c r="K41" s="19" t="n"/>
+      <c r="L41" s="19" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
         </is>
@@ -3239,48 +3239,48 @@
       <c r="P41" s="17" t="n"/>
     </row>
     <row r="42" ht="45" customHeight="1">
-      <c r="A42" s="14" t="inlineStr">
+      <c r="A42" s="19" t="inlineStr">
         <is>
           <t>Auguria-11</t>
         </is>
       </c>
-      <c r="B42" s="14" t="inlineStr">
+      <c r="B42" s="19" t="inlineStr">
         <is>
           <t>Auguria</t>
         </is>
       </c>
-      <c r="C42" s="15" t="inlineStr">
+      <c r="C42" s="24" t="inlineStr">
         <is>
           <t>Omen</t>
         </is>
       </c>
-      <c r="D42" s="14" t="n">
+      <c r="D42" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="E42" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F42" s="16" t="inlineStr">
+      <c r="E42" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F42" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G42" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H42" s="14" t="inlineStr">
+      <c r="G42" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H42" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I42" s="14" t="n"/>
-      <c r="J42" s="14" t="n"/>
-      <c r="K42" s="14" t="n"/>
-      <c r="L42" s="14" t="inlineStr">
+      <c r="I42" s="19" t="n"/>
+      <c r="J42" s="19" t="n"/>
+      <c r="K42" s="19" t="n"/>
+      <c r="L42" s="19" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
         </is>
@@ -3291,48 +3291,48 @@
       <c r="P42" s="17" t="n"/>
     </row>
     <row r="43" ht="45" customHeight="1">
-      <c r="A43" s="14" t="inlineStr">
+      <c r="A43" s="19" t="inlineStr">
         <is>
           <t>Auguria-12</t>
         </is>
       </c>
-      <c r="B43" s="14" t="inlineStr">
+      <c r="B43" s="19" t="inlineStr">
         <is>
           <t>Auguria</t>
         </is>
       </c>
-      <c r="C43" s="15" t="inlineStr">
+      <c r="C43" s="24" t="inlineStr">
         <is>
           <t>Last Oracle</t>
         </is>
       </c>
-      <c r="D43" s="14" t="n">
+      <c r="D43" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="E43" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F43" s="16" t="inlineStr">
+      <c r="E43" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F43" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G43" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H43" s="14" t="inlineStr">
+      <c r="G43" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H43" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I43" s="14" t="n"/>
-      <c r="J43" s="14" t="n"/>
-      <c r="K43" s="14" t="n"/>
-      <c r="L43" s="14" t="inlineStr">
+      <c r="I43" s="19" t="n"/>
+      <c r="J43" s="19" t="n"/>
+      <c r="K43" s="19" t="n"/>
+      <c r="L43" s="19" t="inlineStr">
         <is>
           <t>Auguria è la fazione dei pronostici: si può dare a questa carta un pronostico come Sibyl o Decima.</t>
         </is>
@@ -3343,48 +3343,48 @@
       <c r="P43" s="17" t="n"/>
     </row>
     <row r="44" ht="42" customHeight="1">
-      <c r="A44" s="14" t="inlineStr">
+      <c r="A44" s="19" t="inlineStr">
         <is>
           <t>Reliquiae-0</t>
         </is>
       </c>
-      <c r="B44" s="14" t="inlineStr">
+      <c r="B44" s="19" t="inlineStr">
         <is>
           <t>Reliquiae</t>
         </is>
       </c>
-      <c r="C44" s="15" t="inlineStr">
+      <c r="C44" s="24" t="inlineStr">
         <is>
           <t>Relicta</t>
         </is>
       </c>
-      <c r="D44" s="14" t="n">
+      <c r="D44" s="19" t="n">
         <v>92</v>
       </c>
-      <c r="E44" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F44" s="16" t="inlineStr">
+      <c r="E44" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F44" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G44" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H44" s="14" t="inlineStr">
+      <c r="G44" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H44" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I44" s="14" t="n"/>
-      <c r="J44" s="14" t="n"/>
-      <c r="K44" s="14" t="n"/>
-      <c r="L44" s="14" t="n"/>
+      <c r="I44" s="19" t="n"/>
+      <c r="J44" s="19" t="n"/>
+      <c r="K44" s="19" t="n"/>
+      <c r="L44" s="19" t="n"/>
       <c r="M44" s="17" t="n"/>
       <c r="N44" s="17" t="n"/>
       <c r="O44" s="17" t="n"/>
@@ -3583,48 +3583,48 @@
       <c r="P47" s="17" t="n"/>
     </row>
     <row r="48" ht="42" customHeight="1">
-      <c r="A48" s="14" t="inlineStr">
+      <c r="A48" s="19" t="inlineStr">
         <is>
           <t>Reliquiae-4</t>
         </is>
       </c>
-      <c r="B48" s="14" t="inlineStr">
+      <c r="B48" s="19" t="inlineStr">
         <is>
           <t>Reliquiae</t>
         </is>
       </c>
-      <c r="C48" s="15" t="inlineStr">
+      <c r="C48" s="24" t="inlineStr">
         <is>
           <t>Violet Wraith</t>
         </is>
       </c>
-      <c r="D48" s="14" t="n">
+      <c r="D48" s="19" t="n">
         <v>61</v>
       </c>
-      <c r="E48" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F48" s="16" t="inlineStr">
+      <c r="E48" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F48" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G48" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H48" s="14" t="inlineStr">
+      <c r="G48" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H48" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I48" s="14" t="n"/>
-      <c r="J48" s="14" t="n"/>
-      <c r="K48" s="14" t="n"/>
-      <c r="L48" s="14" t="n"/>
+      <c r="I48" s="19" t="n"/>
+      <c r="J48" s="19" t="n"/>
+      <c r="K48" s="19" t="n"/>
+      <c r="L48" s="19" t="n"/>
       <c r="M48" s="17" t="n"/>
       <c r="N48" s="17" t="n"/>
       <c r="O48" s="17" t="n"/>
@@ -3759,144 +3759,144 @@
       <c r="P50" s="17" t="n"/>
     </row>
     <row r="51" ht="42" customHeight="1">
-      <c r="A51" s="14" t="inlineStr">
+      <c r="A51" s="19" t="inlineStr">
         <is>
           <t>Reliquiae-7</t>
         </is>
       </c>
-      <c r="B51" s="14" t="inlineStr">
+      <c r="B51" s="19" t="inlineStr">
         <is>
           <t>Reliquiae</t>
         </is>
       </c>
-      <c r="C51" s="15" t="inlineStr">
+      <c r="C51" s="24" t="inlineStr">
         <is>
           <t>Lost Saint</t>
         </is>
       </c>
-      <c r="D51" s="14" t="n">
+      <c r="D51" s="19" t="n">
         <v>38</v>
       </c>
-      <c r="E51" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F51" s="16" t="inlineStr">
+      <c r="E51" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F51" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G51" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H51" s="14" t="inlineStr">
+      <c r="G51" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H51" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I51" s="14" t="n"/>
-      <c r="J51" s="14" t="n"/>
-      <c r="K51" s="14" t="n"/>
-      <c r="L51" s="14" t="n"/>
+      <c r="I51" s="19" t="n"/>
+      <c r="J51" s="19" t="n"/>
+      <c r="K51" s="19" t="n"/>
+      <c r="L51" s="19" t="n"/>
       <c r="M51" s="17" t="n"/>
       <c r="N51" s="17" t="n"/>
       <c r="O51" s="17" t="n"/>
       <c r="P51" s="17" t="n"/>
     </row>
     <row r="52" ht="42" customHeight="1">
-      <c r="A52" s="14" t="inlineStr">
+      <c r="A52" s="19" t="inlineStr">
         <is>
           <t>Reliquiae-8</t>
         </is>
       </c>
-      <c r="B52" s="14" t="inlineStr">
+      <c r="B52" s="19" t="inlineStr">
         <is>
           <t>Reliquiae</t>
         </is>
       </c>
-      <c r="C52" s="15" t="inlineStr">
+      <c r="C52" s="24" t="inlineStr">
         <is>
           <t>Remnant</t>
         </is>
       </c>
-      <c r="D52" s="14" t="n">
+      <c r="D52" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="E52" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F52" s="16" t="inlineStr">
+      <c r="E52" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F52" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G52" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H52" s="14" t="inlineStr">
+      <c r="G52" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H52" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I52" s="14" t="n"/>
-      <c r="J52" s="14" t="n"/>
-      <c r="K52" s="14" t="n"/>
-      <c r="L52" s="14" t="n"/>
+      <c r="I52" s="19" t="n"/>
+      <c r="J52" s="19" t="n"/>
+      <c r="K52" s="19" t="n"/>
+      <c r="L52" s="19" t="n"/>
       <c r="M52" s="17" t="n"/>
       <c r="N52" s="17" t="n"/>
       <c r="O52" s="17" t="n"/>
       <c r="P52" s="17" t="n"/>
     </row>
     <row r="53" ht="42" customHeight="1">
-      <c r="A53" s="14" t="inlineStr">
+      <c r="A53" s="19" t="inlineStr">
         <is>
           <t>Reliquiae-9</t>
         </is>
       </c>
-      <c r="B53" s="14" t="inlineStr">
+      <c r="B53" s="19" t="inlineStr">
         <is>
           <t>Reliquiae</t>
         </is>
       </c>
-      <c r="C53" s="15" t="inlineStr">
+      <c r="C53" s="24" t="inlineStr">
         <is>
           <t>Remainder</t>
         </is>
       </c>
-      <c r="D53" s="14" t="n">
+      <c r="D53" s="19" t="n">
         <v>22</v>
       </c>
-      <c r="E53" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F53" s="16" t="inlineStr">
+      <c r="E53" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F53" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G53" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H53" s="14" t="inlineStr">
+      <c r="G53" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H53" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I53" s="14" t="n"/>
-      <c r="J53" s="14" t="n"/>
-      <c r="K53" s="14" t="n"/>
-      <c r="L53" s="14" t="n"/>
+      <c r="I53" s="19" t="n"/>
+      <c r="J53" s="19" t="n"/>
+      <c r="K53" s="19" t="n"/>
+      <c r="L53" s="19" t="n"/>
       <c r="M53" s="17" t="n"/>
       <c r="N53" s="17" t="n"/>
       <c r="O53" s="17" t="n"/>
@@ -4031,144 +4031,144 @@
       <c r="P55" s="17" t="n"/>
     </row>
     <row r="56" ht="42" customHeight="1">
-      <c r="A56" s="14" t="inlineStr">
+      <c r="A56" s="19" t="inlineStr">
         <is>
           <t>Reliquiae-12</t>
         </is>
       </c>
-      <c r="B56" s="14" t="inlineStr">
+      <c r="B56" s="19" t="inlineStr">
         <is>
           <t>Reliquiae</t>
         </is>
       </c>
-      <c r="C56" s="15" t="inlineStr">
+      <c r="C56" s="24" t="inlineStr">
         <is>
           <t>Vestige</t>
         </is>
       </c>
-      <c r="D56" s="14" t="n">
+      <c r="D56" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="E56" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F56" s="16" t="inlineStr">
+      <c r="E56" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F56" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G56" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H56" s="14" t="inlineStr">
+      <c r="G56" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H56" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I56" s="14" t="n"/>
-      <c r="J56" s="14" t="n"/>
-      <c r="K56" s="14" t="n"/>
-      <c r="L56" s="14" t="n"/>
+      <c r="I56" s="19" t="n"/>
+      <c r="J56" s="19" t="n"/>
+      <c r="K56" s="19" t="n"/>
+      <c r="L56" s="19" t="n"/>
       <c r="M56" s="17" t="n"/>
       <c r="N56" s="17" t="n"/>
       <c r="O56" s="17" t="n"/>
       <c r="P56" s="17" t="n"/>
     </row>
     <row r="57" ht="42" customHeight="1">
-      <c r="A57" s="14" t="inlineStr">
+      <c r="A57" s="19" t="inlineStr">
         <is>
           <t>Dominari-0</t>
         </is>
       </c>
-      <c r="B57" s="14" t="inlineStr">
+      <c r="B57" s="19" t="inlineStr">
         <is>
           <t>Dominari</t>
         </is>
       </c>
-      <c r="C57" s="15" t="inlineStr">
+      <c r="C57" s="24" t="inlineStr">
         <is>
           <t>Imperator</t>
         </is>
       </c>
-      <c r="D57" s="14" t="n">
+      <c r="D57" s="19" t="n">
         <v>99</v>
       </c>
-      <c r="E57" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F57" s="16" t="inlineStr">
+      <c r="E57" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F57" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G57" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H57" s="14" t="inlineStr">
+      <c r="G57" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H57" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I57" s="14" t="n"/>
-      <c r="J57" s="14" t="n"/>
-      <c r="K57" s="14" t="n"/>
-      <c r="L57" s="14" t="n"/>
+      <c r="I57" s="19" t="n"/>
+      <c r="J57" s="19" t="n"/>
+      <c r="K57" s="19" t="n"/>
+      <c r="L57" s="19" t="n"/>
       <c r="M57" s="17" t="n"/>
       <c r="N57" s="17" t="n"/>
       <c r="O57" s="17" t="n"/>
       <c r="P57" s="17" t="n"/>
     </row>
     <row r="58" ht="42" customHeight="1">
-      <c r="A58" s="14" t="inlineStr">
+      <c r="A58" s="19" t="inlineStr">
         <is>
           <t>Dominari-1</t>
         </is>
       </c>
-      <c r="B58" s="14" t="inlineStr">
+      <c r="B58" s="19" t="inlineStr">
         <is>
           <t>Dominari</t>
         </is>
       </c>
-      <c r="C58" s="15" t="inlineStr">
+      <c r="C58" s="24" t="inlineStr">
         <is>
           <t>Vexor</t>
         </is>
       </c>
-      <c r="D58" s="14" t="n">
+      <c r="D58" s="19" t="n">
         <v>90</v>
       </c>
-      <c r="E58" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F58" s="16" t="inlineStr">
+      <c r="E58" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F58" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G58" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H58" s="14" t="inlineStr">
+      <c r="G58" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H58" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I58" s="14" t="n"/>
-      <c r="J58" s="14" t="n"/>
-      <c r="K58" s="14" t="n"/>
-      <c r="L58" s="14" t="n"/>
+      <c r="I58" s="19" t="n"/>
+      <c r="J58" s="19" t="n"/>
+      <c r="K58" s="19" t="n"/>
+      <c r="L58" s="19" t="n"/>
       <c r="M58" s="17" t="n"/>
       <c r="N58" s="17" t="n"/>
       <c r="O58" s="17" t="n"/>
@@ -4303,144 +4303,144 @@
       <c r="P60" s="17" t="n"/>
     </row>
     <row r="61" ht="42" customHeight="1">
-      <c r="A61" s="14" t="inlineStr">
+      <c r="A61" s="19" t="inlineStr">
         <is>
           <t>Dominari-4</t>
         </is>
       </c>
-      <c r="B61" s="14" t="inlineStr">
+      <c r="B61" s="19" t="inlineStr">
         <is>
           <t>Dominari</t>
         </is>
       </c>
-      <c r="C61" s="15" t="inlineStr">
+      <c r="C61" s="24" t="inlineStr">
         <is>
           <t>Crimson Crown</t>
         </is>
       </c>
-      <c r="D61" s="14" t="n">
+      <c r="D61" s="19" t="n">
         <v>66</v>
       </c>
-      <c r="E61" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F61" s="16" t="inlineStr">
+      <c r="E61" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F61" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G61" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H61" s="14" t="inlineStr">
+      <c r="G61" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H61" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I61" s="14" t="n"/>
-      <c r="J61" s="14" t="n"/>
-      <c r="K61" s="14" t="n"/>
-      <c r="L61" s="14" t="n"/>
+      <c r="I61" s="19" t="n"/>
+      <c r="J61" s="19" t="n"/>
+      <c r="K61" s="19" t="n"/>
+      <c r="L61" s="19" t="n"/>
       <c r="M61" s="17" t="n"/>
       <c r="N61" s="17" t="n"/>
       <c r="O61" s="17" t="n"/>
       <c r="P61" s="17" t="n"/>
     </row>
     <row r="62" ht="42" customHeight="1">
-      <c r="A62" s="14" t="inlineStr">
+      <c r="A62" s="19" t="inlineStr">
         <is>
           <t>Dominari-5</t>
         </is>
       </c>
-      <c r="B62" s="14" t="inlineStr">
+      <c r="B62" s="19" t="inlineStr">
         <is>
           <t>Dominari</t>
         </is>
       </c>
-      <c r="C62" s="15" t="inlineStr">
+      <c r="C62" s="24" t="inlineStr">
         <is>
           <t>Duelist</t>
         </is>
       </c>
-      <c r="D62" s="14" t="n">
+      <c r="D62" s="19" t="n">
         <v>59</v>
       </c>
-      <c r="E62" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F62" s="16" t="inlineStr">
+      <c r="E62" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F62" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G62" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H62" s="14" t="inlineStr">
+      <c r="G62" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H62" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I62" s="14" t="n"/>
-      <c r="J62" s="14" t="n"/>
-      <c r="K62" s="14" t="n"/>
-      <c r="L62" s="14" t="n"/>
+      <c r="I62" s="19" t="n"/>
+      <c r="J62" s="19" t="n"/>
+      <c r="K62" s="19" t="n"/>
+      <c r="L62" s="19" t="n"/>
       <c r="M62" s="17" t="n"/>
       <c r="N62" s="17" t="n"/>
       <c r="O62" s="17" t="n"/>
       <c r="P62" s="17" t="n"/>
     </row>
     <row r="63" ht="42" customHeight="1">
-      <c r="A63" s="14" t="inlineStr">
+      <c r="A63" s="19" t="inlineStr">
         <is>
           <t>Dominari-6</t>
         </is>
       </c>
-      <c r="B63" s="14" t="inlineStr">
+      <c r="B63" s="19" t="inlineStr">
         <is>
           <t>Dominari</t>
         </is>
       </c>
-      <c r="C63" s="15" t="inlineStr">
+      <c r="C63" s="24" t="inlineStr">
         <is>
           <t>Warhound</t>
         </is>
       </c>
-      <c r="D63" s="14" t="n">
+      <c r="D63" s="19" t="n">
         <v>51</v>
       </c>
-      <c r="E63" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F63" s="16" t="inlineStr">
+      <c r="E63" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F63" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G63" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H63" s="14" t="inlineStr">
+      <c r="G63" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H63" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I63" s="14" t="n"/>
-      <c r="J63" s="14" t="n"/>
-      <c r="K63" s="14" t="n"/>
-      <c r="L63" s="14" t="n"/>
+      <c r="I63" s="19" t="n"/>
+      <c r="J63" s="19" t="n"/>
+      <c r="K63" s="19" t="n"/>
+      <c r="L63" s="19" t="n"/>
       <c r="M63" s="17" t="n"/>
       <c r="N63" s="17" t="n"/>
       <c r="O63" s="17" t="n"/>
@@ -4827,144 +4827,144 @@
       <c r="P69" s="17" t="n"/>
     </row>
     <row r="70" ht="42" customHeight="1">
-      <c r="A70" s="14" t="inlineStr">
+      <c r="A70" s="19" t="inlineStr">
         <is>
           <t>Concordia-0</t>
         </is>
       </c>
-      <c r="B70" s="14" t="inlineStr">
+      <c r="B70" s="19" t="inlineStr">
         <is>
           <t>Concordia</t>
         </is>
       </c>
-      <c r="C70" s="15" t="inlineStr">
+      <c r="C70" s="24" t="inlineStr">
         <is>
           <t>Equilibrium</t>
         </is>
       </c>
-      <c r="D70" s="14" t="n">
+      <c r="D70" s="19" t="n">
         <v>96</v>
       </c>
-      <c r="E70" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F70" s="16" t="inlineStr">
+      <c r="E70" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F70" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G70" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H70" s="14" t="inlineStr">
+      <c r="G70" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H70" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I70" s="14" t="n"/>
-      <c r="J70" s="14" t="n"/>
-      <c r="K70" s="14" t="n"/>
-      <c r="L70" s="14" t="n"/>
+      <c r="I70" s="19" t="n"/>
+      <c r="J70" s="19" t="n"/>
+      <c r="K70" s="19" t="n"/>
+      <c r="L70" s="19" t="n"/>
       <c r="M70" s="17" t="n"/>
       <c r="N70" s="17" t="n"/>
       <c r="O70" s="17" t="n"/>
       <c r="P70" s="17" t="n"/>
     </row>
     <row r="71" ht="42" customHeight="1">
-      <c r="A71" s="14" t="inlineStr">
+      <c r="A71" s="19" t="inlineStr">
         <is>
           <t>Concordia-1</t>
         </is>
       </c>
-      <c r="B71" s="14" t="inlineStr">
+      <c r="B71" s="19" t="inlineStr">
         <is>
           <t>Concordia</t>
         </is>
       </c>
-      <c r="C71" s="15" t="inlineStr">
+      <c r="C71" s="24" t="inlineStr">
         <is>
           <t>Harmonia</t>
         </is>
       </c>
-      <c r="D71" s="14" t="n">
+      <c r="D71" s="19" t="n">
         <v>87</v>
       </c>
-      <c r="E71" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F71" s="16" t="inlineStr">
+      <c r="E71" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F71" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G71" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H71" s="14" t="inlineStr">
+      <c r="G71" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H71" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I71" s="14" t="n"/>
-      <c r="J71" s="14" t="n"/>
-      <c r="K71" s="14" t="n"/>
-      <c r="L71" s="14" t="n"/>
+      <c r="I71" s="19" t="n"/>
+      <c r="J71" s="19" t="n"/>
+      <c r="K71" s="19" t="n"/>
+      <c r="L71" s="19" t="n"/>
       <c r="M71" s="17" t="n"/>
       <c r="N71" s="17" t="n"/>
       <c r="O71" s="17" t="n"/>
       <c r="P71" s="17" t="n"/>
     </row>
     <row r="72" ht="42" customHeight="1">
-      <c r="A72" s="14" t="inlineStr">
+      <c r="A72" s="19" t="inlineStr">
         <is>
           <t>Concordia-2</t>
         </is>
       </c>
-      <c r="B72" s="14" t="inlineStr">
+      <c r="B72" s="19" t="inlineStr">
         <is>
           <t>Concordia</t>
         </is>
       </c>
-      <c r="C72" s="15" t="inlineStr">
+      <c r="C72" s="24" t="inlineStr">
         <is>
           <t>Mediator</t>
         </is>
       </c>
-      <c r="D72" s="14" t="n">
+      <c r="D72" s="19" t="n">
         <v>79</v>
       </c>
-      <c r="E72" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F72" s="16" t="inlineStr">
+      <c r="E72" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F72" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G72" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H72" s="14" t="inlineStr">
+      <c r="G72" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H72" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I72" s="14" t="n"/>
-      <c r="J72" s="14" t="n"/>
-      <c r="K72" s="14" t="n"/>
-      <c r="L72" s="14" t="n"/>
+      <c r="I72" s="19" t="n"/>
+      <c r="J72" s="19" t="n"/>
+      <c r="K72" s="19" t="n"/>
+      <c r="L72" s="19" t="n"/>
       <c r="M72" s="17" t="n"/>
       <c r="N72" s="17" t="n"/>
       <c r="O72" s="17" t="n"/>
@@ -5035,96 +5035,96 @@
       <c r="P73" s="17" t="n"/>
     </row>
     <row r="74" ht="42" customHeight="1">
-      <c r="A74" s="14" t="inlineStr">
+      <c r="A74" s="19" t="inlineStr">
         <is>
           <t>Concordia-4</t>
         </is>
       </c>
-      <c r="B74" s="14" t="inlineStr">
+      <c r="B74" s="19" t="inlineStr">
         <is>
           <t>Concordia</t>
         </is>
       </c>
-      <c r="C74" s="15" t="inlineStr">
+      <c r="C74" s="24" t="inlineStr">
         <is>
           <t>Concord</t>
         </is>
       </c>
-      <c r="D74" s="14" t="n">
+      <c r="D74" s="19" t="n">
         <v>63</v>
       </c>
-      <c r="E74" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F74" s="16" t="inlineStr">
+      <c r="E74" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F74" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G74" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H74" s="14" t="inlineStr">
+      <c r="G74" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H74" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I74" s="14" t="n"/>
-      <c r="J74" s="14" t="n"/>
-      <c r="K74" s="14" t="n"/>
-      <c r="L74" s="14" t="n"/>
+      <c r="I74" s="19" t="n"/>
+      <c r="J74" s="19" t="n"/>
+      <c r="K74" s="19" t="n"/>
+      <c r="L74" s="19" t="n"/>
       <c r="M74" s="17" t="n"/>
       <c r="N74" s="17" t="n"/>
       <c r="O74" s="17" t="n"/>
       <c r="P74" s="17" t="n"/>
     </row>
     <row r="75" ht="42" customHeight="1">
-      <c r="A75" s="14" t="inlineStr">
+      <c r="A75" s="19" t="inlineStr">
         <is>
           <t>Concordia-5</t>
         </is>
       </c>
-      <c r="B75" s="14" t="inlineStr">
+      <c r="B75" s="19" t="inlineStr">
         <is>
           <t>Concordia</t>
         </is>
       </c>
-      <c r="C75" s="15" t="inlineStr">
+      <c r="C75" s="24" t="inlineStr">
         <is>
           <t>Bridge</t>
         </is>
       </c>
-      <c r="D75" s="14" t="n">
+      <c r="D75" s="19" t="n">
         <v>55</v>
       </c>
-      <c r="E75" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F75" s="16" t="inlineStr">
+      <c r="E75" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F75" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G75" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H75" s="14" t="inlineStr">
+      <c r="G75" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H75" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I75" s="14" t="n"/>
-      <c r="J75" s="14" t="n"/>
-      <c r="K75" s="14" t="n"/>
-      <c r="L75" s="14" t="n"/>
+      <c r="I75" s="19" t="n"/>
+      <c r="J75" s="19" t="n"/>
+      <c r="K75" s="19" t="n"/>
+      <c r="L75" s="19" t="n"/>
       <c r="M75" s="17" t="n"/>
       <c r="N75" s="17" t="n"/>
       <c r="O75" s="17" t="n"/>
@@ -5259,96 +5259,96 @@
       <c r="P77" s="17" t="n"/>
     </row>
     <row r="78" ht="42" customHeight="1">
-      <c r="A78" s="14" t="inlineStr">
+      <c r="A78" s="19" t="inlineStr">
         <is>
           <t>Concordia-8</t>
         </is>
       </c>
-      <c r="B78" s="14" t="inlineStr">
+      <c r="B78" s="19" t="inlineStr">
         <is>
           <t>Concordia</t>
         </is>
       </c>
-      <c r="C78" s="15" t="inlineStr">
+      <c r="C78" s="24" t="inlineStr">
         <is>
           <t>Kin</t>
         </is>
       </c>
-      <c r="D78" s="14" t="n">
+      <c r="D78" s="19" t="n">
         <v>31</v>
       </c>
-      <c r="E78" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F78" s="16" t="inlineStr">
+      <c r="E78" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F78" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G78" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H78" s="14" t="inlineStr">
+      <c r="G78" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H78" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I78" s="14" t="n"/>
-      <c r="J78" s="14" t="n"/>
-      <c r="K78" s="14" t="n"/>
-      <c r="L78" s="14" t="n"/>
+      <c r="I78" s="19" t="n"/>
+      <c r="J78" s="19" t="n"/>
+      <c r="K78" s="19" t="n"/>
+      <c r="L78" s="19" t="n"/>
       <c r="M78" s="17" t="n"/>
       <c r="N78" s="17" t="n"/>
       <c r="O78" s="17" t="n"/>
       <c r="P78" s="17" t="n"/>
     </row>
     <row r="79" ht="42" customHeight="1">
-      <c r="A79" s="14" t="inlineStr">
+      <c r="A79" s="19" t="inlineStr">
         <is>
           <t>Concordia-9</t>
         </is>
       </c>
-      <c r="B79" s="14" t="inlineStr">
+      <c r="B79" s="19" t="inlineStr">
         <is>
           <t>Concordia</t>
         </is>
       </c>
-      <c r="C79" s="15" t="inlineStr">
+      <c r="C79" s="24" t="inlineStr">
         <is>
           <t>Medius</t>
         </is>
       </c>
-      <c r="D79" s="14" t="n">
+      <c r="D79" s="19" t="n">
         <v>23</v>
       </c>
-      <c r="E79" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F79" s="16" t="inlineStr">
+      <c r="E79" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F79" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G79" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H79" s="14" t="inlineStr">
+      <c r="G79" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H79" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I79" s="14" t="n"/>
-      <c r="J79" s="14" t="n"/>
-      <c r="K79" s="14" t="n"/>
-      <c r="L79" s="14" t="n"/>
+      <c r="I79" s="19" t="n"/>
+      <c r="J79" s="19" t="n"/>
+      <c r="K79" s="19" t="n"/>
+      <c r="L79" s="19" t="n"/>
       <c r="M79" s="17" t="n"/>
       <c r="N79" s="17" t="n"/>
       <c r="O79" s="17" t="n"/>
@@ -5479,144 +5479,144 @@
       <c r="P81" s="17" t="n"/>
     </row>
     <row r="82" ht="42" customHeight="1">
-      <c r="A82" s="14" t="inlineStr">
+      <c r="A82" s="19" t="inlineStr">
         <is>
           <t>Concordia-12</t>
         </is>
       </c>
-      <c r="B82" s="14" t="inlineStr">
+      <c r="B82" s="19" t="inlineStr">
         <is>
           <t>Concordia</t>
         </is>
       </c>
-      <c r="C82" s="15" t="inlineStr">
+      <c r="C82" s="24" t="inlineStr">
         <is>
           <t>Union</t>
         </is>
       </c>
-      <c r="D82" s="14" t="n">
+      <c r="D82" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="E82" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F82" s="16" t="inlineStr">
+      <c r="E82" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F82" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G82" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H82" s="14" t="inlineStr">
+      <c r="G82" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H82" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I82" s="14" t="n"/>
-      <c r="J82" s="14" t="n"/>
-      <c r="K82" s="14" t="n"/>
-      <c r="L82" s="14" t="n"/>
+      <c r="I82" s="19" t="n"/>
+      <c r="J82" s="19" t="n"/>
+      <c r="K82" s="19" t="n"/>
+      <c r="L82" s="19" t="n"/>
       <c r="M82" s="17" t="n"/>
       <c r="N82" s="17" t="n"/>
       <c r="O82" s="17" t="n"/>
       <c r="P82" s="17" t="n"/>
     </row>
     <row r="83" ht="42" customHeight="1">
-      <c r="A83" s="14" t="inlineStr">
+      <c r="A83" s="19" t="inlineStr">
         <is>
           <t>Axiomata-0</t>
         </is>
       </c>
-      <c r="B83" s="14" t="inlineStr">
+      <c r="B83" s="19" t="inlineStr">
         <is>
           <t>Axiomata</t>
         </is>
       </c>
-      <c r="C83" s="15" t="inlineStr">
+      <c r="C83" s="24" t="inlineStr">
         <is>
           <t>Lex Prime</t>
         </is>
       </c>
-      <c r="D83" s="14" t="n">
+      <c r="D83" s="19" t="n">
         <v>97</v>
       </c>
-      <c r="E83" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F83" s="16" t="inlineStr">
+      <c r="E83" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F83" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G83" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H83" s="14" t="inlineStr">
+      <c r="G83" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H83" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I83" s="14" t="n"/>
-      <c r="J83" s="14" t="n"/>
-      <c r="K83" s="14" t="n"/>
-      <c r="L83" s="14" t="n"/>
+      <c r="I83" s="19" t="n"/>
+      <c r="J83" s="19" t="n"/>
+      <c r="K83" s="19" t="n"/>
+      <c r="L83" s="19" t="n"/>
       <c r="M83" s="17" t="n"/>
       <c r="N83" s="17" t="n"/>
       <c r="O83" s="17" t="n"/>
       <c r="P83" s="17" t="n"/>
     </row>
     <row r="84" ht="42" customHeight="1">
-      <c r="A84" s="14" t="inlineStr">
+      <c r="A84" s="19" t="inlineStr">
         <is>
           <t>Axiomata-1</t>
         </is>
       </c>
-      <c r="B84" s="14" t="inlineStr">
+      <c r="B84" s="19" t="inlineStr">
         <is>
           <t>Axiomata</t>
         </is>
       </c>
-      <c r="C84" s="15" t="inlineStr">
+      <c r="C84" s="24" t="inlineStr">
         <is>
           <t>Canon</t>
         </is>
       </c>
-      <c r="D84" s="14" t="n">
+      <c r="D84" s="19" t="n">
         <v>88</v>
       </c>
-      <c r="E84" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F84" s="16" t="inlineStr">
+      <c r="E84" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F84" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G84" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H84" s="14" t="inlineStr">
+      <c r="G84" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H84" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I84" s="14" t="n"/>
-      <c r="J84" s="14" t="n"/>
-      <c r="K84" s="14" t="n"/>
-      <c r="L84" s="14" t="n"/>
+      <c r="I84" s="19" t="n"/>
+      <c r="J84" s="19" t="n"/>
+      <c r="K84" s="19" t="n"/>
+      <c r="L84" s="19" t="n"/>
       <c r="M84" s="17" t="n"/>
       <c r="N84" s="17" t="n"/>
       <c r="O84" s="17" t="n"/>
@@ -5687,96 +5687,96 @@
       <c r="P85" s="17" t="n"/>
     </row>
     <row r="86" ht="42" customHeight="1">
-      <c r="A86" s="14" t="inlineStr">
+      <c r="A86" s="19" t="inlineStr">
         <is>
           <t>Axiomata-3</t>
         </is>
       </c>
-      <c r="B86" s="14" t="inlineStr">
+      <c r="B86" s="19" t="inlineStr">
         <is>
           <t>Axiomata</t>
         </is>
       </c>
-      <c r="C86" s="15" t="inlineStr">
+      <c r="C86" s="24" t="inlineStr">
         <is>
           <t>Edict</t>
         </is>
       </c>
-      <c r="D86" s="14" t="n">
+      <c r="D86" s="19" t="n">
         <v>72</v>
       </c>
-      <c r="E86" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F86" s="16" t="inlineStr">
+      <c r="E86" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F86" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G86" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H86" s="14" t="inlineStr">
+      <c r="G86" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H86" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I86" s="14" t="n"/>
-      <c r="J86" s="14" t="n"/>
-      <c r="K86" s="14" t="n"/>
-      <c r="L86" s="14" t="n"/>
+      <c r="I86" s="19" t="n"/>
+      <c r="J86" s="19" t="n"/>
+      <c r="K86" s="19" t="n"/>
+      <c r="L86" s="19" t="n"/>
       <c r="M86" s="17" t="n"/>
       <c r="N86" s="17" t="n"/>
       <c r="O86" s="17" t="n"/>
       <c r="P86" s="17" t="n"/>
     </row>
     <row r="87" ht="42" customHeight="1">
-      <c r="A87" s="14" t="inlineStr">
+      <c r="A87" s="19" t="inlineStr">
         <is>
           <t>Axiomata-4</t>
         </is>
       </c>
-      <c r="B87" s="14" t="inlineStr">
+      <c r="B87" s="19" t="inlineStr">
         <is>
           <t>Axiomata</t>
         </is>
       </c>
-      <c r="C87" s="15" t="inlineStr">
+      <c r="C87" s="24" t="inlineStr">
         <is>
           <t>Constant</t>
         </is>
       </c>
-      <c r="D87" s="14" t="n">
+      <c r="D87" s="19" t="n">
         <v>64</v>
       </c>
-      <c r="E87" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F87" s="16" t="inlineStr">
+      <c r="E87" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F87" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G87" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H87" s="14" t="inlineStr">
+      <c r="G87" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H87" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I87" s="14" t="n"/>
-      <c r="J87" s="14" t="n"/>
-      <c r="K87" s="14" t="n"/>
-      <c r="L87" s="14" t="n"/>
+      <c r="I87" s="19" t="n"/>
+      <c r="J87" s="19" t="n"/>
+      <c r="K87" s="19" t="n"/>
+      <c r="L87" s="19" t="n"/>
       <c r="M87" s="17" t="n"/>
       <c r="N87" s="17" t="n"/>
       <c r="O87" s="17" t="n"/>
@@ -5847,48 +5847,48 @@
       <c r="P88" s="17" t="n"/>
     </row>
     <row r="89" ht="42" customHeight="1">
-      <c r="A89" s="14" t="inlineStr">
+      <c r="A89" s="19" t="inlineStr">
         <is>
           <t>Axiomata-6</t>
         </is>
       </c>
-      <c r="B89" s="14" t="inlineStr">
+      <c r="B89" s="19" t="inlineStr">
         <is>
           <t>Axiomata</t>
         </is>
       </c>
-      <c r="C89" s="15" t="inlineStr">
+      <c r="C89" s="24" t="inlineStr">
         <is>
           <t>Clause</t>
         </is>
       </c>
-      <c r="D89" s="14" t="n">
+      <c r="D89" s="19" t="n">
         <v>47</v>
       </c>
-      <c r="E89" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F89" s="16" t="inlineStr">
+      <c r="E89" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F89" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G89" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H89" s="14" t="inlineStr">
+      <c r="G89" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H89" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I89" s="14" t="n"/>
-      <c r="J89" s="14" t="n"/>
-      <c r="K89" s="14" t="n"/>
-      <c r="L89" s="14" t="n"/>
+      <c r="I89" s="19" t="n"/>
+      <c r="J89" s="19" t="n"/>
+      <c r="K89" s="19" t="n"/>
+      <c r="L89" s="19" t="n"/>
       <c r="M89" s="17" t="n"/>
       <c r="N89" s="17" t="n"/>
       <c r="O89" s="17" t="n"/>
@@ -5959,144 +5959,144 @@
       <c r="P90" s="17" t="n"/>
     </row>
     <row r="91" ht="42" customHeight="1">
-      <c r="A91" s="14" t="inlineStr">
+      <c r="A91" s="19" t="inlineStr">
         <is>
           <t>Axiomata-8</t>
         </is>
       </c>
-      <c r="B91" s="14" t="inlineStr">
+      <c r="B91" s="19" t="inlineStr">
         <is>
           <t>Axiomata</t>
         </is>
       </c>
-      <c r="C91" s="15" t="inlineStr">
+      <c r="C91" s="24" t="inlineStr">
         <is>
           <t>Notary</t>
         </is>
       </c>
-      <c r="D91" s="14" t="n">
+      <c r="D91" s="19" t="n">
         <v>31</v>
       </c>
-      <c r="E91" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F91" s="16" t="inlineStr">
+      <c r="E91" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F91" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G91" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H91" s="14" t="inlineStr">
+      <c r="G91" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H91" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I91" s="14" t="n"/>
-      <c r="J91" s="14" t="n"/>
-      <c r="K91" s="14" t="n"/>
-      <c r="L91" s="14" t="n"/>
+      <c r="I91" s="19" t="n"/>
+      <c r="J91" s="19" t="n"/>
+      <c r="K91" s="19" t="n"/>
+      <c r="L91" s="19" t="n"/>
       <c r="M91" s="17" t="n"/>
       <c r="N91" s="17" t="n"/>
       <c r="O91" s="17" t="n"/>
       <c r="P91" s="17" t="n"/>
     </row>
     <row r="92" ht="42" customHeight="1">
-      <c r="A92" s="14" t="inlineStr">
+      <c r="A92" s="19" t="inlineStr">
         <is>
           <t>Axiomata-9</t>
         </is>
       </c>
-      <c r="B92" s="14" t="inlineStr">
+      <c r="B92" s="19" t="inlineStr">
         <is>
           <t>Axiomata</t>
         </is>
       </c>
-      <c r="C92" s="15" t="inlineStr">
+      <c r="C92" s="24" t="inlineStr">
         <is>
           <t>Seal</t>
         </is>
       </c>
-      <c r="D92" s="14" t="n">
+      <c r="D92" s="19" t="n">
         <v>23</v>
       </c>
-      <c r="E92" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F92" s="16" t="inlineStr">
+      <c r="E92" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F92" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G92" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H92" s="14" t="inlineStr">
+      <c r="G92" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H92" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I92" s="14" t="n"/>
-      <c r="J92" s="14" t="n"/>
-      <c r="K92" s="14" t="n"/>
-      <c r="L92" s="14" t="n"/>
+      <c r="I92" s="19" t="n"/>
+      <c r="J92" s="19" t="n"/>
+      <c r="K92" s="19" t="n"/>
+      <c r="L92" s="19" t="n"/>
       <c r="M92" s="17" t="n"/>
       <c r="N92" s="17" t="n"/>
       <c r="O92" s="17" t="n"/>
       <c r="P92" s="17" t="n"/>
     </row>
     <row r="93" ht="42" customHeight="1">
-      <c r="A93" s="14" t="inlineStr">
+      <c r="A93" s="19" t="inlineStr">
         <is>
           <t>Axiomata-10</t>
         </is>
       </c>
-      <c r="B93" s="14" t="inlineStr">
+      <c r="B93" s="19" t="inlineStr">
         <is>
           <t>Axiomata</t>
         </is>
       </c>
-      <c r="C93" s="15" t="inlineStr">
+      <c r="C93" s="24" t="inlineStr">
         <is>
           <t>Proof</t>
         </is>
       </c>
-      <c r="D93" s="14" t="n">
+      <c r="D93" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="E93" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F93" s="16" t="inlineStr">
+      <c r="E93" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F93" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G93" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H93" s="14" t="inlineStr">
+      <c r="G93" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H93" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I93" s="14" t="n"/>
-      <c r="J93" s="14" t="n"/>
-      <c r="K93" s="14" t="n"/>
-      <c r="L93" s="14" t="n"/>
+      <c r="I93" s="19" t="n"/>
+      <c r="J93" s="19" t="n"/>
+      <c r="K93" s="19" t="n"/>
+      <c r="L93" s="19" t="n"/>
       <c r="M93" s="17" t="n"/>
       <c r="N93" s="17" t="n"/>
       <c r="O93" s="17" t="n"/>
@@ -6167,144 +6167,144 @@
       <c r="P94" s="17" t="n"/>
     </row>
     <row r="95" ht="42" customHeight="1">
-      <c r="A95" s="14" t="inlineStr">
+      <c r="A95" s="19" t="inlineStr">
         <is>
           <t>Axiomata-12</t>
         </is>
       </c>
-      <c r="B95" s="14" t="inlineStr">
+      <c r="B95" s="19" t="inlineStr">
         <is>
           <t>Axiomata</t>
         </is>
       </c>
-      <c r="C95" s="15" t="inlineStr">
+      <c r="C95" s="24" t="inlineStr">
         <is>
           <t>Exception</t>
         </is>
       </c>
-      <c r="D95" s="14" t="n">
+      <c r="D95" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="E95" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F95" s="16" t="inlineStr">
+      <c r="E95" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F95" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G95" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H95" s="14" t="inlineStr">
+      <c r="G95" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H95" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I95" s="14" t="n"/>
-      <c r="J95" s="14" t="n"/>
-      <c r="K95" s="14" t="n"/>
-      <c r="L95" s="14" t="n"/>
+      <c r="I95" s="19" t="n"/>
+      <c r="J95" s="19" t="n"/>
+      <c r="K95" s="19" t="n"/>
+      <c r="L95" s="19" t="n"/>
       <c r="M95" s="17" t="n"/>
       <c r="N95" s="17" t="n"/>
       <c r="O95" s="17" t="n"/>
       <c r="P95" s="17" t="n"/>
     </row>
     <row r="96" ht="42" customHeight="1">
-      <c r="A96" s="14" t="inlineStr">
+      <c r="A96" s="19" t="inlineStr">
         <is>
           <t>Conflux-0</t>
         </is>
       </c>
-      <c r="B96" s="14" t="inlineStr">
+      <c r="B96" s="19" t="inlineStr">
         <is>
           <t>Conflux</t>
         </is>
       </c>
-      <c r="C96" s="15" t="inlineStr">
+      <c r="C96" s="24" t="inlineStr">
         <is>
           <t>Flux Regent</t>
         </is>
       </c>
-      <c r="D96" s="14" t="n">
+      <c r="D96" s="19" t="n">
         <v>97</v>
       </c>
-      <c r="E96" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F96" s="16" t="inlineStr">
+      <c r="E96" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F96" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G96" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H96" s="14" t="inlineStr">
+      <c r="G96" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H96" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I96" s="14" t="n"/>
-      <c r="J96" s="14" t="n"/>
-      <c r="K96" s="14" t="n"/>
-      <c r="L96" s="14" t="n"/>
+      <c r="I96" s="19" t="n"/>
+      <c r="J96" s="19" t="n"/>
+      <c r="K96" s="19" t="n"/>
+      <c r="L96" s="19" t="n"/>
       <c r="M96" s="17" t="n"/>
       <c r="N96" s="17" t="n"/>
       <c r="O96" s="17" t="n"/>
       <c r="P96" s="17" t="n"/>
     </row>
     <row r="97" ht="42" customHeight="1">
-      <c r="A97" s="14" t="inlineStr">
+      <c r="A97" s="19" t="inlineStr">
         <is>
           <t>Conflux-1</t>
         </is>
       </c>
-      <c r="B97" s="14" t="inlineStr">
+      <c r="B97" s="19" t="inlineStr">
         <is>
           <t>Conflux</t>
         </is>
       </c>
-      <c r="C97" s="15" t="inlineStr">
+      <c r="C97" s="24" t="inlineStr">
         <is>
           <t>Mosaic</t>
         </is>
       </c>
-      <c r="D97" s="14" t="n">
+      <c r="D97" s="19" t="n">
         <v>89</v>
       </c>
-      <c r="E97" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F97" s="16" t="inlineStr">
+      <c r="E97" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F97" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G97" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H97" s="14" t="inlineStr">
+      <c r="G97" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H97" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I97" s="14" t="n"/>
-      <c r="J97" s="14" t="n"/>
-      <c r="K97" s="14" t="n"/>
-      <c r="L97" s="14" t="n"/>
+      <c r="I97" s="19" t="n"/>
+      <c r="J97" s="19" t="n"/>
+      <c r="K97" s="19" t="n"/>
+      <c r="L97" s="19" t="n"/>
       <c r="M97" s="17" t="n"/>
       <c r="N97" s="17" t="n"/>
       <c r="O97" s="17" t="n"/>
@@ -6431,96 +6431,96 @@
       <c r="P99" s="17" t="n"/>
     </row>
     <row r="100" ht="42" customHeight="1">
-      <c r="A100" s="14" t="inlineStr">
+      <c r="A100" s="19" t="inlineStr">
         <is>
           <t>Conflux-4</t>
         </is>
       </c>
-      <c r="B100" s="14" t="inlineStr">
+      <c r="B100" s="19" t="inlineStr">
         <is>
           <t>Conflux</t>
         </is>
       </c>
-      <c r="C100" s="15" t="inlineStr">
+      <c r="C100" s="24" t="inlineStr">
         <is>
           <t>Chimera</t>
         </is>
       </c>
-      <c r="D100" s="14" t="n">
+      <c r="D100" s="19" t="n">
         <v>67</v>
       </c>
-      <c r="E100" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F100" s="16" t="inlineStr">
+      <c r="E100" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F100" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G100" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H100" s="14" t="inlineStr">
+      <c r="G100" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H100" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I100" s="14" t="n"/>
-      <c r="J100" s="14" t="n"/>
-      <c r="K100" s="14" t="n"/>
-      <c r="L100" s="14" t="n"/>
+      <c r="I100" s="19" t="n"/>
+      <c r="J100" s="19" t="n"/>
+      <c r="K100" s="19" t="n"/>
+      <c r="L100" s="19" t="n"/>
       <c r="M100" s="17" t="n"/>
       <c r="N100" s="17" t="n"/>
       <c r="O100" s="17" t="n"/>
       <c r="P100" s="17" t="n"/>
     </row>
     <row r="101" ht="42" customHeight="1">
-      <c r="A101" s="14" t="inlineStr">
+      <c r="A101" s="19" t="inlineStr">
         <is>
           <t>Conflux-5</t>
         </is>
       </c>
-      <c r="B101" s="14" t="inlineStr">
+      <c r="B101" s="19" t="inlineStr">
         <is>
           <t>Conflux</t>
         </is>
       </c>
-      <c r="C101" s="15" t="inlineStr">
+      <c r="C101" s="24" t="inlineStr">
         <is>
           <t>Crossfade</t>
         </is>
       </c>
-      <c r="D101" s="14" t="n">
+      <c r="D101" s="19" t="n">
         <v>59</v>
       </c>
-      <c r="E101" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F101" s="16" t="inlineStr">
+      <c r="E101" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F101" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G101" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H101" s="14" t="inlineStr">
+      <c r="G101" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H101" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I101" s="14" t="n"/>
-      <c r="J101" s="14" t="n"/>
-      <c r="K101" s="14" t="n"/>
-      <c r="L101" s="14" t="n"/>
+      <c r="I101" s="19" t="n"/>
+      <c r="J101" s="19" t="n"/>
+      <c r="K101" s="19" t="n"/>
+      <c r="L101" s="19" t="n"/>
       <c r="M101" s="17" t="n"/>
       <c r="N101" s="17" t="n"/>
       <c r="O101" s="17" t="n"/>
@@ -6591,96 +6591,96 @@
       <c r="P102" s="17" t="n"/>
     </row>
     <row r="103" ht="42" customHeight="1">
-      <c r="A103" s="14" t="inlineStr">
+      <c r="A103" s="19" t="inlineStr">
         <is>
           <t>Conflux-7</t>
         </is>
       </c>
-      <c r="B103" s="14" t="inlineStr">
+      <c r="B103" s="19" t="inlineStr">
         <is>
           <t>Conflux</t>
         </is>
       </c>
-      <c r="C103" s="15" t="inlineStr">
+      <c r="C103" s="24" t="inlineStr">
         <is>
           <t>Mirror Twin</t>
         </is>
       </c>
-      <c r="D103" s="14" t="n">
+      <c r="D103" s="19" t="n">
         <v>43</v>
       </c>
-      <c r="E103" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F103" s="16" t="inlineStr">
+      <c r="E103" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F103" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G103" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H103" s="14" t="inlineStr">
+      <c r="G103" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H103" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I103" s="14" t="n"/>
-      <c r="J103" s="14" t="n"/>
-      <c r="K103" s="14" t="n"/>
-      <c r="L103" s="14" t="n"/>
+      <c r="I103" s="19" t="n"/>
+      <c r="J103" s="19" t="n"/>
+      <c r="K103" s="19" t="n"/>
+      <c r="L103" s="19" t="n"/>
       <c r="M103" s="17" t="n"/>
       <c r="N103" s="17" t="n"/>
       <c r="O103" s="17" t="n"/>
       <c r="P103" s="17" t="n"/>
     </row>
     <row r="104" ht="42" customHeight="1">
-      <c r="A104" s="14" t="inlineStr">
+      <c r="A104" s="19" t="inlineStr">
         <is>
           <t>Conflux-8</t>
         </is>
       </c>
-      <c r="B104" s="14" t="inlineStr">
+      <c r="B104" s="19" t="inlineStr">
         <is>
           <t>Conflux</t>
         </is>
       </c>
-      <c r="C104" s="15" t="inlineStr">
+      <c r="C104" s="24" t="inlineStr">
         <is>
           <t>Flicker</t>
         </is>
       </c>
-      <c r="D104" s="14" t="n">
+      <c r="D104" s="19" t="n">
         <v>35</v>
       </c>
-      <c r="E104" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F104" s="16" t="inlineStr">
+      <c r="E104" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F104" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G104" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H104" s="14" t="inlineStr">
+      <c r="G104" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H104" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I104" s="14" t="n"/>
-      <c r="J104" s="14" t="n"/>
-      <c r="K104" s="14" t="n"/>
-      <c r="L104" s="14" t="n"/>
+      <c r="I104" s="19" t="n"/>
+      <c r="J104" s="19" t="n"/>
+      <c r="K104" s="19" t="n"/>
+      <c r="L104" s="19" t="n"/>
       <c r="M104" s="17" t="n"/>
       <c r="N104" s="17" t="n"/>
       <c r="O104" s="17" t="n"/>
@@ -6871,48 +6871,48 @@
       <c r="P107" s="17" t="n"/>
     </row>
     <row r="108" ht="42" customHeight="1">
-      <c r="A108" s="14" t="inlineStr">
+      <c r="A108" s="19" t="inlineStr">
         <is>
           <t>Conflux-12</t>
         </is>
       </c>
-      <c r="B108" s="14" t="inlineStr">
+      <c r="B108" s="19" t="inlineStr">
         <is>
           <t>Conflux</t>
         </is>
       </c>
-      <c r="C108" s="15" t="inlineStr">
+      <c r="C108" s="24" t="inlineStr">
         <is>
           <t>Convergence</t>
         </is>
       </c>
-      <c r="D108" s="14" t="n">
+      <c r="D108" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="E108" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F108" s="16" t="inlineStr">
+      <c r="E108" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F108" s="25" t="inlineStr">
         <is>
           <t>Senza potere</t>
         </is>
       </c>
-      <c r="G108" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H108" s="14" t="inlineStr">
+      <c r="G108" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H108" s="19" t="inlineStr">
         <is>
           <t>Nessun potere.</t>
         </is>
       </c>
-      <c r="I108" s="14" t="n"/>
-      <c r="J108" s="14" t="n"/>
-      <c r="K108" s="14" t="n"/>
-      <c r="L108" s="14" t="n"/>
+      <c r="I108" s="19" t="n"/>
+      <c r="J108" s="19" t="n"/>
+      <c r="K108" s="19" t="n"/>
+      <c r="L108" s="19" t="n"/>
       <c r="M108" s="17" t="n"/>
       <c r="N108" s="17" t="n"/>
       <c r="O108" s="17" t="n"/>
@@ -7266,7 +7266,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="20" t="inlineStr">
         <is>
@@ -7327,7 +7326,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="16.8" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
@@ -7395,7 +7393,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="16.8" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>

</xml_diff>